<commit_message>
integration of OFF extraction, full integration of dataclasses, major bugfixes
</commit_message>
<xml_diff>
--- a/EconAutomation/src/supporting_docs/sorted_econ_files/PV2 (color coded).xlsx
+++ b/EconAutomation/src/supporting_docs/sorted_econ_files/PV2 (color coded).xlsx
@@ -9,9 +9,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EricBussey\GitHub\EconAutomation-REP\EconAutomation\src\supporting_docs\sorted_econ_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37289FC9-9471-468D-A655-9FEE320B99A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA190262-7409-40D4-A646-59372B6C3F4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="3195" windowWidth="29040" windowHeight="15720" tabRatio="795" xr2:uid="{25EC3B8A-402B-47FF-80A9-5B0690A475CD}"/>
+    <workbookView xWindow="28680" yWindow="-60" windowWidth="29040" windowHeight="15720" tabRatio="795" xr2:uid="{25EC3B8A-402B-47FF-80A9-5B0690A475CD}"/>
   </bookViews>
   <sheets>
     <sheet name="REPORT_OUTPUTS" sheetId="33" r:id="rId1"/>
@@ -1138,31 +1138,16 @@
     <t>G71</t>
   </si>
   <si>
-    <t>Base 1 PV Loss to Age</t>
-  </si>
-  <si>
     <t>Base 2 PV Loss WLE</t>
-  </si>
-  <si>
-    <t>Base 2 PV Loss to Age</t>
   </si>
   <si>
     <t>Base 3 PV Loss WLE</t>
   </si>
   <si>
-    <t>Base 3 PV Loss to Age</t>
-  </si>
-  <si>
     <t>Base 4 PV Loss WLE</t>
   </si>
   <si>
-    <t>Base 4 PV Loss to Age</t>
-  </si>
-  <si>
     <t>Base 5 PV Loss WLE</t>
-  </si>
-  <si>
-    <t>Base 5 PV Loss to Age</t>
   </si>
   <si>
     <t>E73</t>
@@ -1429,13 +1414,28 @@
     <t>est_rate_of_infl</t>
   </si>
   <si>
-    <t>real_rate</t>
+    <t>&lt;-- pulling from Voc report</t>
   </si>
   <si>
-    <t>PV2_discount_rate</t>
+    <t>Base 1 PV Loss To Age</t>
   </si>
   <si>
-    <t>&lt;-- pulling from Voc report</t>
+    <t>Base 2 PV Loss To Age</t>
+  </si>
+  <si>
+    <t>Base 3 PV Loss To Age</t>
+  </si>
+  <si>
+    <t>Base 4 PV Loss To Age</t>
+  </si>
+  <si>
+    <t>Base 5 PV Loss To Age</t>
+  </si>
+  <si>
+    <t>PV2_disc_rate_default</t>
+  </si>
+  <si>
+    <t>PV2_disc_rate_real</t>
   </si>
 </sst>
 </file>
@@ -2290,6 +2290,9 @@
     <xf numFmtId="0" fontId="29" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="29" fillId="13" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="26" fillId="23" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2322,9 +2325,6 @@
     <xf numFmtId="0" fontId="17" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="29" fillId="13" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Currency" xfId="5" builtinId="4"/>
@@ -3817,12 +3817,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.2">
-      <c r="A1" s="107" t="s">
+      <c r="A1" s="108" t="s">
         <v>260</v>
       </c>
-      <c r="B1" s="108"/>
-      <c r="C1" s="108"/>
-      <c r="D1" s="109"/>
+      <c r="B1" s="109"/>
+      <c r="C1" s="109"/>
+      <c r="D1" s="110"/>
     </row>
     <row r="2" spans="1:8" ht="15.75" x14ac:dyDescent="0.2">
       <c r="A2" s="77" t="s">
@@ -3913,7 +3913,7 @@
         <v>281</v>
       </c>
       <c r="H6" t="s">
-        <v>440</v>
+        <v>433</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15" x14ac:dyDescent="0.2">
@@ -3933,7 +3933,7 @@
     </row>
     <row r="8" spans="1:8" ht="15" x14ac:dyDescent="0.2">
       <c r="A8" s="83" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="B8" s="84" t="s">
         <v>318</v>
@@ -3948,7 +3948,7 @@
     </row>
     <row r="9" spans="1:8" ht="15" x14ac:dyDescent="0.2">
       <c r="A9" s="97" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="B9" s="98" t="s">
         <v>318</v>
@@ -3963,7 +3963,7 @@
     </row>
     <row r="10" spans="1:8" ht="15" x14ac:dyDescent="0.2">
       <c r="A10" s="83" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="B10" s="84" t="s">
         <v>318</v>
@@ -4039,13 +4039,13 @@
     </row>
     <row r="15" spans="1:8" ht="15" x14ac:dyDescent="0.2">
       <c r="A15" s="97" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="B15" s="98" t="s">
         <v>332</v>
       </c>
       <c r="C15" s="98" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="D15" s="101" cm="1">
         <f t="array" aca="1" ref="D15" ca="1">IF(OR(IF(OR(A15="", B15="", C15=""), "", INDIRECT("'" &amp; B15 &amp; "'!" &amp; C15))=0, IF(OR(A15="", B15="", C15=""), "", INDIRECT("'" &amp; B15 &amp; "'!" &amp; C15))=""),"",INDIRECT("'" &amp; B15 &amp; "'!" &amp; C15))</f>
@@ -4055,13 +4055,13 @@
     </row>
     <row r="16" spans="1:8" ht="15" x14ac:dyDescent="0.2">
       <c r="A16" s="83" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
       <c r="B16" s="84" t="s">
         <v>332</v>
       </c>
       <c r="C16" s="84" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="D16" s="105" cm="1">
         <f t="array" aca="1" ref="D16" ca="1">IF(OR(IF(OR(A16="", B16="", C16=""), "", INDIRECT("'" &amp; B16 &amp; "'!" &amp; C16))=0, IF(OR(A16="", B16="", C16=""), "", INDIRECT("'" &amp; B16 &amp; "'!" &amp; C16))=""),"",INDIRECT("'" &amp; B16 &amp; "'!" &amp; C16))</f>
@@ -4087,7 +4087,7 @@
     </row>
     <row r="18" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A18" s="83" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
       <c r="B18" s="84" t="s">
         <v>332</v>
@@ -4118,7 +4118,7 @@
     </row>
     <row r="20" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A20" s="83" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
       <c r="B20" s="84" t="s">
         <v>332</v>
@@ -4133,13 +4133,13 @@
     </row>
     <row r="21" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A21" s="97" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="B21" s="98" t="s">
-        <v>341</v>
+        <v>434</v>
       </c>
       <c r="C21" s="98" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="D21" s="101" cm="1">
         <f t="array" aca="1" ref="D21" ca="1">IF(OR(IF(OR(A21="", B21="", C21=""), "", INDIRECT("'" &amp; B21 &amp; "'!" &amp; C21))=0, IF(OR(A21="", B21="", C21=""), "", INDIRECT("'" &amp; B21 &amp; "'!" &amp; C21))=""),"",INDIRECT("'" &amp; B21 &amp; "'!" &amp; C21))</f>
@@ -4148,13 +4148,13 @@
     </row>
     <row r="22" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A22" s="83" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
       <c r="B22" s="84" t="s">
-        <v>341</v>
+        <v>434</v>
       </c>
       <c r="C22" s="84" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="D22" s="105" cm="1">
         <f t="array" aca="1" ref="D22" ca="1">IF(OR(IF(OR(A22="", B22="", C22=""), "", INDIRECT("'" &amp; B22 &amp; "'!" &amp; C22))=0, IF(OR(A22="", B22="", C22=""), "", INDIRECT("'" &amp; B22 &amp; "'!" &amp; C22))=""),"",INDIRECT("'" &amp; B22 &amp; "'!" &amp; C22))</f>
@@ -4166,7 +4166,7 @@
         <v>290</v>
       </c>
       <c r="B23" s="87" t="s">
-        <v>341</v>
+        <v>434</v>
       </c>
       <c r="C23" s="87" t="s">
         <v>338</v>
@@ -4178,10 +4178,10 @@
     </row>
     <row r="24" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A24" s="83" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
       <c r="B24" s="84" t="s">
-        <v>341</v>
+        <v>434</v>
       </c>
       <c r="C24" s="84" t="s">
         <v>333</v>
@@ -4196,7 +4196,7 @@
         <v>291</v>
       </c>
       <c r="B25" s="87" t="s">
-        <v>341</v>
+        <v>434</v>
       </c>
       <c r="C25" s="87" t="s">
         <v>339</v>
@@ -4208,10 +4208,10 @@
     </row>
     <row r="26" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A26" s="83" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="B26" s="84" t="s">
-        <v>341</v>
+        <v>434</v>
       </c>
       <c r="C26" s="84" t="s">
         <v>340</v>
@@ -4229,7 +4229,7 @@
         <v>332</v>
       </c>
       <c r="C27" s="87" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="D27" s="101" cm="1">
         <f t="array" aca="1" ref="D27" ca="1">IF(OR(IF(OR(A27="", B27="", C27=""), "", INDIRECT("'" &amp; B27 &amp; "'!" &amp; C27))=0, IF(OR(A27="", B27="", C27=""), "", INDIRECT("'" &amp; B27 &amp; "'!" &amp; C27))=""),"",INDIRECT("'" &amp; B27 &amp; "'!" &amp; C27))</f>
@@ -4238,13 +4238,13 @@
     </row>
     <row r="28" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A28" s="83" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
       <c r="B28" s="84" t="s">
         <v>332</v>
       </c>
       <c r="C28" s="84" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="D28" s="102" cm="1">
         <f t="array" aca="1" ref="D28" ca="1">IF(OR(IF(OR(A28="", B28="", C28=""), "", INDIRECT("'" &amp; B28 &amp; "'!" &amp; C28))=0, IF(OR(A28="", B28="", C28=""), "", INDIRECT("'" &amp; B28 &amp; "'!" &amp; C28))=""),"",INDIRECT("'" &amp; B28 &amp; "'!" &amp; C28))</f>
@@ -4256,10 +4256,10 @@
         <v>293</v>
       </c>
       <c r="B29" s="87" t="s">
-        <v>341</v>
+        <v>434</v>
       </c>
       <c r="C29" s="87" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="D29" s="101" cm="1">
         <f t="array" aca="1" ref="D29" ca="1">IF(OR(IF(OR(A29="", B29="", C29=""), "", INDIRECT("'" &amp; B29 &amp; "'!" &amp; C29))=0, IF(OR(A29="", B29="", C29=""), "", INDIRECT("'" &amp; B29 &amp; "'!" &amp; C29))=""),"",INDIRECT("'" &amp; B29 &amp; "'!" &amp; C29))</f>
@@ -4268,13 +4268,13 @@
     </row>
     <row r="30" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A30" s="83" t="s">
-        <v>383</v>
+        <v>378</v>
       </c>
       <c r="B30" s="84" t="s">
-        <v>341</v>
+        <v>434</v>
       </c>
       <c r="C30" s="84" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="D30" s="102" cm="1">
         <f t="array" aca="1" ref="D30" ca="1">IF(OR(IF(OR(A30="", B30="", C30=""), "", INDIRECT("'" &amp; B30 &amp; "'!" &amp; C30))=0, IF(OR(A30="", B30="", C30=""), "", INDIRECT("'" &amp; B30 &amp; "'!" &amp; C30))=""),"",INDIRECT("'" &amp; B30 &amp; "'!" &amp; C30))</f>
@@ -4283,13 +4283,13 @@
     </row>
     <row r="31" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A31" s="97" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
       <c r="B31" s="98" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C31" s="98" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="D31" s="101" cm="1">
         <f t="array" aca="1" ref="D31" ca="1">IF(OR(IF(OR(A31="", B31="", C31=""), "", INDIRECT("'" &amp; B31 &amp; "'!" &amp; C31))=0, IF(OR(A31="", B31="", C31=""), "", INDIRECT("'" &amp; B31 &amp; "'!" &amp; C31))=""),"",INDIRECT("'" &amp; B31 &amp; "'!" &amp; C31))</f>
@@ -4298,13 +4298,13 @@
     </row>
     <row r="32" spans="1:5" ht="15" x14ac:dyDescent="0.2">
       <c r="A32" s="83" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="B32" s="84" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C32" s="84" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="D32" s="105" cm="1">
         <f t="array" aca="1" ref="D32" ca="1">IF(OR(IF(OR(A32="", B32="", C32=""), "", INDIRECT("'" &amp; B32 &amp; "'!" &amp; C32))=0, IF(OR(A32="", B32="", C32=""), "", INDIRECT("'" &amp; B32 &amp; "'!" &amp; C32))=""),"",INDIRECT("'" &amp; B32 &amp; "'!" &amp; C32))</f>
@@ -4316,7 +4316,7 @@
         <v>299</v>
       </c>
       <c r="B33" s="87" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C33" s="87" t="s">
         <v>338</v>
@@ -4328,10 +4328,10 @@
     </row>
     <row r="34" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A34" s="83" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
       <c r="B34" s="84" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C34" s="84" t="s">
         <v>333</v>
@@ -4346,7 +4346,7 @@
         <v>294</v>
       </c>
       <c r="B35" s="87" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C35" s="87" t="s">
         <v>339</v>
@@ -4358,10 +4358,10 @@
     </row>
     <row r="36" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A36" s="83" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="B36" s="84" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C36" s="84" t="s">
         <v>340</v>
@@ -4373,13 +4373,13 @@
     </row>
     <row r="37" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A37" s="97" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
       <c r="B37" s="98" t="s">
-        <v>343</v>
+        <v>435</v>
       </c>
       <c r="C37" s="98" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="D37" s="101" cm="1">
         <f t="array" aca="1" ref="D37" ca="1">IF(OR(IF(OR(A37="", B37="", C37=""), "", INDIRECT("'" &amp; B37 &amp; "'!" &amp; C37))=0, IF(OR(A37="", B37="", C37=""), "", INDIRECT("'" &amp; B37 &amp; "'!" &amp; C37))=""),"",INDIRECT("'" &amp; B37 &amp; "'!" &amp; C37))</f>
@@ -4388,13 +4388,13 @@
     </row>
     <row r="38" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A38" s="83" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
       <c r="B38" s="84" t="s">
-        <v>343</v>
+        <v>435</v>
       </c>
       <c r="C38" s="84" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="D38" s="105" cm="1">
         <f t="array" aca="1" ref="D38" ca="1">IF(OR(IF(OR(A38="", B38="", C38=""), "", INDIRECT("'" &amp; B38 &amp; "'!" &amp; C38))=0, IF(OR(A38="", B38="", C38=""), "", INDIRECT("'" &amp; B38 &amp; "'!" &amp; C38))=""),"",INDIRECT("'" &amp; B38 &amp; "'!" &amp; C38))</f>
@@ -4406,7 +4406,7 @@
         <v>295</v>
       </c>
       <c r="B39" s="87" t="s">
-        <v>343</v>
+        <v>435</v>
       </c>
       <c r="C39" s="87" t="s">
         <v>338</v>
@@ -4418,10 +4418,10 @@
     </row>
     <row r="40" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A40" s="83" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="B40" s="84" t="s">
-        <v>343</v>
+        <v>435</v>
       </c>
       <c r="C40" s="84" t="s">
         <v>333</v>
@@ -4436,7 +4436,7 @@
         <v>296</v>
       </c>
       <c r="B41" s="87" t="s">
-        <v>343</v>
+        <v>435</v>
       </c>
       <c r="C41" s="87" t="s">
         <v>339</v>
@@ -4448,10 +4448,10 @@
     </row>
     <row r="42" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A42" s="83" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="B42" s="84" t="s">
-        <v>343</v>
+        <v>435</v>
       </c>
       <c r="C42" s="84" t="s">
         <v>340</v>
@@ -4466,10 +4466,10 @@
         <v>297</v>
       </c>
       <c r="B43" s="87" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C43" s="87" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="D43" s="101" cm="1">
         <f t="array" aca="1" ref="D43" ca="1">IF(OR(IF(OR(A43="", B43="", C43=""), "", INDIRECT("'" &amp; B43 &amp; "'!" &amp; C43))=0, IF(OR(A43="", B43="", C43=""), "", INDIRECT("'" &amp; B43 &amp; "'!" &amp; C43))=""),"",INDIRECT("'" &amp; B43 &amp; "'!" &amp; C43))</f>
@@ -4478,13 +4478,13 @@
     </row>
     <row r="44" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A44" s="83" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
       <c r="B44" s="84" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C44" s="84" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="D44" s="102" cm="1">
         <f t="array" aca="1" ref="D44" ca="1">IF(OR(IF(OR(A44="", B44="", C44=""), "", INDIRECT("'" &amp; B44 &amp; "'!" &amp; C44))=0, IF(OR(A44="", B44="", C44=""), "", INDIRECT("'" &amp; B44 &amp; "'!" &amp; C44))=""),"",INDIRECT("'" &amp; B44 &amp; "'!" &amp; C44))</f>
@@ -4496,10 +4496,10 @@
         <v>298</v>
       </c>
       <c r="B45" s="87" t="s">
-        <v>343</v>
+        <v>435</v>
       </c>
       <c r="C45" s="87" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="D45" s="101" cm="1">
         <f t="array" aca="1" ref="D45" ca="1">IF(OR(IF(OR(A45="", B45="", C45=""), "", INDIRECT("'" &amp; B45 &amp; "'!" &amp; C45))=0, IF(OR(A45="", B45="", C45=""), "", INDIRECT("'" &amp; B45 &amp; "'!" &amp; C45))=""),"",INDIRECT("'" &amp; B45 &amp; "'!" &amp; C45))</f>
@@ -4508,13 +4508,13 @@
     </row>
     <row r="46" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A46" s="83" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
       <c r="B46" s="84" t="s">
-        <v>343</v>
+        <v>435</v>
       </c>
       <c r="C46" s="84" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="D46" s="102" cm="1">
         <f t="array" aca="1" ref="D46" ca="1">IF(OR(IF(OR(A46="", B46="", C46=""), "", INDIRECT("'" &amp; B46 &amp; "'!" &amp; C46))=0, IF(OR(A46="", B46="", C46=""), "", INDIRECT("'" &amp; B46 &amp; "'!" &amp; C46))=""),"",INDIRECT("'" &amp; B46 &amp; "'!" &amp; C46))</f>
@@ -4523,13 +4523,13 @@
     </row>
     <row r="47" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A47" s="97" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="B47" s="98" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="C47" s="98" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="D47" s="101" cm="1">
         <f t="array" aca="1" ref="D47" ca="1">IF(OR(IF(OR(A47="", B47="", C47=""), "", INDIRECT("'" &amp; B47 &amp; "'!" &amp; C47))=0, IF(OR(A47="", B47="", C47=""), "", INDIRECT("'" &amp; B47 &amp; "'!" &amp; C47))=""),"",INDIRECT("'" &amp; B47 &amp; "'!" &amp; C47))</f>
@@ -4538,13 +4538,13 @@
     </row>
     <row r="48" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A48" s="83" t="s">
-        <v>375</v>
+        <v>370</v>
       </c>
       <c r="B48" s="84" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="C48" s="84" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="D48" s="105" cm="1">
         <f t="array" aca="1" ref="D48" ca="1">IF(OR(IF(OR(A48="", B48="", C48=""), "", INDIRECT("'" &amp; B48 &amp; "'!" &amp; C48))=0, IF(OR(A48="", B48="", C48=""), "", INDIRECT("'" &amp; B48 &amp; "'!" &amp; C48))=""),"",INDIRECT("'" &amp; B48 &amp; "'!" &amp; C48))</f>
@@ -4556,7 +4556,7 @@
         <v>300</v>
       </c>
       <c r="B49" s="87" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="C49" s="87" t="s">
         <v>338</v>
@@ -4568,10 +4568,10 @@
     </row>
     <row r="50" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A50" s="83" t="s">
-        <v>390</v>
+        <v>385</v>
       </c>
       <c r="B50" s="84" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="C50" s="84" t="s">
         <v>333</v>
@@ -4586,7 +4586,7 @@
         <v>301</v>
       </c>
       <c r="B51" s="87" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="C51" s="87" t="s">
         <v>339</v>
@@ -4598,10 +4598,10 @@
     </row>
     <row r="52" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A52" s="83" t="s">
-        <v>391</v>
+        <v>386</v>
       </c>
       <c r="B52" s="84" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="C52" s="84" t="s">
         <v>340</v>
@@ -4613,13 +4613,13 @@
     </row>
     <row r="53" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A53" s="97" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="B53" s="98" t="s">
-        <v>345</v>
+        <v>436</v>
       </c>
       <c r="C53" s="98" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="D53" s="101" cm="1">
         <f t="array" aca="1" ref="D53" ca="1">IF(OR(IF(OR(A53="", B53="", C53=""), "", INDIRECT("'" &amp; B53 &amp; "'!" &amp; C53))=0, IF(OR(A53="", B53="", C53=""), "", INDIRECT("'" &amp; B53 &amp; "'!" &amp; C53))=""),"",INDIRECT("'" &amp; B53 &amp; "'!" &amp; C53))</f>
@@ -4628,13 +4628,13 @@
     </row>
     <row r="54" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A54" s="83" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="B54" s="84" t="s">
-        <v>345</v>
+        <v>436</v>
       </c>
       <c r="C54" s="84" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="D54" s="105" cm="1">
         <f t="array" aca="1" ref="D54" ca="1">IF(OR(IF(OR(A54="", B54="", C54=""), "", INDIRECT("'" &amp; B54 &amp; "'!" &amp; C54))=0, IF(OR(A54="", B54="", C54=""), "", INDIRECT("'" &amp; B54 &amp; "'!" &amp; C54))=""),"",INDIRECT("'" &amp; B54 &amp; "'!" &amp; C54))</f>
@@ -4646,7 +4646,7 @@
         <v>302</v>
       </c>
       <c r="B55" s="87" t="s">
-        <v>345</v>
+        <v>436</v>
       </c>
       <c r="C55" s="87" t="s">
         <v>338</v>
@@ -4658,10 +4658,10 @@
     </row>
     <row r="56" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A56" s="83" t="s">
-        <v>392</v>
+        <v>387</v>
       </c>
       <c r="B56" s="84" t="s">
-        <v>345</v>
+        <v>436</v>
       </c>
       <c r="C56" s="84" t="s">
         <v>333</v>
@@ -4676,7 +4676,7 @@
         <v>303</v>
       </c>
       <c r="B57" s="87" t="s">
-        <v>345</v>
+        <v>436</v>
       </c>
       <c r="C57" s="87" t="s">
         <v>339</v>
@@ -4688,10 +4688,10 @@
     </row>
     <row r="58" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A58" s="83" t="s">
-        <v>393</v>
+        <v>388</v>
       </c>
       <c r="B58" s="84" t="s">
-        <v>345</v>
+        <v>436</v>
       </c>
       <c r="C58" s="84" t="s">
         <v>340</v>
@@ -4706,10 +4706,10 @@
         <v>304</v>
       </c>
       <c r="B59" s="87" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="C59" s="87" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="D59" s="101" cm="1">
         <f t="array" aca="1" ref="D59" ca="1">IF(OR(IF(OR(A59="", B59="", C59=""), "", INDIRECT("'" &amp; B59 &amp; "'!" &amp; C59))=0, IF(OR(A59="", B59="", C59=""), "", INDIRECT("'" &amp; B59 &amp; "'!" &amp; C59))=""),"",INDIRECT("'" &amp; B59 &amp; "'!" &amp; C59))</f>
@@ -4718,13 +4718,13 @@
     </row>
     <row r="60" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A60" s="83" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
       <c r="B60" s="84" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="C60" s="84" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="D60" s="102" cm="1">
         <f t="array" aca="1" ref="D60" ca="1">IF(OR(IF(OR(A60="", B60="", C60=""), "", INDIRECT("'" &amp; B60 &amp; "'!" &amp; C60))=0, IF(OR(A60="", B60="", C60=""), "", INDIRECT("'" &amp; B60 &amp; "'!" &amp; C60))=""),"",INDIRECT("'" &amp; B60 &amp; "'!" &amp; C60))</f>
@@ -4736,10 +4736,10 @@
         <v>305</v>
       </c>
       <c r="B61" s="87" t="s">
+        <v>436</v>
+      </c>
+      <c r="C61" s="87" t="s">
         <v>345</v>
-      </c>
-      <c r="C61" s="87" t="s">
-        <v>350</v>
       </c>
       <c r="D61" s="101" cm="1">
         <f t="array" aca="1" ref="D61" ca="1">IF(OR(IF(OR(A61="", B61="", C61=""), "", INDIRECT("'" &amp; B61 &amp; "'!" &amp; C61))=0, IF(OR(A61="", B61="", C61=""), "", INDIRECT("'" &amp; B61 &amp; "'!" &amp; C61))=""),"",INDIRECT("'" &amp; B61 &amp; "'!" &amp; C61))</f>
@@ -4748,13 +4748,13 @@
     </row>
     <row r="62" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A62" s="83" t="s">
-        <v>395</v>
+        <v>390</v>
       </c>
       <c r="B62" s="84" t="s">
-        <v>345</v>
+        <v>436</v>
       </c>
       <c r="C62" s="84" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="D62" s="102" cm="1">
         <f t="array" aca="1" ref="D62" ca="1">IF(OR(IF(OR(A62="", B62="", C62=""), "", INDIRECT("'" &amp; B62 &amp; "'!" &amp; C62))=0, IF(OR(A62="", B62="", C62=""), "", INDIRECT("'" &amp; B62 &amp; "'!" &amp; C62))=""),"",INDIRECT("'" &amp; B62 &amp; "'!" &amp; C62))</f>
@@ -4763,13 +4763,13 @@
     </row>
     <row r="63" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A63" s="97" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="B63" s="98" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="C63" s="98" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="D63" s="101" cm="1">
         <f t="array" aca="1" ref="D63" ca="1">IF(OR(IF(OR(A63="", B63="", C63=""), "", INDIRECT("'" &amp; B63 &amp; "'!" &amp; C63))=0, IF(OR(A63="", B63="", C63=""), "", INDIRECT("'" &amp; B63 &amp; "'!" &amp; C63))=""),"",INDIRECT("'" &amp; B63 &amp; "'!" &amp; C63))</f>
@@ -4778,13 +4778,13 @@
     </row>
     <row r="64" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A64" s="83" t="s">
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="B64" s="84" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="C64" s="84" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="D64" s="105" cm="1">
         <f t="array" aca="1" ref="D64" ca="1">IF(OR(IF(OR(A64="", B64="", C64=""), "", INDIRECT("'" &amp; B64 &amp; "'!" &amp; C64))=0, IF(OR(A64="", B64="", C64=""), "", INDIRECT("'" &amp; B64 &amp; "'!" &amp; C64))=""),"",INDIRECT("'" &amp; B64 &amp; "'!" &amp; C64))</f>
@@ -4796,7 +4796,7 @@
         <v>306</v>
       </c>
       <c r="B65" s="87" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="C65" s="87" t="s">
         <v>338</v>
@@ -4808,10 +4808,10 @@
     </row>
     <row r="66" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A66" s="83" t="s">
-        <v>396</v>
+        <v>391</v>
       </c>
       <c r="B66" s="84" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="C66" s="84" t="s">
         <v>333</v>
@@ -4826,7 +4826,7 @@
         <v>307</v>
       </c>
       <c r="B67" s="87" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="C67" s="87" t="s">
         <v>339</v>
@@ -4838,10 +4838,10 @@
     </row>
     <row r="68" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A68" s="83" t="s">
-        <v>397</v>
+        <v>392</v>
       </c>
       <c r="B68" s="84" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="C68" s="84" t="s">
         <v>340</v>
@@ -4853,13 +4853,13 @@
     </row>
     <row r="69" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A69" s="97" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="B69" s="98" t="s">
-        <v>347</v>
+        <v>437</v>
       </c>
       <c r="C69" s="98" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="D69" s="101" cm="1">
         <f t="array" aca="1" ref="D69" ca="1">IF(OR(IF(OR(A69="", B69="", C69=""), "", INDIRECT("'" &amp; B69 &amp; "'!" &amp; C69))=0, IF(OR(A69="", B69="", C69=""), "", INDIRECT("'" &amp; B69 &amp; "'!" &amp; C69))=""),"",INDIRECT("'" &amp; B69 &amp; "'!" &amp; C69))</f>
@@ -4868,13 +4868,13 @@
     </row>
     <row r="70" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A70" s="83" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
       <c r="B70" s="84" t="s">
-        <v>347</v>
+        <v>437</v>
       </c>
       <c r="C70" s="84" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="D70" s="105" cm="1">
         <f t="array" aca="1" ref="D70" ca="1">IF(OR(IF(OR(A70="", B70="", C70=""), "", INDIRECT("'" &amp; B70 &amp; "'!" &amp; C70))=0, IF(OR(A70="", B70="", C70=""), "", INDIRECT("'" &amp; B70 &amp; "'!" &amp; C70))=""),"",INDIRECT("'" &amp; B70 &amp; "'!" &amp; C70))</f>
@@ -4886,7 +4886,7 @@
         <v>308</v>
       </c>
       <c r="B71" s="87" t="s">
-        <v>347</v>
+        <v>437</v>
       </c>
       <c r="C71" s="87" t="s">
         <v>338</v>
@@ -4898,10 +4898,10 @@
     </row>
     <row r="72" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A72" s="83" t="s">
-        <v>398</v>
+        <v>393</v>
       </c>
       <c r="B72" s="84" t="s">
-        <v>347</v>
+        <v>437</v>
       </c>
       <c r="C72" s="84" t="s">
         <v>333</v>
@@ -4916,7 +4916,7 @@
         <v>309</v>
       </c>
       <c r="B73" s="87" t="s">
-        <v>347</v>
+        <v>437</v>
       </c>
       <c r="C73" s="87" t="s">
         <v>339</v>
@@ -4928,10 +4928,10 @@
     </row>
     <row r="74" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A74" s="83" t="s">
-        <v>399</v>
+        <v>394</v>
       </c>
       <c r="B74" s="84" t="s">
-        <v>347</v>
+        <v>437</v>
       </c>
       <c r="C74" s="84" t="s">
         <v>340</v>
@@ -4946,10 +4946,10 @@
         <v>310</v>
       </c>
       <c r="B75" s="87" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="C75" s="87" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="D75" s="101" cm="1">
         <f t="array" aca="1" ref="D75" ca="1">IF(OR(IF(OR(A75="", B75="", C75=""), "", INDIRECT("'" &amp; B75 &amp; "'!" &amp; C75))=0, IF(OR(A75="", B75="", C75=""), "", INDIRECT("'" &amp; B75 &amp; "'!" &amp; C75))=""),"",INDIRECT("'" &amp; B75 &amp; "'!" &amp; C75))</f>
@@ -4958,13 +4958,13 @@
     </row>
     <row r="76" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A76" s="94" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="B76" s="84" t="s">
+        <v>343</v>
+      </c>
+      <c r="C76" s="88" t="s">
         <v>346</v>
-      </c>
-      <c r="C76" s="88" t="s">
-        <v>351</v>
       </c>
       <c r="D76" s="102" cm="1">
         <f t="array" aca="1" ref="D76" ca="1">IF(OR(IF(OR(A76="", B76="", C76=""), "", INDIRECT("'" &amp; B76 &amp; "'!" &amp; C76))=0, IF(OR(A76="", B76="", C76=""), "", INDIRECT("'" &amp; B76 &amp; "'!" &amp; C76))=""),"",INDIRECT("'" &amp; B76 &amp; "'!" &amp; C76))</f>
@@ -4976,10 +4976,10 @@
         <v>311</v>
       </c>
       <c r="B77" s="87" t="s">
-        <v>347</v>
+        <v>437</v>
       </c>
       <c r="C77" s="89" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="D77" s="101" cm="1">
         <f t="array" aca="1" ref="D77" ca="1">IF(OR(IF(OR(A77="", B77="", C77=""), "", INDIRECT("'" &amp; B77 &amp; "'!" &amp; C77))=0, IF(OR(A77="", B77="", C77=""), "", INDIRECT("'" &amp; B77 &amp; "'!" &amp; C77))=""),"",INDIRECT("'" &amp; B77 &amp; "'!" &amp; C77))</f>
@@ -4988,13 +4988,13 @@
     </row>
     <row r="78" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A78" s="94" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="B78" s="84" t="s">
-        <v>347</v>
+        <v>437</v>
       </c>
       <c r="C78" s="88" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="D78" s="102" cm="1">
         <f t="array" aca="1" ref="D78" ca="1">IF(OR(IF(OR(A78="", B78="", C78=""), "", INDIRECT("'" &amp; B78 &amp; "'!" &amp; C78))=0, IF(OR(A78="", B78="", C78=""), "", INDIRECT("'" &amp; B78 &amp; "'!" &amp; C78))=""),"",INDIRECT("'" &amp; B78 &amp; "'!" &amp; C78))</f>
@@ -5003,13 +5003,13 @@
     </row>
     <row r="79" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A79" s="97" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="B79" s="98" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="C79" s="98" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="D79" s="101" cm="1">
         <f t="array" aca="1" ref="D79" ca="1">IF(OR(IF(OR(A79="", B79="", C79=""), "", INDIRECT("'" &amp; B79 &amp; "'!" &amp; C79))=0, IF(OR(A79="", B79="", C79=""), "", INDIRECT("'" &amp; B79 &amp; "'!" &amp; C79))=""),"",INDIRECT("'" &amp; B79 &amp; "'!" &amp; C79))</f>
@@ -5018,13 +5018,13 @@
     </row>
     <row r="80" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A80" s="83" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="B80" s="84" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="C80" s="84" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="D80" s="105" cm="1">
         <f t="array" aca="1" ref="D80" ca="1">IF(OR(IF(OR(A80="", B80="", C80=""), "", INDIRECT("'" &amp; B80 &amp; "'!" &amp; C80))=0, IF(OR(A80="", B80="", C80=""), "", INDIRECT("'" &amp; B80 &amp; "'!" &amp; C80))=""),"",INDIRECT("'" &amp; B80 &amp; "'!" &amp; C80))</f>
@@ -5036,7 +5036,7 @@
         <v>312</v>
       </c>
       <c r="B81" s="89" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="C81" s="89" t="s">
         <v>338</v>
@@ -5048,10 +5048,10 @@
     </row>
     <row r="82" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A82" s="83" t="s">
-        <v>402</v>
+        <v>397</v>
       </c>
       <c r="B82" s="88" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="C82" s="88" t="s">
         <v>333</v>
@@ -5066,7 +5066,7 @@
         <v>313</v>
       </c>
       <c r="B83" s="89" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="C83" s="89" t="s">
         <v>339</v>
@@ -5078,10 +5078,10 @@
     </row>
     <row r="84" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A84" s="83" t="s">
-        <v>403</v>
+        <v>398</v>
       </c>
       <c r="B84" s="88" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="C84" s="88" t="s">
         <v>340</v>
@@ -5093,13 +5093,13 @@
     </row>
     <row r="85" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A85" s="97" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="B85" s="98" t="s">
-        <v>349</v>
+        <v>438</v>
       </c>
       <c r="C85" s="98" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="D85" s="101" cm="1">
         <f t="array" aca="1" ref="D85" ca="1">IF(OR(IF(OR(A85="", B85="", C85=""), "", INDIRECT("'" &amp; B85 &amp; "'!" &amp; C85))=0, IF(OR(A85="", B85="", C85=""), "", INDIRECT("'" &amp; B85 &amp; "'!" &amp; C85))=""),"",INDIRECT("'" &amp; B85 &amp; "'!" &amp; C85))</f>
@@ -5108,13 +5108,13 @@
     </row>
     <row r="86" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A86" s="83" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
       <c r="B86" s="84" t="s">
-        <v>349</v>
+        <v>438</v>
       </c>
       <c r="C86" s="84" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="D86" s="105" cm="1">
         <f t="array" aca="1" ref="D86" ca="1">IF(OR(IF(OR(A86="", B86="", C86=""), "", INDIRECT("'" &amp; B86 &amp; "'!" &amp; C86))=0, IF(OR(A86="", B86="", C86=""), "", INDIRECT("'" &amp; B86 &amp; "'!" &amp; C86))=""),"",INDIRECT("'" &amp; B86 &amp; "'!" &amp; C86))</f>
@@ -5126,7 +5126,7 @@
         <v>314</v>
       </c>
       <c r="B87" s="89" t="s">
-        <v>349</v>
+        <v>438</v>
       </c>
       <c r="C87" s="89" t="s">
         <v>338</v>
@@ -5138,10 +5138,10 @@
     </row>
     <row r="88" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A88" s="83" t="s">
-        <v>404</v>
+        <v>399</v>
       </c>
       <c r="B88" s="88" t="s">
-        <v>349</v>
+        <v>438</v>
       </c>
       <c r="C88" s="88" t="s">
         <v>333</v>
@@ -5156,7 +5156,7 @@
         <v>315</v>
       </c>
       <c r="B89" s="89" t="s">
-        <v>349</v>
+        <v>438</v>
       </c>
       <c r="C89" s="89" t="s">
         <v>339</v>
@@ -5168,10 +5168,10 @@
     </row>
     <row r="90" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A90" s="83" t="s">
-        <v>405</v>
+        <v>400</v>
       </c>
       <c r="B90" s="88" t="s">
-        <v>349</v>
+        <v>438</v>
       </c>
       <c r="C90" s="88" t="s">
         <v>340</v>
@@ -5186,10 +5186,10 @@
         <v>316</v>
       </c>
       <c r="B91" s="89" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="C91" s="89" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="D91" s="101" cm="1">
         <f t="array" aca="1" ref="D91" ca="1">IF(OR(IF(OR(A91="", B91="", C91=""), "", INDIRECT("'" &amp; B91 &amp; "'!" &amp; C91))=0, IF(OR(A91="", B91="", C91=""), "", INDIRECT("'" &amp; B91 &amp; "'!" &amp; C91))=""),"",INDIRECT("'" &amp; B91 &amp; "'!" &amp; C91))</f>
@@ -5198,13 +5198,13 @@
     </row>
     <row r="92" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A92" s="94" t="s">
-        <v>406</v>
+        <v>401</v>
       </c>
       <c r="B92" s="88" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="C92" s="88" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="D92" s="102" cm="1">
         <f t="array" aca="1" ref="D92" ca="1">IF(OR(IF(OR(A92="", B92="", C92=""), "", INDIRECT("'" &amp; B92 &amp; "'!" &amp; C92))=0, IF(OR(A92="", B92="", C92=""), "", INDIRECT("'" &amp; B92 &amp; "'!" &amp; C92))=""),"",INDIRECT("'" &amp; B92 &amp; "'!" &amp; C92))</f>
@@ -5216,10 +5216,10 @@
         <v>317</v>
       </c>
       <c r="B93" s="89" t="s">
-        <v>349</v>
+        <v>438</v>
       </c>
       <c r="C93" s="89" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="D93" s="101" cm="1">
         <f t="array" aca="1" ref="D93" ca="1">IF(OR(IF(OR(A93="", B93="", C93=""), "", INDIRECT("'" &amp; B93 &amp; "'!" &amp; C93))=0, IF(OR(A93="", B93="", C93=""), "", INDIRECT("'" &amp; B93 &amp; "'!" &amp; C93))=""),"",INDIRECT("'" &amp; B93 &amp; "'!" &amp; C93))</f>
@@ -5228,13 +5228,13 @@
     </row>
     <row r="94" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A94" s="94" t="s">
-        <v>407</v>
+        <v>402</v>
       </c>
       <c r="B94" s="88" t="s">
-        <v>349</v>
+        <v>438</v>
       </c>
       <c r="C94" s="88" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="D94" s="102" cm="1">
         <f t="array" aca="1" ref="D94" ca="1">IF(OR(IF(OR(A94="", B94="", C94=""), "", INDIRECT("'" &amp; B94 &amp; "'!" &amp; C94))=0, IF(OR(A94="", B94="", C94=""), "", INDIRECT("'" &amp; B94 &amp; "'!" &amp; C94))=""),"",INDIRECT("'" &amp; B94 &amp; "'!" &amp; C94))</f>
@@ -5242,8 +5242,8 @@
       </c>
     </row>
     <row r="95" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A95" s="125" t="s">
-        <v>437</v>
+      <c r="A95" s="107" t="s">
+        <v>432</v>
       </c>
       <c r="B95" s="89"/>
       <c r="C95" s="89"/>
@@ -5253,8 +5253,8 @@
       </c>
     </row>
     <row r="96" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A96" s="125" t="s">
-        <v>438</v>
+      <c r="A96" s="107" t="s">
+        <v>440</v>
       </c>
       <c r="B96" s="88"/>
       <c r="C96" s="88"/>
@@ -5264,7 +5264,7 @@
       </c>
     </row>
     <row r="97" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A97" s="125" t="s">
+      <c r="A97" s="107" t="s">
         <v>439</v>
       </c>
       <c r="B97" s="89"/>
@@ -5546,15 +5546,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="113" t="s">
+      <c r="A1" s="114" t="s">
         <v>134</v>
       </c>
-      <c r="B1" s="113"/>
-      <c r="C1" s="113"/>
-      <c r="D1" s="113"/>
-      <c r="E1" s="113"/>
-      <c r="F1" s="113"/>
-      <c r="G1" s="113"/>
+      <c r="B1" s="114"/>
+      <c r="C1" s="114"/>
+      <c r="D1" s="114"/>
+      <c r="E1" s="114"/>
+      <c r="F1" s="114"/>
+      <c r="G1" s="114"/>
       <c r="AE1" s="3"/>
       <c r="AF1" s="5"/>
       <c r="AG1" s="5"/>
@@ -5641,15 +5641,15 @@
       <c r="AF6" s="7"/>
     </row>
     <row r="7" spans="1:36" x14ac:dyDescent="0.2">
-      <c r="A7" s="120" t="s">
+      <c r="A7" s="121" t="s">
         <v>115</v>
       </c>
-      <c r="B7" s="112"/>
-      <c r="C7" s="112"/>
-      <c r="D7" s="112"/>
-      <c r="E7" s="112"/>
-      <c r="F7" s="112"/>
-      <c r="G7" s="112"/>
+      <c r="B7" s="113"/>
+      <c r="C7" s="113"/>
+      <c r="D7" s="113"/>
+      <c r="E7" s="113"/>
+      <c r="F7" s="113"/>
+      <c r="G7" s="113"/>
       <c r="AE7" s="7"/>
       <c r="AF7" s="7"/>
     </row>
@@ -5926,15 +5926,15 @@
       <c r="AF18" s="7"/>
     </row>
     <row r="19" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="A19" s="121" t="s">
+      <c r="A19" s="122" t="s">
         <v>120</v>
       </c>
-      <c r="B19" s="121"/>
-      <c r="C19" s="121"/>
-      <c r="D19" s="121"/>
-      <c r="E19" s="121"/>
-      <c r="F19" s="121"/>
-      <c r="G19" s="121"/>
+      <c r="B19" s="122"/>
+      <c r="C19" s="122"/>
+      <c r="D19" s="122"/>
+      <c r="E19" s="122"/>
+      <c r="F19" s="122"/>
+      <c r="G19" s="122"/>
       <c r="AE19" s="7"/>
       <c r="AF19" s="7"/>
     </row>
@@ -7657,15 +7657,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" ht="18" x14ac:dyDescent="0.25">
-      <c r="A1" s="123" t="s">
+      <c r="A1" s="124" t="s">
         <v>145</v>
       </c>
-      <c r="B1" s="112"/>
-      <c r="C1" s="112"/>
-      <c r="D1" s="112"/>
-      <c r="E1" s="112"/>
-      <c r="F1" s="112"/>
-      <c r="G1" s="112"/>
+      <c r="B1" s="113"/>
+      <c r="C1" s="113"/>
+      <c r="D1" s="113"/>
+      <c r="E1" s="113"/>
+      <c r="F1" s="113"/>
+      <c r="G1" s="113"/>
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
@@ -7731,15 +7731,15 @@
       </c>
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="A7" s="120" t="s">
+      <c r="A7" s="121" t="s">
         <v>115</v>
       </c>
-      <c r="B7" s="112"/>
-      <c r="C7" s="112"/>
-      <c r="D7" s="112"/>
-      <c r="E7" s="112"/>
-      <c r="F7" s="112"/>
-      <c r="G7" s="112"/>
+      <c r="B7" s="113"/>
+      <c r="C7" s="113"/>
+      <c r="D7" s="113"/>
+      <c r="E7" s="113"/>
+      <c r="F7" s="113"/>
+      <c r="G7" s="113"/>
       <c r="AE7" s="7"/>
       <c r="AF7" s="7"/>
     </row>
@@ -7986,15 +7986,15 @@
       </c>
     </row>
     <row r="19" spans="1:8" s="46" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="124" t="s">
+      <c r="A19" s="125" t="s">
         <v>118</v>
       </c>
-      <c r="B19" s="124"/>
-      <c r="C19" s="124"/>
-      <c r="D19" s="124"/>
-      <c r="E19" s="124"/>
-      <c r="F19" s="124"/>
-      <c r="G19" s="124"/>
+      <c r="B19" s="125"/>
+      <c r="C19" s="125"/>
+      <c r="D19" s="125"/>
+      <c r="E19" s="125"/>
+      <c r="F19" s="125"/>
+      <c r="G19" s="125"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20">
@@ -9566,15 +9566,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" ht="18" x14ac:dyDescent="0.25">
-      <c r="A1" s="123" t="s">
+      <c r="A1" s="124" t="s">
         <v>146</v>
       </c>
-      <c r="B1" s="112"/>
-      <c r="C1" s="112"/>
-      <c r="D1" s="112"/>
-      <c r="E1" s="112"/>
-      <c r="F1" s="112"/>
-      <c r="G1" s="112"/>
+      <c r="B1" s="113"/>
+      <c r="C1" s="113"/>
+      <c r="D1" s="113"/>
+      <c r="E1" s="113"/>
+      <c r="F1" s="113"/>
+      <c r="G1" s="113"/>
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
@@ -9640,15 +9640,15 @@
       </c>
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="A7" s="120" t="s">
+      <c r="A7" s="121" t="s">
         <v>115</v>
       </c>
-      <c r="B7" s="112"/>
-      <c r="C7" s="112"/>
-      <c r="D7" s="112"/>
-      <c r="E7" s="112"/>
-      <c r="F7" s="112"/>
-      <c r="G7" s="112"/>
+      <c r="B7" s="113"/>
+      <c r="C7" s="113"/>
+      <c r="D7" s="113"/>
+      <c r="E7" s="113"/>
+      <c r="F7" s="113"/>
+      <c r="G7" s="113"/>
       <c r="AE7" s="7"/>
       <c r="AF7" s="7"/>
     </row>
@@ -9895,15 +9895,15 @@
       </c>
     </row>
     <row r="19" spans="1:8" s="46" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="124" t="s">
+      <c r="A19" s="125" t="s">
         <v>151</v>
       </c>
-      <c r="B19" s="124"/>
-      <c r="C19" s="124"/>
-      <c r="D19" s="124"/>
-      <c r="E19" s="124"/>
-      <c r="F19" s="124"/>
-      <c r="G19" s="124"/>
+      <c r="B19" s="125"/>
+      <c r="C19" s="125"/>
+      <c r="D19" s="125"/>
+      <c r="E19" s="125"/>
+      <c r="F19" s="125"/>
+      <c r="G19" s="125"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20">
@@ -11475,15 +11475,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" ht="18" x14ac:dyDescent="0.25">
-      <c r="A1" s="123" t="s">
+      <c r="A1" s="124" t="s">
         <v>147</v>
       </c>
-      <c r="B1" s="112"/>
-      <c r="C1" s="112"/>
-      <c r="D1" s="112"/>
-      <c r="E1" s="112"/>
-      <c r="F1" s="112"/>
-      <c r="G1" s="112"/>
+      <c r="B1" s="113"/>
+      <c r="C1" s="113"/>
+      <c r="D1" s="113"/>
+      <c r="E1" s="113"/>
+      <c r="F1" s="113"/>
+      <c r="G1" s="113"/>
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
@@ -11549,15 +11549,15 @@
       </c>
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="A7" s="120" t="s">
+      <c r="A7" s="121" t="s">
         <v>115</v>
       </c>
-      <c r="B7" s="112"/>
-      <c r="C7" s="112"/>
-      <c r="D7" s="112"/>
-      <c r="E7" s="112"/>
-      <c r="F7" s="112"/>
-      <c r="G7" s="112"/>
+      <c r="B7" s="113"/>
+      <c r="C7" s="113"/>
+      <c r="D7" s="113"/>
+      <c r="E7" s="113"/>
+      <c r="F7" s="113"/>
+      <c r="G7" s="113"/>
       <c r="AE7" s="7"/>
       <c r="AF7" s="7"/>
     </row>
@@ -11804,15 +11804,15 @@
       </c>
     </row>
     <row r="19" spans="1:8" s="46" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="124" t="s">
+      <c r="A19" s="125" t="s">
         <v>118</v>
       </c>
-      <c r="B19" s="124"/>
-      <c r="C19" s="124"/>
-      <c r="D19" s="124"/>
-      <c r="E19" s="124"/>
-      <c r="F19" s="124"/>
-      <c r="G19" s="124"/>
+      <c r="B19" s="125"/>
+      <c r="C19" s="125"/>
+      <c r="D19" s="125"/>
+      <c r="E19" s="125"/>
+      <c r="F19" s="125"/>
+      <c r="G19" s="125"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20">
@@ -13385,15 +13385,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" ht="18" x14ac:dyDescent="0.25">
-      <c r="A1" s="123" t="s">
+      <c r="A1" s="124" t="s">
         <v>148</v>
       </c>
-      <c r="B1" s="112"/>
-      <c r="C1" s="112"/>
-      <c r="D1" s="112"/>
-      <c r="E1" s="112"/>
-      <c r="F1" s="112"/>
-      <c r="G1" s="112"/>
+      <c r="B1" s="113"/>
+      <c r="C1" s="113"/>
+      <c r="D1" s="113"/>
+      <c r="E1" s="113"/>
+      <c r="F1" s="113"/>
+      <c r="G1" s="113"/>
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
@@ -13462,15 +13462,15 @@
       </c>
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="A7" s="120" t="s">
+      <c r="A7" s="121" t="s">
         <v>115</v>
       </c>
-      <c r="B7" s="112"/>
-      <c r="C7" s="112"/>
-      <c r="D7" s="112"/>
-      <c r="E7" s="112"/>
-      <c r="F7" s="112"/>
-      <c r="G7" s="112"/>
+      <c r="B7" s="113"/>
+      <c r="C7" s="113"/>
+      <c r="D7" s="113"/>
+      <c r="E7" s="113"/>
+      <c r="F7" s="113"/>
+      <c r="G7" s="113"/>
       <c r="AE7" s="7"/>
       <c r="AF7" s="7"/>
     </row>
@@ -13717,15 +13717,15 @@
       </c>
     </row>
     <row r="19" spans="1:8" s="46" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="124" t="s">
+      <c r="A19" s="125" t="s">
         <v>151</v>
       </c>
-      <c r="B19" s="124"/>
-      <c r="C19" s="124"/>
-      <c r="D19" s="124"/>
-      <c r="E19" s="124"/>
-      <c r="F19" s="124"/>
-      <c r="G19" s="124"/>
+      <c r="B19" s="125"/>
+      <c r="C19" s="125"/>
+      <c r="D19" s="125"/>
+      <c r="E19" s="125"/>
+      <c r="F19" s="125"/>
+      <c r="G19" s="125"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20">
@@ -15314,7 +15314,7 @@
         <v>6</v>
       </c>
       <c r="C2" s="33" t="s">
-        <v>408</v>
+        <v>403</v>
       </c>
       <c r="E2" s="34" t="s">
         <v>106</v>
@@ -15329,7 +15329,7 @@
         <v>8</v>
       </c>
       <c r="C3" s="33" t="s">
-        <v>409</v>
+        <v>404</v>
       </c>
       <c r="G3" s="6"/>
     </row>
@@ -15341,7 +15341,7 @@
         <v>10</v>
       </c>
       <c r="C4" s="33" t="s">
-        <v>410</v>
+        <v>405</v>
       </c>
       <c r="G4" s="6"/>
     </row>
@@ -15353,7 +15353,7 @@
         <v>12</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>411</v>
+        <v>406</v>
       </c>
       <c r="G5" s="6"/>
     </row>
@@ -15365,7 +15365,7 @@
         <v>14</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>412</v>
+        <v>407</v>
       </c>
       <c r="G6" s="6"/>
     </row>
@@ -15377,7 +15377,7 @@
         <v>16</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>413</v>
+        <v>408</v>
       </c>
       <c r="G7" s="6"/>
     </row>
@@ -15389,7 +15389,7 @@
         <v>18</v>
       </c>
       <c r="C8" s="33" t="s">
-        <v>414</v>
+        <v>409</v>
       </c>
       <c r="G8" s="6"/>
     </row>
@@ -15401,7 +15401,7 @@
         <v>20</v>
       </c>
       <c r="C9" s="33" t="s">
-        <v>415</v>
+        <v>410</v>
       </c>
       <c r="G9" s="6"/>
     </row>
@@ -15413,7 +15413,7 @@
         <v>22</v>
       </c>
       <c r="C10" s="33" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
       <c r="G10" s="6"/>
     </row>
@@ -15425,7 +15425,7 @@
         <v>24</v>
       </c>
       <c r="C11" s="33" t="s">
-        <v>417</v>
+        <v>412</v>
       </c>
       <c r="G11" s="6"/>
     </row>
@@ -15449,7 +15449,7 @@
         <v>28</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>418</v>
+        <v>413</v>
       </c>
       <c r="G13" s="6"/>
     </row>
@@ -15461,7 +15461,7 @@
         <v>30</v>
       </c>
       <c r="C14" s="33" t="s">
-        <v>419</v>
+        <v>414</v>
       </c>
       <c r="G14" s="6"/>
     </row>
@@ -15473,7 +15473,7 @@
         <v>32</v>
       </c>
       <c r="C15" s="33" t="s">
-        <v>420</v>
+        <v>415</v>
       </c>
       <c r="G15" s="6"/>
     </row>
@@ -15485,7 +15485,7 @@
         <v>34</v>
       </c>
       <c r="C16" s="33" t="s">
-        <v>421</v>
+        <v>416</v>
       </c>
       <c r="G16" s="6"/>
     </row>
@@ -15497,7 +15497,7 @@
         <v>36</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>422</v>
+        <v>417</v>
       </c>
       <c r="G17" s="6"/>
     </row>
@@ -15509,7 +15509,7 @@
         <v>38</v>
       </c>
       <c r="C18" s="33" t="s">
-        <v>423</v>
+        <v>418</v>
       </c>
       <c r="G18" s="6"/>
     </row>
@@ -15521,7 +15521,7 @@
         <v>40</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>424</v>
+        <v>419</v>
       </c>
       <c r="G19" s="6"/>
     </row>
@@ -15533,7 +15533,7 @@
         <v>42</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>425</v>
+        <v>420</v>
       </c>
       <c r="G20" s="6"/>
     </row>
@@ -15545,7 +15545,7 @@
         <v>44</v>
       </c>
       <c r="C21" s="33" t="s">
-        <v>426</v>
+        <v>421</v>
       </c>
       <c r="G21" s="6"/>
     </row>
@@ -15557,7 +15557,7 @@
         <v>46</v>
       </c>
       <c r="C22" s="33" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
       <c r="G22" s="6"/>
     </row>
@@ -15569,7 +15569,7 @@
         <v>48</v>
       </c>
       <c r="C23" s="33" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
       <c r="G23" s="6"/>
     </row>
@@ -15581,7 +15581,7 @@
         <v>50</v>
       </c>
       <c r="C24" s="33" t="s">
-        <v>429</v>
+        <v>424</v>
       </c>
       <c r="G24" s="6"/>
     </row>
@@ -15593,7 +15593,7 @@
         <v>52</v>
       </c>
       <c r="C25" s="33" t="s">
-        <v>430</v>
+        <v>425</v>
       </c>
       <c r="G25" s="6"/>
     </row>
@@ -15605,7 +15605,7 @@
         <v>54</v>
       </c>
       <c r="C26" s="33" t="s">
-        <v>431</v>
+        <v>426</v>
       </c>
       <c r="G26" s="6"/>
     </row>
@@ -15617,7 +15617,7 @@
         <v>56</v>
       </c>
       <c r="C27" s="33" t="s">
-        <v>432</v>
+        <v>427</v>
       </c>
       <c r="G27" s="6"/>
     </row>
@@ -15629,7 +15629,7 @@
         <v>58</v>
       </c>
       <c r="C28" s="33" t="s">
-        <v>433</v>
+        <v>428</v>
       </c>
       <c r="G28" s="6"/>
     </row>
@@ -15641,7 +15641,7 @@
         <v>60</v>
       </c>
       <c r="C29" s="33" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
       <c r="G29" s="6"/>
     </row>
@@ -15653,7 +15653,7 @@
         <v>62</v>
       </c>
       <c r="C30" s="33" t="s">
-        <v>435</v>
+        <v>430</v>
       </c>
       <c r="G30" s="6"/>
     </row>
@@ -15665,7 +15665,7 @@
         <v>64</v>
       </c>
       <c r="C31" s="33" t="s">
-        <v>436</v>
+        <v>431</v>
       </c>
       <c r="G31" s="6"/>
     </row>
@@ -15679,7 +15679,7 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="C37" s="103" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
@@ -37698,12 +37698,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="18" x14ac:dyDescent="0.25">
-      <c r="A1" s="113" t="s">
+      <c r="A1" s="114" t="s">
         <v>79</v>
       </c>
-      <c r="B1" s="113"/>
-      <c r="C1" s="113"/>
-      <c r="D1" s="113"/>
+      <c r="B1" s="114"/>
+      <c r="C1" s="114"/>
+      <c r="D1" s="114"/>
       <c r="K1" s="9"/>
       <c r="L1" s="9"/>
     </row>
@@ -37797,12 +37797,12 @@
       <c r="Q11" s="9"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="114" t="s">
+      <c r="A12" s="115" t="s">
         <v>87</v>
       </c>
-      <c r="B12" s="114"/>
-      <c r="C12" s="114"/>
-      <c r="D12" s="114"/>
+      <c r="B12" s="115"/>
+      <c r="C12" s="115"/>
+      <c r="D12" s="115"/>
       <c r="Q12" s="9"/>
     </row>
     <row r="13" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
@@ -37934,12 +37934,12 @@
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A26" s="115" t="s">
+      <c r="A26" s="116" t="s">
         <v>96</v>
       </c>
-      <c r="B26" s="112"/>
-      <c r="C26" s="112"/>
-      <c r="D26" s="112"/>
+      <c r="B26" s="113"/>
+      <c r="C26" s="113"/>
+      <c r="D26" s="113"/>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
@@ -37973,10 +37973,10 @@
       <c r="F30" s="7"/>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A31" s="110"/>
-      <c r="B31" s="111"/>
-      <c r="C31" s="112"/>
-      <c r="D31" s="112"/>
+      <c r="A31" s="111"/>
+      <c r="B31" s="112"/>
+      <c r="C31" s="113"/>
+      <c r="D31" s="113"/>
       <c r="F31" s="7"/>
     </row>
     <row r="32" spans="1:15" ht="13.35" customHeight="1" x14ac:dyDescent="0.2">
@@ -38605,16 +38605,16 @@
       </c>
     </row>
     <row r="21" spans="1:6" ht="19.7" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="116" t="s">
+      <c r="A21" s="117" t="s">
         <v>172</v>
       </c>
-      <c r="B21" s="112"/>
-      <c r="C21" s="112"/>
-      <c r="D21" s="116" t="s">
+      <c r="B21" s="113"/>
+      <c r="C21" s="113"/>
+      <c r="D21" s="117" t="s">
         <v>247</v>
       </c>
-      <c r="E21" s="112"/>
-      <c r="F21" s="112"/>
+      <c r="E21" s="113"/>
+      <c r="F21" s="113"/>
     </row>
     <row r="22" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A22" s="49" t="s">
@@ -38765,11 +38765,11 @@
       </c>
     </row>
     <row r="34" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A34" s="116" t="s">
+      <c r="A34" s="117" t="s">
         <v>176</v>
       </c>
-      <c r="B34" s="116"/>
-      <c r="C34" s="116"/>
+      <c r="B34" s="117"/>
+      <c r="C34" s="117"/>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" t="str">
@@ -38888,11 +38888,11 @@
       </c>
     </row>
     <row r="46" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A46" s="116" t="s">
+      <c r="A46" s="117" t="s">
         <v>177</v>
       </c>
-      <c r="B46" s="116"/>
-      <c r="C46" s="116"/>
+      <c r="B46" s="117"/>
+      <c r="C46" s="117"/>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A47" t="str">
@@ -39011,11 +39011,11 @@
       </c>
     </row>
     <row r="58" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A58" s="117" t="s">
+      <c r="A58" s="118" t="s">
         <v>205</v>
       </c>
-      <c r="B58" s="117"/>
-      <c r="C58" s="117"/>
+      <c r="B58" s="118"/>
+      <c r="C58" s="118"/>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A59" t="str">
@@ -39134,11 +39134,11 @@
       </c>
     </row>
     <row r="70" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A70" s="117" t="s">
+      <c r="A70" s="118" t="s">
         <v>206</v>
       </c>
-      <c r="B70" s="117"/>
-      <c r="C70" s="117"/>
+      <c r="B70" s="118"/>
+      <c r="C70" s="118"/>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A71" t="str">
@@ -39298,10 +39298,10 @@
       </c>
     </row>
     <row r="86" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A86" s="116" t="s">
+      <c r="A86" s="117" t="s">
         <v>182</v>
       </c>
-      <c r="B86" s="116"/>
+      <c r="B86" s="117"/>
       <c r="F86" t="s">
         <v>195</v>
       </c>
@@ -39612,12 +39612,12 @@
       </c>
     </row>
     <row r="3" spans="1:9" ht="99.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="119" t="str">
+      <c r="B3" s="120" t="str">
         <f>"Here are the estimates you have requested with respect to the diminution of earning capacity and associated economic impairment sustained by your client. The following records were considered in connection with the opinion below: "&amp;Inputs!B20&amp;"."</f>
         <v>Here are the estimates you have requested with respect to the diminution of earning capacity and associated economic impairment sustained by your client. The following records were considered in connection with the opinion below: Tax Returns 2020-2024, W-2s from ABC, Co. Inc; Schedule C's and the Claimant Information Sheet..</v>
       </c>
-      <c r="C3" s="119"/>
-      <c r="D3" s="119"/>
+      <c r="C3" s="120"/>
+      <c r="D3" s="120"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="61" t="s">
@@ -39946,12 +39946,12 @@
       <c r="G21" s="60"/>
     </row>
     <row r="22" spans="1:7" ht="65.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="118" t="str">
+      <c r="B22" s="119" t="str">
         <f>"1.     Earnings and Employment Background indicates that your client was working as a "&amp;Inputs!$D$20&amp;" at the time of the accident."</f>
         <v>1.     Earnings and Employment Background indicates that your client was working as a Plumber for ABC, Inc at the time of the accident.</v>
       </c>
-      <c r="C22" s="118"/>
-      <c r="D22" s="118"/>
+      <c r="C22" s="119"/>
+      <c r="D22" s="119"/>
       <c r="E22" s="70" t="b">
         <v>0</v>
       </c>
@@ -39973,12 +39973,12 @@
       <c r="A24" s="8" t="s">
         <v>250</v>
       </c>
-      <c r="B24" s="118" t="str">
+      <c r="B24" s="119" t="str">
         <f>_xlfn._LONGTEXT("Discount Rates form the basis upon which post-trial earning capacity streams are commuted to present value. The discounting ensures that the lump sum award will dissipate entirely by the end of the calculating period and will be used to replicate the stre","am of anticipated earning capacity, without windfall to your client. This analysis employs a laddered discount rate approach with rates derived from current rates of interest on AAA-rated municipal bonds ranging from ")&amp;TEXT(Inputs!$E$22,"0.0%")&amp;" to "&amp;TEXT(Inputs!$F$22,"0.0%")&amp;"."</f>
         <v>Discount Rates form the basis upon which post-trial earning capacity streams are commuted to present value. The discounting ensures that the lump sum award will dissipate entirely by the end of the calculating period and will be used to replicate the stream of anticipated earning capacity, without windfall to your client. This analysis employs a laddered discount rate approach with rates derived from current rates of interest on AAA-rated municipal bonds ranging from 2.3% to 3.3%.</v>
       </c>
-      <c r="C24" s="118"/>
-      <c r="D24" s="118"/>
+      <c r="C24" s="119"/>
+      <c r="D24" s="119"/>
       <c r="E24" s="70" t="b">
         <v>0</v>
       </c>
@@ -39987,12 +39987,12 @@
       <c r="A25" s="8" t="s">
         <v>251</v>
       </c>
-      <c r="B25" s="118" t="str">
+      <c r="B25" s="119" t="str">
         <f>CONCATENATE(_xlfn._LONGTEXT("Below Market Discount Rates form the basis upon which post-trial earning capacity streams are commuted to present value. The discounting ensures that the lump sum award will dissipate entirely by the end of the calculating period and will be used to repli","cate the stream of anticipated earning capacity, without windfall to your client. This analysis employs a laddered discount rate approach with rates derived from of current real rates of interest on AAA-rated municipal bonds adjusted for the forecased int","ermediate long run inflation estimate as reported in the Annual Report of the Board of Trustees of the Social Security Administration (2025). These rates currently range from "),TEXT(Inputs!$E$22,"0.0%")," to ",TEXT(Inputs!$F$22,"0.0%"),".")</f>
         <v>Below Market Discount Rates form the basis upon which post-trial earning capacity streams are commuted to present value. The discounting ensures that the lump sum award will dissipate entirely by the end of the calculating period and will be used to replicate the stream of anticipated earning capacity, without windfall to your client. This analysis employs a laddered discount rate approach with rates derived from of current real rates of interest on AAA-rated municipal bonds adjusted for the forecased intermediate long run inflation estimate as reported in the Annual Report of the Board of Trustees of the Social Security Administration (2025). These rates currently range from 2.3% to 3.3%.</v>
       </c>
-      <c r="C25" s="118"/>
-      <c r="D25" s="118"/>
+      <c r="C25" s="119"/>
+      <c r="D25" s="119"/>
       <c r="E25" s="70" t="b">
         <v>0</v>
       </c>
@@ -40001,12 +40001,12 @@
       <c r="A26" s="8" t="s">
         <v>253</v>
       </c>
-      <c r="B26" s="118" t="str">
+      <c r="B26" s="119" t="str">
         <f>_xlfn._LONGTEXT("Discount Rates form the basis upon which post-trial earning capacity streams are commuted to present value. The discounting ensures that the lump sum award will dissipate entirely by the end of the calculating period and will be used to replicate the stre","am of anticipated earning capacity, without windfall to your client. This analysis employs a laddered discount rate approach with rates derived from current rates of interest on AAA-rated municipal bonds ranging from ")&amp;TEXT(Inputs!$E$23,"0.0%")&amp;" to "&amp;TEXT(Inputs!$F$23,"0.0%")&amp;"."</f>
         <v>Discount Rates form the basis upon which post-trial earning capacity streams are commuted to present value. The discounting ensures that the lump sum award will dissipate entirely by the end of the calculating period and will be used to replicate the stream of anticipated earning capacity, without windfall to your client. This analysis employs a laddered discount rate approach with rates derived from current rates of interest on AAA-rated municipal bonds ranging from 2.3% to 3.9%.</v>
       </c>
-      <c r="C26" s="118"/>
-      <c r="D26" s="118"/>
+      <c r="C26" s="119"/>
+      <c r="D26" s="119"/>
       <c r="E26" s="70" t="b">
         <v>0</v>
       </c>
@@ -40146,15 +40146,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="113" t="s">
+      <c r="A1" s="114" t="s">
         <v>143</v>
       </c>
-      <c r="B1" s="113"/>
-      <c r="C1" s="113"/>
-      <c r="D1" s="113"/>
-      <c r="E1" s="113"/>
-      <c r="F1" s="113"/>
-      <c r="G1" s="113"/>
+      <c r="B1" s="114"/>
+      <c r="C1" s="114"/>
+      <c r="D1" s="114"/>
+      <c r="E1" s="114"/>
+      <c r="F1" s="114"/>
+      <c r="G1" s="114"/>
       <c r="AE1" s="3"/>
       <c r="AF1" s="5"/>
       <c r="AG1" s="5"/>
@@ -40247,15 +40247,15 @@
       <c r="AF6" s="7"/>
     </row>
     <row r="7" spans="1:36" x14ac:dyDescent="0.2">
-      <c r="A7" s="120" t="s">
+      <c r="A7" s="121" t="s">
         <v>115</v>
       </c>
-      <c r="B7" s="112"/>
-      <c r="C7" s="112"/>
-      <c r="D7" s="112"/>
-      <c r="E7" s="112"/>
-      <c r="F7" s="112"/>
-      <c r="G7" s="112"/>
+      <c r="B7" s="113"/>
+      <c r="C7" s="113"/>
+      <c r="D7" s="113"/>
+      <c r="E7" s="113"/>
+      <c r="F7" s="113"/>
+      <c r="G7" s="113"/>
       <c r="AE7" s="7"/>
       <c r="AF7" s="7"/>
     </row>
@@ -40539,15 +40539,15 @@
       <c r="AF18" s="7"/>
     </row>
     <row r="19" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="A19" s="121" t="s">
+      <c r="A19" s="122" t="s">
         <v>118</v>
       </c>
-      <c r="B19" s="121"/>
-      <c r="C19" s="121"/>
-      <c r="D19" s="121"/>
-      <c r="E19" s="121"/>
-      <c r="F19" s="121"/>
-      <c r="G19" s="121"/>
+      <c r="B19" s="122"/>
+      <c r="C19" s="122"/>
+      <c r="D19" s="122"/>
+      <c r="E19" s="122"/>
+      <c r="F19" s="122"/>
+      <c r="G19" s="122"/>
       <c r="AE19" s="7"/>
       <c r="AF19" s="7"/>
     </row>
@@ -42273,15 +42273,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="113" t="s">
+      <c r="A1" s="114" t="s">
         <v>144</v>
       </c>
-      <c r="B1" s="113"/>
-      <c r="C1" s="113"/>
-      <c r="D1" s="113"/>
-      <c r="E1" s="113"/>
-      <c r="F1" s="113"/>
-      <c r="G1" s="113"/>
+      <c r="B1" s="114"/>
+      <c r="C1" s="114"/>
+      <c r="D1" s="114"/>
+      <c r="E1" s="114"/>
+      <c r="F1" s="114"/>
+      <c r="G1" s="114"/>
       <c r="AE1" s="3"/>
       <c r="AF1" s="5"/>
       <c r="AG1" s="5"/>
@@ -42371,15 +42371,15 @@
       <c r="AF6" s="7"/>
     </row>
     <row r="7" spans="1:36" x14ac:dyDescent="0.2">
-      <c r="A7" s="120" t="s">
+      <c r="A7" s="121" t="s">
         <v>115</v>
       </c>
-      <c r="B7" s="112"/>
-      <c r="C7" s="112"/>
-      <c r="D7" s="112"/>
-      <c r="E7" s="112"/>
-      <c r="F7" s="112"/>
-      <c r="G7" s="112"/>
+      <c r="B7" s="113"/>
+      <c r="C7" s="113"/>
+      <c r="D7" s="113"/>
+      <c r="E7" s="113"/>
+      <c r="F7" s="113"/>
+      <c r="G7" s="113"/>
       <c r="AE7" s="7"/>
       <c r="AF7" s="7"/>
     </row>
@@ -42656,15 +42656,15 @@
       <c r="AF18" s="7"/>
     </row>
     <row r="19" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="A19" s="121" t="s">
+      <c r="A19" s="122" t="s">
         <v>120</v>
       </c>
-      <c r="B19" s="121"/>
-      <c r="C19" s="121"/>
-      <c r="D19" s="121"/>
-      <c r="E19" s="121"/>
-      <c r="F19" s="121"/>
-      <c r="G19" s="121"/>
+      <c r="B19" s="122"/>
+      <c r="C19" s="122"/>
+      <c r="D19" s="122"/>
+      <c r="E19" s="122"/>
+      <c r="F19" s="122"/>
+      <c r="G19" s="122"/>
       <c r="AE19" s="7"/>
       <c r="AF19" s="7"/>
     </row>
@@ -44387,15 +44387,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="113" t="s">
+      <c r="A1" s="114" t="s">
         <v>131</v>
       </c>
-      <c r="B1" s="113"/>
-      <c r="C1" s="113"/>
-      <c r="D1" s="113"/>
-      <c r="E1" s="113"/>
-      <c r="F1" s="113"/>
-      <c r="G1" s="113"/>
+      <c r="B1" s="114"/>
+      <c r="C1" s="114"/>
+      <c r="D1" s="114"/>
+      <c r="E1" s="114"/>
+      <c r="F1" s="114"/>
+      <c r="G1" s="114"/>
       <c r="AE1" s="3"/>
       <c r="AF1" s="5"/>
       <c r="AG1" s="5"/>
@@ -44482,15 +44482,15 @@
       <c r="AF6" s="7"/>
     </row>
     <row r="7" spans="1:36" x14ac:dyDescent="0.2">
-      <c r="A7" s="120" t="s">
+      <c r="A7" s="121" t="s">
         <v>115</v>
       </c>
-      <c r="B7" s="112"/>
-      <c r="C7" s="112"/>
-      <c r="D7" s="112"/>
-      <c r="E7" s="112"/>
-      <c r="F7" s="112"/>
-      <c r="G7" s="112"/>
+      <c r="B7" s="113"/>
+      <c r="C7" s="113"/>
+      <c r="D7" s="113"/>
+      <c r="E7" s="113"/>
+      <c r="F7" s="113"/>
+      <c r="G7" s="113"/>
       <c r="AE7" s="7"/>
       <c r="AF7" s="7"/>
     </row>
@@ -44767,15 +44767,15 @@
       <c r="AF18" s="7"/>
     </row>
     <row r="19" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="A19" s="121" t="s">
+      <c r="A19" s="122" t="s">
         <v>118</v>
       </c>
-      <c r="B19" s="121"/>
-      <c r="C19" s="121"/>
-      <c r="D19" s="121"/>
-      <c r="E19" s="121"/>
-      <c r="F19" s="121"/>
-      <c r="G19" s="121"/>
+      <c r="B19" s="122"/>
+      <c r="C19" s="122"/>
+      <c r="D19" s="122"/>
+      <c r="E19" s="122"/>
+      <c r="F19" s="122"/>
+      <c r="G19" s="122"/>
       <c r="AE19" s="7"/>
       <c r="AF19" s="7"/>
     </row>
@@ -46498,15 +46498,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="113" t="s">
+      <c r="A1" s="114" t="s">
         <v>132</v>
       </c>
-      <c r="B1" s="113"/>
-      <c r="C1" s="113"/>
-      <c r="D1" s="113"/>
-      <c r="E1" s="113"/>
-      <c r="F1" s="113"/>
-      <c r="G1" s="113"/>
+      <c r="B1" s="114"/>
+      <c r="C1" s="114"/>
+      <c r="D1" s="114"/>
+      <c r="E1" s="114"/>
+      <c r="F1" s="114"/>
+      <c r="G1" s="114"/>
       <c r="AE1" s="3"/>
       <c r="AF1" s="5"/>
       <c r="AG1" s="5"/>
@@ -46596,15 +46596,15 @@
       <c r="AF6" s="7"/>
     </row>
     <row r="7" spans="1:36" x14ac:dyDescent="0.2">
-      <c r="A7" s="120" t="s">
+      <c r="A7" s="121" t="s">
         <v>115</v>
       </c>
-      <c r="B7" s="112"/>
-      <c r="C7" s="112"/>
-      <c r="D7" s="112"/>
-      <c r="E7" s="112"/>
-      <c r="F7" s="112"/>
-      <c r="G7" s="112"/>
+      <c r="B7" s="113"/>
+      <c r="C7" s="113"/>
+      <c r="D7" s="113"/>
+      <c r="E7" s="113"/>
+      <c r="F7" s="113"/>
+      <c r="G7" s="113"/>
       <c r="AE7" s="7"/>
       <c r="AF7" s="7"/>
     </row>
@@ -46881,15 +46881,15 @@
       <c r="AF18" s="7"/>
     </row>
     <row r="19" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="A19" s="122" t="s">
+      <c r="A19" s="123" t="s">
         <v>152</v>
       </c>
-      <c r="B19" s="121"/>
-      <c r="C19" s="121"/>
-      <c r="D19" s="121"/>
-      <c r="E19" s="121"/>
-      <c r="F19" s="121"/>
-      <c r="G19" s="121"/>
+      <c r="B19" s="122"/>
+      <c r="C19" s="122"/>
+      <c r="D19" s="122"/>
+      <c r="E19" s="122"/>
+      <c r="F19" s="122"/>
+      <c r="G19" s="122"/>
       <c r="AE19" s="7"/>
       <c r="AF19" s="7"/>
     </row>
@@ -48612,15 +48612,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="113" t="s">
+      <c r="A1" s="114" t="s">
         <v>133</v>
       </c>
-      <c r="B1" s="113"/>
-      <c r="C1" s="113"/>
-      <c r="D1" s="113"/>
-      <c r="E1" s="113"/>
-      <c r="F1" s="113"/>
-      <c r="G1" s="113"/>
+      <c r="B1" s="114"/>
+      <c r="C1" s="114"/>
+      <c r="D1" s="114"/>
+      <c r="E1" s="114"/>
+      <c r="F1" s="114"/>
+      <c r="G1" s="114"/>
       <c r="AE1" s="3"/>
       <c r="AF1" s="5"/>
       <c r="AG1" s="5"/>
@@ -48707,15 +48707,15 @@
       <c r="AF6" s="7"/>
     </row>
     <row r="7" spans="1:36" x14ac:dyDescent="0.2">
-      <c r="A7" s="120" t="s">
+      <c r="A7" s="121" t="s">
         <v>115</v>
       </c>
-      <c r="B7" s="112"/>
-      <c r="C7" s="112"/>
-      <c r="D7" s="112"/>
-      <c r="E7" s="112"/>
-      <c r="F7" s="112"/>
-      <c r="G7" s="112"/>
+      <c r="B7" s="113"/>
+      <c r="C7" s="113"/>
+      <c r="D7" s="113"/>
+      <c r="E7" s="113"/>
+      <c r="F7" s="113"/>
+      <c r="G7" s="113"/>
       <c r="AE7" s="7"/>
       <c r="AF7" s="7"/>
     </row>
@@ -48992,15 +48992,15 @@
       <c r="AF18" s="7"/>
     </row>
     <row r="19" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="A19" s="121" t="s">
+      <c r="A19" s="122" t="s">
         <v>118</v>
       </c>
-      <c r="B19" s="121"/>
-      <c r="C19" s="121"/>
-      <c r="D19" s="121"/>
-      <c r="E19" s="121"/>
-      <c r="F19" s="121"/>
-      <c r="G19" s="121"/>
+      <c r="B19" s="122"/>
+      <c r="C19" s="122"/>
+      <c r="D19" s="122"/>
+      <c r="E19" s="122"/>
+      <c r="F19" s="122"/>
+      <c r="G19" s="122"/>
       <c r="AE19" s="7"/>
       <c r="AF19" s="7"/>
     </row>

</xml_diff>

<commit_message>
Further Corrections & Updates
</commit_message>
<xml_diff>
--- a/EconAutomation/src/supporting_docs/sorted_econ_files/PV2 (color coded).xlsx
+++ b/EconAutomation/src/supporting_docs/sorted_econ_files/PV2 (color coded).xlsx
@@ -9,7 +9,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EricBussey\GitHub\EconAutomation-REP\EconAutomation\src\supporting_docs\sorted_econ_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA190262-7409-40D4-A646-59372B6C3F4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0F44193-C338-4DAD-9AC2-39CE075C7C08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-60" windowWidth="29040" windowHeight="15720" tabRatio="795" xr2:uid="{25EC3B8A-402B-47FF-80A9-5B0690A475CD}"/>
   </bookViews>
@@ -112,7 +112,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3634" uniqueCount="441">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3643" uniqueCount="449">
   <si>
     <t>Year</t>
   </si>
@@ -1437,6 +1437,82 @@
   <si>
     <t>PV2_disc_rate_real</t>
   </si>
+  <si>
+    <t>eff_tax_rate</t>
+  </si>
+  <si>
+    <t>E5</t>
+  </si>
+  <si>
+    <t>PV2_disc_rate_low</t>
+  </si>
+  <si>
+    <t>PV2_disc_rate_high</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Functionally: </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="9"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>life expectancy from trial + age at trial</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Age at accident is calculated = LE from accident </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">If LCP with annual costs is present, number is pulled from </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <u/>
+        <sz val="9"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>LCP report instead</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">If only earnings, </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="9"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">LE at trial (calculated using LE from accident) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">+ </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="9"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>age at trial</t>
+    </r>
+  </si>
 </sst>
 </file>
 
@@ -1451,7 +1527,7 @@
     <numFmt numFmtId="168" formatCode="0.0000"/>
     <numFmt numFmtId="169" formatCode="0.000"/>
   </numFmts>
-  <fonts count="34" x14ac:knownFonts="1">
+  <fonts count="37" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -1666,6 +1742,25 @@
       <u/>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="9"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <u/>
+      <sz val="9"/>
+      <name val="Segoe UI"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -2065,7 +2160,7 @@
     <xf numFmtId="9" fontId="18" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="30" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="126">
+  <cellXfs count="129">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2325,6 +2420,15 @@
     <xf numFmtId="0" fontId="17" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="29" fillId="6" borderId="12" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="13" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Currency" xfId="5" builtinId="4"/>
@@ -5275,16 +5379,24 @@
       </c>
     </row>
     <row r="98" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A98" s="94"/>
-      <c r="B98" s="88"/>
-      <c r="C98" s="88"/>
-      <c r="D98" s="85" t="str" cm="1">
+      <c r="A98" s="94" t="s">
+        <v>441</v>
+      </c>
+      <c r="B98" s="88" t="s">
+        <v>332</v>
+      </c>
+      <c r="C98" s="88" t="s">
+        <v>442</v>
+      </c>
+      <c r="D98" s="126" cm="1">
         <f t="array" aca="1" ref="D98" ca="1">IF(OR(IF(OR(A98="", B98="", C98=""), "", INDIRECT("'" &amp; B98 &amp; "'!" &amp; C98))=0, IF(OR(A98="", B98="", C98=""), "", INDIRECT("'" &amp; B98 &amp; "'!" &amp; C98))=""),"",INDIRECT("'" &amp; B98 &amp; "'!" &amp; C98))</f>
-        <v/>
+        <v>0.1</v>
       </c>
     </row>
     <row r="99" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A99" s="95"/>
+      <c r="A99" s="127" t="s">
+        <v>443</v>
+      </c>
       <c r="B99" s="89"/>
       <c r="C99" s="89"/>
       <c r="D99" s="82" t="str" cm="1">
@@ -5293,7 +5405,9 @@
       </c>
     </row>
     <row r="100" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A100" s="94"/>
+      <c r="A100" s="127" t="s">
+        <v>444</v>
+      </c>
       <c r="B100" s="88"/>
       <c r="C100" s="88"/>
       <c r="D100" s="85" t="str" cm="1">
@@ -38380,7 +38494,7 @@
   <sheetPr>
     <tabColor rgb="FF70AD47"/>
   </sheetPr>
-  <dimension ref="A1:H106"/>
+  <dimension ref="A1:L106"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="32.42578125" customWidth="1"/>
@@ -38547,7 +38661,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" s="75" t="str">
         <f>"Date of "&amp;B19</f>
         <v>Date of Trial</v>
@@ -38565,7 +38679,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" s="75" t="s">
         <v>168</v>
       </c>
@@ -38582,15 +38696,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" s="75" t="s">
         <v>169</v>
       </c>
       <c r="B19" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" ht="99.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L19" s="128" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" ht="99.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="76" t="s">
         <v>171</v>
       </c>
@@ -38604,7 +38721,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="19.7" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12" ht="19.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="117" t="s">
         <v>172</v>
       </c>
@@ -38615,8 +38732,11 @@
       </c>
       <c r="E21" s="113"/>
       <c r="F21" s="113"/>
-    </row>
-    <row r="22" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="L21" s="128" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" ht="15" x14ac:dyDescent="0.25">
       <c r="A22" s="49" t="s">
         <v>173</v>
       </c>
@@ -38636,7 +38756,7 @@
         <v>3.2969999999999999E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12" ht="15" x14ac:dyDescent="0.25">
       <c r="A23" s="49" t="str">
         <f>"Base 1: "&amp;TEXT(B87,"$#,##0")</f>
         <v>Base 1: $67,453</v>
@@ -38656,8 +38776,11 @@
         <f t="array" ref="F23">MAX(IF(ISNUMBER('Base 1 PV Loss To Age'!D20:D49),'Base 1 PV Loss To Age'!D20:D49))</f>
         <v>3.9269999999999999E-2</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="L23" s="128" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" t="str">
         <f>"Loss To "&amp;$B$19</f>
         <v>Loss To Trial</v>
@@ -38669,7 +38792,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" t="str">
         <f>"Fringe Benefits Loss To "&amp;$B$19</f>
         <v>Fringe Benefits Loss To Trial</v>
@@ -38680,8 +38803,11 @@
       <c r="C25" s="53" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="L25" s="128" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" t="str">
         <f>"Meal Cost to "&amp;$B$19</f>
         <v>Meal Cost to Trial</v>
@@ -38693,7 +38819,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" t="str">
         <f>"Household Service Loss To "&amp;$B$19</f>
         <v>Household Service Loss To Trial</v>
@@ -38705,7 +38831,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>175</v>
       </c>
@@ -38713,7 +38839,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" t="str">
         <f>"After Credit 1: "&amp;TEXT(B88,"$#,##0")</f>
         <v>After Credit 1: $141,416</v>
@@ -38722,7 +38848,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A30" t="str">
         <f>"After Credit 2: "&amp;TEXT(B89,"$#,##0")</f>
         <v>After Credit 2: $250,000</v>
@@ -38731,7 +38857,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A31" t="str">
         <f>"After Credit 3: "&amp;TEXT(B90,"$#,##0")</f>
         <v>After Credit 3: $75,000</v>
@@ -38740,7 +38866,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A32" t="str">
         <f>"Fringe Benefits Loss From "&amp;$B$19</f>
         <v>Fringe Benefits Loss From Trial</v>
@@ -39580,6 +39706,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Major bugfixes, pydantic integration
</commit_message>
<xml_diff>
--- a/EconAutomation/src/supporting_docs/sorted_econ_files/PV2 (color coded).xlsx
+++ b/EconAutomation/src/supporting_docs/sorted_econ_files/PV2 (color coded).xlsx
@@ -9,9 +9,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EricBussey\GitHub\EconAutomation-REP\EconAutomation\src\supporting_docs\sorted_econ_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0F44193-C338-4DAD-9AC2-39CE075C7C08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FA4E890-3D2A-46A8-B39D-0AC2C2146075}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-60" windowWidth="29040" windowHeight="15720" tabRatio="795" xr2:uid="{25EC3B8A-402B-47FF-80A9-5B0690A475CD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="795" xr2:uid="{25EC3B8A-402B-47FF-80A9-5B0690A475CD}"/>
   </bookViews>
   <sheets>
     <sheet name="REPORT_OUTPUTS" sheetId="33" r:id="rId1"/>
@@ -2388,6 +2388,15 @@
     <xf numFmtId="0" fontId="29" fillId="13" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="9" fontId="29" fillId="6" borderId="12" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="13" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="26" fillId="23" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2420,15 +2429,6 @@
     <xf numFmtId="0" fontId="17" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="9" fontId="29" fillId="6" borderId="12" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="13" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Currency" xfId="5" builtinId="4"/>
@@ -3913,7 +3913,7 @@
   <dimension ref="A1:H124"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="27.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.5703125" bestFit="1" customWidth="1"/>
@@ -3921,12 +3921,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.2">
-      <c r="A1" s="108" t="s">
+      <c r="A1" s="111" t="s">
         <v>260</v>
       </c>
-      <c r="B1" s="109"/>
-      <c r="C1" s="109"/>
-      <c r="D1" s="110"/>
+      <c r="B1" s="112"/>
+      <c r="C1" s="112"/>
+      <c r="D1" s="113"/>
     </row>
     <row r="2" spans="1:8" ht="15.75" x14ac:dyDescent="0.2">
       <c r="A2" s="77" t="s">
@@ -4201,7 +4201,7 @@
       </c>
       <c r="D18" s="102" cm="1">
         <f t="array" aca="1" ref="D18" ca="1">IF(OR(IF(OR(A18="", B18="", C18=""), "", INDIRECT("'" &amp; B18 &amp; "'!" &amp; C18))=0, IF(OR(A18="", B18="", C18=""), "", INDIRECT("'" &amp; B18 &amp; "'!" &amp; C18))=""),"",INDIRECT("'" &amp; B18 &amp; "'!" &amp; C18))</f>
-        <v>320301.36986301368</v>
+        <v>355890.41095890413</v>
       </c>
       <c r="E18" s="8"/>
     </row>
@@ -4232,7 +4232,7 @@
       </c>
       <c r="D20" s="102" cm="1">
         <f t="array" aca="1" ref="D20" ca="1">IF(OR(IF(OR(A20="", B20="", C20=""), "", INDIRECT("'" &amp; B20 &amp; "'!" &amp; C20))=0, IF(OR(A20="", B20="", C20=""), "", INDIRECT("'" &amp; B20 &amp; "'!" &amp; C20))=""),"",INDIRECT("'" &amp; B20 &amp; "'!" &amp; C20))</f>
-        <v>982721.66500856355</v>
+        <v>1091912.9611206262</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -4352,7 +4352,7 @@
       </c>
       <c r="D28" s="102" cm="1">
         <f t="array" aca="1" ref="D28" ca="1">IF(OR(IF(OR(A28="", B28="", C28=""), "", INDIRECT("'" &amp; B28 &amp; "'!" &amp; C28))=0, IF(OR(A28="", B28="", C28=""), "", INDIRECT("'" &amp; B28 &amp; "'!" &amp; C28))=""),"",INDIRECT("'" &amp; B28 &amp; "'!" &amp; C28))</f>
-        <v>1303023.0348715773</v>
+        <v>1447803.3720795303</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="15" x14ac:dyDescent="0.2">
@@ -5388,13 +5388,13 @@
       <c r="C98" s="88" t="s">
         <v>442</v>
       </c>
-      <c r="D98" s="126" cm="1">
+      <c r="D98" s="108" cm="1">
         <f t="array" aca="1" ref="D98" ca="1">IF(OR(IF(OR(A98="", B98="", C98=""), "", INDIRECT("'" &amp; B98 &amp; "'!" &amp; C98))=0, IF(OR(A98="", B98="", C98=""), "", INDIRECT("'" &amp; B98 &amp; "'!" &amp; C98))=""),"",INDIRECT("'" &amp; B98 &amp; "'!" &amp; C98))</f>
         <v>0.1</v>
       </c>
     </row>
     <row r="99" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A99" s="127" t="s">
+      <c r="A99" s="109" t="s">
         <v>443</v>
       </c>
       <c r="B99" s="89"/>
@@ -5405,7 +5405,7 @@
       </c>
     </row>
     <row r="100" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A100" s="127" t="s">
+      <c r="A100" s="109" t="s">
         <v>444</v>
       </c>
       <c r="B100" s="88"/>
@@ -5660,15 +5660,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="114" t="s">
+      <c r="A1" s="117" t="s">
         <v>134</v>
       </c>
-      <c r="B1" s="114"/>
-      <c r="C1" s="114"/>
-      <c r="D1" s="114"/>
-      <c r="E1" s="114"/>
-      <c r="F1" s="114"/>
-      <c r="G1" s="114"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
       <c r="AE1" s="3"/>
       <c r="AF1" s="5"/>
       <c r="AG1" s="5"/>
@@ -5755,15 +5755,15 @@
       <c r="AF6" s="7"/>
     </row>
     <row r="7" spans="1:36" x14ac:dyDescent="0.2">
-      <c r="A7" s="121" t="s">
+      <c r="A7" s="124" t="s">
         <v>115</v>
       </c>
-      <c r="B7" s="113"/>
-      <c r="C7" s="113"/>
-      <c r="D7" s="113"/>
-      <c r="E7" s="113"/>
-      <c r="F7" s="113"/>
-      <c r="G7" s="113"/>
+      <c r="B7" s="116"/>
+      <c r="C7" s="116"/>
+      <c r="D7" s="116"/>
+      <c r="E7" s="116"/>
+      <c r="F7" s="116"/>
+      <c r="G7" s="116"/>
       <c r="AE7" s="7"/>
       <c r="AF7" s="7"/>
     </row>
@@ -6040,15 +6040,15 @@
       <c r="AF18" s="7"/>
     </row>
     <row r="19" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="A19" s="122" t="s">
+      <c r="A19" s="125" t="s">
         <v>120</v>
       </c>
-      <c r="B19" s="122"/>
-      <c r="C19" s="122"/>
-      <c r="D19" s="122"/>
-      <c r="E19" s="122"/>
-      <c r="F19" s="122"/>
-      <c r="G19" s="122"/>
+      <c r="B19" s="125"/>
+      <c r="C19" s="125"/>
+      <c r="D19" s="125"/>
+      <c r="E19" s="125"/>
+      <c r="F19" s="125"/>
+      <c r="G19" s="125"/>
       <c r="AE19" s="7"/>
       <c r="AF19" s="7"/>
     </row>
@@ -7771,15 +7771,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" ht="18" x14ac:dyDescent="0.25">
-      <c r="A1" s="124" t="s">
+      <c r="A1" s="127" t="s">
         <v>145</v>
       </c>
-      <c r="B1" s="113"/>
-      <c r="C1" s="113"/>
-      <c r="D1" s="113"/>
-      <c r="E1" s="113"/>
-      <c r="F1" s="113"/>
-      <c r="G1" s="113"/>
+      <c r="B1" s="116"/>
+      <c r="C1" s="116"/>
+      <c r="D1" s="116"/>
+      <c r="E1" s="116"/>
+      <c r="F1" s="116"/>
+      <c r="G1" s="116"/>
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
@@ -7845,15 +7845,15 @@
       </c>
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="A7" s="121" t="s">
+      <c r="A7" s="124" t="s">
         <v>115</v>
       </c>
-      <c r="B7" s="113"/>
-      <c r="C7" s="113"/>
-      <c r="D7" s="113"/>
-      <c r="E7" s="113"/>
-      <c r="F7" s="113"/>
-      <c r="G7" s="113"/>
+      <c r="B7" s="116"/>
+      <c r="C7" s="116"/>
+      <c r="D7" s="116"/>
+      <c r="E7" s="116"/>
+      <c r="F7" s="116"/>
+      <c r="G7" s="116"/>
       <c r="AE7" s="7"/>
       <c r="AF7" s="7"/>
     </row>
@@ -8100,15 +8100,15 @@
       </c>
     </row>
     <row r="19" spans="1:8" s="46" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="125" t="s">
+      <c r="A19" s="128" t="s">
         <v>118</v>
       </c>
-      <c r="B19" s="125"/>
-      <c r="C19" s="125"/>
-      <c r="D19" s="125"/>
-      <c r="E19" s="125"/>
-      <c r="F19" s="125"/>
-      <c r="G19" s="125"/>
+      <c r="B19" s="128"/>
+      <c r="C19" s="128"/>
+      <c r="D19" s="128"/>
+      <c r="E19" s="128"/>
+      <c r="F19" s="128"/>
+      <c r="G19" s="128"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20">
@@ -9680,15 +9680,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" ht="18" x14ac:dyDescent="0.25">
-      <c r="A1" s="124" t="s">
+      <c r="A1" s="127" t="s">
         <v>146</v>
       </c>
-      <c r="B1" s="113"/>
-      <c r="C1" s="113"/>
-      <c r="D1" s="113"/>
-      <c r="E1" s="113"/>
-      <c r="F1" s="113"/>
-      <c r="G1" s="113"/>
+      <c r="B1" s="116"/>
+      <c r="C1" s="116"/>
+      <c r="D1" s="116"/>
+      <c r="E1" s="116"/>
+      <c r="F1" s="116"/>
+      <c r="G1" s="116"/>
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
@@ -9754,15 +9754,15 @@
       </c>
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="A7" s="121" t="s">
+      <c r="A7" s="124" t="s">
         <v>115</v>
       </c>
-      <c r="B7" s="113"/>
-      <c r="C7" s="113"/>
-      <c r="D7" s="113"/>
-      <c r="E7" s="113"/>
-      <c r="F7" s="113"/>
-      <c r="G7" s="113"/>
+      <c r="B7" s="116"/>
+      <c r="C7" s="116"/>
+      <c r="D7" s="116"/>
+      <c r="E7" s="116"/>
+      <c r="F7" s="116"/>
+      <c r="G7" s="116"/>
       <c r="AE7" s="7"/>
       <c r="AF7" s="7"/>
     </row>
@@ -10009,15 +10009,15 @@
       </c>
     </row>
     <row r="19" spans="1:8" s="46" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="125" t="s">
+      <c r="A19" s="128" t="s">
         <v>151</v>
       </c>
-      <c r="B19" s="125"/>
-      <c r="C19" s="125"/>
-      <c r="D19" s="125"/>
-      <c r="E19" s="125"/>
-      <c r="F19" s="125"/>
-      <c r="G19" s="125"/>
+      <c r="B19" s="128"/>
+      <c r="C19" s="128"/>
+      <c r="D19" s="128"/>
+      <c r="E19" s="128"/>
+      <c r="F19" s="128"/>
+      <c r="G19" s="128"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20">
@@ -11589,15 +11589,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" ht="18" x14ac:dyDescent="0.25">
-      <c r="A1" s="124" t="s">
+      <c r="A1" s="127" t="s">
         <v>147</v>
       </c>
-      <c r="B1" s="113"/>
-      <c r="C1" s="113"/>
-      <c r="D1" s="113"/>
-      <c r="E1" s="113"/>
-      <c r="F1" s="113"/>
-      <c r="G1" s="113"/>
+      <c r="B1" s="116"/>
+      <c r="C1" s="116"/>
+      <c r="D1" s="116"/>
+      <c r="E1" s="116"/>
+      <c r="F1" s="116"/>
+      <c r="G1" s="116"/>
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
@@ -11663,15 +11663,15 @@
       </c>
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="A7" s="121" t="s">
+      <c r="A7" s="124" t="s">
         <v>115</v>
       </c>
-      <c r="B7" s="113"/>
-      <c r="C7" s="113"/>
-      <c r="D7" s="113"/>
-      <c r="E7" s="113"/>
-      <c r="F7" s="113"/>
-      <c r="G7" s="113"/>
+      <c r="B7" s="116"/>
+      <c r="C7" s="116"/>
+      <c r="D7" s="116"/>
+      <c r="E7" s="116"/>
+      <c r="F7" s="116"/>
+      <c r="G7" s="116"/>
       <c r="AE7" s="7"/>
       <c r="AF7" s="7"/>
     </row>
@@ -11918,15 +11918,15 @@
       </c>
     </row>
     <row r="19" spans="1:8" s="46" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="125" t="s">
+      <c r="A19" s="128" t="s">
         <v>118</v>
       </c>
-      <c r="B19" s="125"/>
-      <c r="C19" s="125"/>
-      <c r="D19" s="125"/>
-      <c r="E19" s="125"/>
-      <c r="F19" s="125"/>
-      <c r="G19" s="125"/>
+      <c r="B19" s="128"/>
+      <c r="C19" s="128"/>
+      <c r="D19" s="128"/>
+      <c r="E19" s="128"/>
+      <c r="F19" s="128"/>
+      <c r="G19" s="128"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20">
@@ -13499,15 +13499,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" ht="18" x14ac:dyDescent="0.25">
-      <c r="A1" s="124" t="s">
+      <c r="A1" s="127" t="s">
         <v>148</v>
       </c>
-      <c r="B1" s="113"/>
-      <c r="C1" s="113"/>
-      <c r="D1" s="113"/>
-      <c r="E1" s="113"/>
-      <c r="F1" s="113"/>
-      <c r="G1" s="113"/>
+      <c r="B1" s="116"/>
+      <c r="C1" s="116"/>
+      <c r="D1" s="116"/>
+      <c r="E1" s="116"/>
+      <c r="F1" s="116"/>
+      <c r="G1" s="116"/>
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
@@ -13576,15 +13576,15 @@
       </c>
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="A7" s="121" t="s">
+      <c r="A7" s="124" t="s">
         <v>115</v>
       </c>
-      <c r="B7" s="113"/>
-      <c r="C7" s="113"/>
-      <c r="D7" s="113"/>
-      <c r="E7" s="113"/>
-      <c r="F7" s="113"/>
-      <c r="G7" s="113"/>
+      <c r="B7" s="116"/>
+      <c r="C7" s="116"/>
+      <c r="D7" s="116"/>
+      <c r="E7" s="116"/>
+      <c r="F7" s="116"/>
+      <c r="G7" s="116"/>
       <c r="AE7" s="7"/>
       <c r="AF7" s="7"/>
     </row>
@@ -13831,15 +13831,15 @@
       </c>
     </row>
     <row r="19" spans="1:8" s="46" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="125" t="s">
+      <c r="A19" s="128" t="s">
         <v>151</v>
       </c>
-      <c r="B19" s="125"/>
-      <c r="C19" s="125"/>
-      <c r="D19" s="125"/>
-      <c r="E19" s="125"/>
-      <c r="F19" s="125"/>
-      <c r="G19" s="125"/>
+      <c r="B19" s="128"/>
+      <c r="C19" s="128"/>
+      <c r="D19" s="128"/>
+      <c r="E19" s="128"/>
+      <c r="F19" s="128"/>
+      <c r="G19" s="128"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20">
@@ -37812,12 +37812,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="18" x14ac:dyDescent="0.25">
-      <c r="A1" s="114" t="s">
+      <c r="A1" s="117" t="s">
         <v>79</v>
       </c>
-      <c r="B1" s="114"/>
-      <c r="C1" s="114"/>
-      <c r="D1" s="114"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
       <c r="K1" s="9"/>
       <c r="L1" s="9"/>
     </row>
@@ -37911,12 +37911,12 @@
       <c r="Q11" s="9"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="115" t="s">
+      <c r="A12" s="118" t="s">
         <v>87</v>
       </c>
-      <c r="B12" s="115"/>
-      <c r="C12" s="115"/>
-      <c r="D12" s="115"/>
+      <c r="B12" s="118"/>
+      <c r="C12" s="118"/>
+      <c r="D12" s="118"/>
       <c r="Q12" s="9"/>
     </row>
     <row r="13" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
@@ -38048,12 +38048,12 @@
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A26" s="116" t="s">
+      <c r="A26" s="119" t="s">
         <v>96</v>
       </c>
-      <c r="B26" s="113"/>
-      <c r="C26" s="113"/>
-      <c r="D26" s="113"/>
+      <c r="B26" s="116"/>
+      <c r="C26" s="116"/>
+      <c r="D26" s="116"/>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
@@ -38087,10 +38087,10 @@
       <c r="F30" s="7"/>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A31" s="111"/>
-      <c r="B31" s="112"/>
-      <c r="C31" s="113"/>
-      <c r="D31" s="113"/>
+      <c r="A31" s="114"/>
+      <c r="B31" s="115"/>
+      <c r="C31" s="116"/>
+      <c r="D31" s="116"/>
       <c r="F31" s="7"/>
     </row>
     <row r="32" spans="1:15" ht="13.35" customHeight="1" x14ac:dyDescent="0.2">
@@ -38115,7 +38115,7 @@
       </c>
       <c r="B35" s="7">
         <f>'Base 1 PV Loss WLE'!G17</f>
-        <v>320301.36986301368</v>
+        <v>355890.41095890413</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.2">
@@ -38124,7 +38124,7 @@
       </c>
       <c r="B36" s="7">
         <f>'Base 1 PV Loss WLE'!G71</f>
-        <v>982721.66500856355</v>
+        <v>1091912.9611206262</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.2">
@@ -38133,7 +38133,7 @@
       </c>
       <c r="B37" s="7">
         <f>'Base 1 PV Loss WLE'!G73</f>
-        <v>1303023.0348715773</v>
+        <v>1447803.3720795303</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.2">
@@ -38703,7 +38703,7 @@
       <c r="B19" t="s">
         <v>170</v>
       </c>
-      <c r="L19" s="128" t="s">
+      <c r="L19" s="110" t="s">
         <v>445</v>
       </c>
     </row>
@@ -38722,17 +38722,17 @@
       </c>
     </row>
     <row r="21" spans="1:12" ht="19.7" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="117" t="s">
+      <c r="A21" s="120" t="s">
         <v>172</v>
       </c>
-      <c r="B21" s="113"/>
-      <c r="C21" s="113"/>
-      <c r="D21" s="117" t="s">
+      <c r="B21" s="116"/>
+      <c r="C21" s="116"/>
+      <c r="D21" s="120" t="s">
         <v>247</v>
       </c>
-      <c r="E21" s="113"/>
-      <c r="F21" s="113"/>
-      <c r="L21" s="128" t="s">
+      <c r="E21" s="116"/>
+      <c r="F21" s="116"/>
+      <c r="L21" s="110" t="s">
         <v>446</v>
       </c>
     </row>
@@ -38776,7 +38776,7 @@
         <f t="array" ref="F23">MAX(IF(ISNUMBER('Base 1 PV Loss To Age'!D20:D49),'Base 1 PV Loss To Age'!D20:D49))</f>
         <v>3.9269999999999999E-2</v>
       </c>
-      <c r="L23" s="128" t="s">
+      <c r="L23" s="110" t="s">
         <v>447</v>
       </c>
     </row>
@@ -38803,7 +38803,7 @@
       <c r="C25" s="53" t="b">
         <v>1</v>
       </c>
-      <c r="L25" s="128" t="s">
+      <c r="L25" s="110" t="s">
         <v>448</v>
       </c>
     </row>
@@ -38891,11 +38891,11 @@
       </c>
     </row>
     <row r="34" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A34" s="117" t="s">
+      <c r="A34" s="120" t="s">
         <v>176</v>
       </c>
-      <c r="B34" s="117"/>
-      <c r="C34" s="117"/>
+      <c r="B34" s="120"/>
+      <c r="C34" s="120"/>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" t="str">
@@ -39014,11 +39014,11 @@
       </c>
     </row>
     <row r="46" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A46" s="117" t="s">
+      <c r="A46" s="120" t="s">
         <v>177</v>
       </c>
-      <c r="B46" s="117"/>
-      <c r="C46" s="117"/>
+      <c r="B46" s="120"/>
+      <c r="C46" s="120"/>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A47" t="str">
@@ -39137,11 +39137,11 @@
       </c>
     </row>
     <row r="58" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A58" s="118" t="s">
+      <c r="A58" s="121" t="s">
         <v>205</v>
       </c>
-      <c r="B58" s="118"/>
-      <c r="C58" s="118"/>
+      <c r="B58" s="121"/>
+      <c r="C58" s="121"/>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A59" t="str">
@@ -39260,11 +39260,11 @@
       </c>
     </row>
     <row r="70" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A70" s="118" t="s">
+      <c r="A70" s="121" t="s">
         <v>206</v>
       </c>
-      <c r="B70" s="118"/>
-      <c r="C70" s="118"/>
+      <c r="B70" s="121"/>
+      <c r="C70" s="121"/>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A71" t="str">
@@ -39424,10 +39424,10 @@
       </c>
     </row>
     <row r="86" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A86" s="117" t="s">
+      <c r="A86" s="120" t="s">
         <v>182</v>
       </c>
-      <c r="B86" s="117"/>
+      <c r="B86" s="120"/>
       <c r="F86" t="s">
         <v>195</v>
       </c>
@@ -39739,12 +39739,12 @@
       </c>
     </row>
     <row r="3" spans="1:9" ht="99.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="120" t="str">
+      <c r="B3" s="123" t="str">
         <f>"Here are the estimates you have requested with respect to the diminution of earning capacity and associated economic impairment sustained by your client. The following records were considered in connection with the opinion below: "&amp;Inputs!B20&amp;"."</f>
         <v>Here are the estimates you have requested with respect to the diminution of earning capacity and associated economic impairment sustained by your client. The following records were considered in connection with the opinion below: Tax Returns 2020-2024, W-2s from ABC, Co. Inc; Schedule C's and the Claimant Information Sheet..</v>
       </c>
-      <c r="C3" s="120"/>
-      <c r="D3" s="120"/>
+      <c r="C3" s="123"/>
+      <c r="D3" s="123"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="61" t="s">
@@ -40073,12 +40073,12 @@
       <c r="G21" s="60"/>
     </row>
     <row r="22" spans="1:7" ht="65.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="119" t="str">
+      <c r="B22" s="122" t="str">
         <f>"1.     Earnings and Employment Background indicates that your client was working as a "&amp;Inputs!$D$20&amp;" at the time of the accident."</f>
         <v>1.     Earnings and Employment Background indicates that your client was working as a Plumber for ABC, Inc at the time of the accident.</v>
       </c>
-      <c r="C22" s="119"/>
-      <c r="D22" s="119"/>
+      <c r="C22" s="122"/>
+      <c r="D22" s="122"/>
       <c r="E22" s="70" t="b">
         <v>0</v>
       </c>
@@ -40100,12 +40100,12 @@
       <c r="A24" s="8" t="s">
         <v>250</v>
       </c>
-      <c r="B24" s="119" t="str">
+      <c r="B24" s="122" t="str">
         <f>_xlfn._LONGTEXT("Discount Rates form the basis upon which post-trial earning capacity streams are commuted to present value. The discounting ensures that the lump sum award will dissipate entirely by the end of the calculating period and will be used to replicate the stre","am of anticipated earning capacity, without windfall to your client. This analysis employs a laddered discount rate approach with rates derived from current rates of interest on AAA-rated municipal bonds ranging from ")&amp;TEXT(Inputs!$E$22,"0.0%")&amp;" to "&amp;TEXT(Inputs!$F$22,"0.0%")&amp;"."</f>
         <v>Discount Rates form the basis upon which post-trial earning capacity streams are commuted to present value. The discounting ensures that the lump sum award will dissipate entirely by the end of the calculating period and will be used to replicate the stream of anticipated earning capacity, without windfall to your client. This analysis employs a laddered discount rate approach with rates derived from current rates of interest on AAA-rated municipal bonds ranging from 2.3% to 3.3%.</v>
       </c>
-      <c r="C24" s="119"/>
-      <c r="D24" s="119"/>
+      <c r="C24" s="122"/>
+      <c r="D24" s="122"/>
       <c r="E24" s="70" t="b">
         <v>0</v>
       </c>
@@ -40114,12 +40114,12 @@
       <c r="A25" s="8" t="s">
         <v>251</v>
       </c>
-      <c r="B25" s="119" t="str">
+      <c r="B25" s="122" t="str">
         <f>CONCATENATE(_xlfn._LONGTEXT("Below Market Discount Rates form the basis upon which post-trial earning capacity streams are commuted to present value. The discounting ensures that the lump sum award will dissipate entirely by the end of the calculating period and will be used to repli","cate the stream of anticipated earning capacity, without windfall to your client. This analysis employs a laddered discount rate approach with rates derived from of current real rates of interest on AAA-rated municipal bonds adjusted for the forecased int","ermediate long run inflation estimate as reported in the Annual Report of the Board of Trustees of the Social Security Administration (2025). These rates currently range from "),TEXT(Inputs!$E$22,"0.0%")," to ",TEXT(Inputs!$F$22,"0.0%"),".")</f>
         <v>Below Market Discount Rates form the basis upon which post-trial earning capacity streams are commuted to present value. The discounting ensures that the lump sum award will dissipate entirely by the end of the calculating period and will be used to replicate the stream of anticipated earning capacity, without windfall to your client. This analysis employs a laddered discount rate approach with rates derived from of current real rates of interest on AAA-rated municipal bonds adjusted for the forecased intermediate long run inflation estimate as reported in the Annual Report of the Board of Trustees of the Social Security Administration (2025). These rates currently range from 2.3% to 3.3%.</v>
       </c>
-      <c r="C25" s="119"/>
-      <c r="D25" s="119"/>
+      <c r="C25" s="122"/>
+      <c r="D25" s="122"/>
       <c r="E25" s="70" t="b">
         <v>0</v>
       </c>
@@ -40128,12 +40128,12 @@
       <c r="A26" s="8" t="s">
         <v>253</v>
       </c>
-      <c r="B26" s="119" t="str">
+      <c r="B26" s="122" t="str">
         <f>_xlfn._LONGTEXT("Discount Rates form the basis upon which post-trial earning capacity streams are commuted to present value. The discounting ensures that the lump sum award will dissipate entirely by the end of the calculating period and will be used to replicate the stre","am of anticipated earning capacity, without windfall to your client. This analysis employs a laddered discount rate approach with rates derived from current rates of interest on AAA-rated municipal bonds ranging from ")&amp;TEXT(Inputs!$E$23,"0.0%")&amp;" to "&amp;TEXT(Inputs!$F$23,"0.0%")&amp;"."</f>
         <v>Discount Rates form the basis upon which post-trial earning capacity streams are commuted to present value. The discounting ensures that the lump sum award will dissipate entirely by the end of the calculating period and will be used to replicate the stream of anticipated earning capacity, without windfall to your client. This analysis employs a laddered discount rate approach with rates derived from current rates of interest on AAA-rated municipal bonds ranging from 2.3% to 3.9%.</v>
       </c>
-      <c r="C26" s="119"/>
-      <c r="D26" s="119"/>
+      <c r="C26" s="122"/>
+      <c r="D26" s="122"/>
       <c r="E26" s="70" t="b">
         <v>0</v>
       </c>
@@ -40267,21 +40267,21 @@
     <col min="5" max="5" width="21.42578125" customWidth="1"/>
     <col min="6" max="6" width="19.42578125" customWidth="1"/>
     <col min="7" max="7" width="23.140625" customWidth="1"/>
-    <col min="8" max="8" width="14.140625" customWidth="1"/>
+    <col min="8" max="8" width="15.85546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12.42578125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:36" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="114" t="s">
+      <c r="A1" s="117" t="s">
         <v>143</v>
       </c>
-      <c r="B1" s="114"/>
-      <c r="C1" s="114"/>
-      <c r="D1" s="114"/>
-      <c r="E1" s="114"/>
-      <c r="F1" s="114"/>
-      <c r="G1" s="114"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
       <c r="AE1" s="3"/>
       <c r="AF1" s="5"/>
       <c r="AG1" s="5"/>
@@ -40354,7 +40354,7 @@
         <v>0.1</v>
       </c>
       <c r="F5" s="53" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AE5" s="7"/>
       <c r="AF5" s="7"/>
@@ -40374,15 +40374,15 @@
       <c r="AF6" s="7"/>
     </row>
     <row r="7" spans="1:36" x14ac:dyDescent="0.2">
-      <c r="A7" s="121" t="s">
+      <c r="A7" s="124" t="s">
         <v>115</v>
       </c>
-      <c r="B7" s="113"/>
-      <c r="C7" s="113"/>
-      <c r="D7" s="113"/>
-      <c r="E7" s="113"/>
-      <c r="F7" s="113"/>
-      <c r="G7" s="113"/>
+      <c r="B7" s="116"/>
+      <c r="C7" s="116"/>
+      <c r="D7" s="116"/>
+      <c r="E7" s="116"/>
+      <c r="F7" s="116"/>
+      <c r="G7" s="116"/>
       <c r="AE7" s="7"/>
       <c r="AF7" s="7"/>
     </row>
@@ -40442,7 +40442,7 @@
       </c>
       <c r="G9" s="7">
         <f>C9*F9*IF($F$5,1-$E$5,1)</f>
-        <v>22376.712328767127</v>
+        <v>24863.01369863014</v>
       </c>
       <c r="H9" s="7">
         <f>C9*F9</f>
@@ -40480,7 +40480,7 @@
       </c>
       <c r="G10" s="7">
         <f>C10*F10*IF($F$5,1-$E$5,1)</f>
-        <v>67500</v>
+        <v>75000</v>
       </c>
       <c r="H10" s="7">
         <f t="shared" ref="H10:H15" si="0">C10*F10</f>
@@ -40518,7 +40518,7 @@
       </c>
       <c r="G11" s="7">
         <f>C11*F11*IF($F$5,1-$E$5,1)</f>
-        <v>67500</v>
+        <v>75000</v>
       </c>
       <c r="H11" s="7">
         <f t="shared" si="0"/>
@@ -40554,7 +40554,7 @@
       </c>
       <c r="G12" s="7">
         <f>IF(A12="","",C12*F12*IF($F$5,1-$E$5,1))</f>
-        <v>67500</v>
+        <v>75000</v>
       </c>
       <c r="H12" s="7">
         <f t="shared" si="0"/>
@@ -40590,7 +40590,7 @@
       </c>
       <c r="G13" s="7">
         <f>IF(A13="","",C13*F13*IF($F$5,1-$E$5,1))</f>
-        <v>67500</v>
+        <v>75000</v>
       </c>
       <c r="H13" s="7">
         <f t="shared" si="0"/>
@@ -40630,7 +40630,7 @@
       </c>
       <c r="G15" s="7">
         <f>C15*F15*IF($F$5,1-$E$5,1)</f>
-        <v>27924.657534246577</v>
+        <v>31027.397260273974</v>
       </c>
       <c r="H15" s="7">
         <f t="shared" si="0"/>
@@ -40652,7 +40652,7 @@
       <c r="D17" s="38"/>
       <c r="G17" s="30">
         <f>SUM(G9:G15)</f>
-        <v>320301.36986301368</v>
+        <v>355890.41095890413</v>
       </c>
       <c r="H17" s="30">
         <f>SUM(H9:H15)</f>
@@ -40666,15 +40666,15 @@
       <c r="AF18" s="7"/>
     </row>
     <row r="19" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="A19" s="122" t="s">
+      <c r="A19" s="125" t="s">
         <v>118</v>
       </c>
-      <c r="B19" s="122"/>
-      <c r="C19" s="122"/>
-      <c r="D19" s="122"/>
-      <c r="E19" s="122"/>
-      <c r="F19" s="122"/>
-      <c r="G19" s="122"/>
+      <c r="B19" s="125"/>
+      <c r="C19" s="125"/>
+      <c r="D19" s="125"/>
+      <c r="E19" s="125"/>
+      <c r="F19" s="125"/>
+      <c r="G19" s="125"/>
       <c r="AE19" s="7"/>
       <c r="AF19" s="7"/>
     </row>
@@ -40705,7 +40705,7 @@
       </c>
       <c r="G20" s="7">
         <f t="shared" ref="G20:G51" si="4">IF(A20="","",E20*F20*IF($F$5,1-$E$5,1))</f>
-        <v>68027.194260075659</v>
+        <v>75585.771400084064</v>
       </c>
       <c r="AE20" s="7"/>
       <c r="AF20" s="7"/>
@@ -40737,7 +40737,7 @@
       </c>
       <c r="G21" s="7">
         <f t="shared" si="4"/>
-        <v>68571.911314752855</v>
+        <v>76191.01257194762</v>
       </c>
       <c r="AE21" s="7"/>
       <c r="AF21" s="7"/>
@@ -40769,7 +40769,7 @@
       </c>
       <c r="G22" s="7">
         <f t="shared" si="4"/>
-        <v>69118.287612481217</v>
+        <v>76798.097347201343</v>
       </c>
       <c r="AE22" s="7"/>
       <c r="AF22" s="7"/>
@@ -40801,7 +40801,7 @@
       </c>
       <c r="G23" s="7">
         <f t="shared" si="4"/>
-        <v>69511.224486057166</v>
+        <v>77234.693873396856</v>
       </c>
       <c r="AE23" s="7"/>
       <c r="AF23" s="7"/>
@@ -40833,7 +40833,7 @@
       </c>
       <c r="G24" s="7">
         <f t="shared" si="4"/>
-        <v>69849.119251805125</v>
+        <v>77610.132502005697</v>
       </c>
       <c r="AE24" s="7"/>
       <c r="AF24" s="7"/>
@@ -40865,7 +40865,7 @@
       </c>
       <c r="G25" s="7">
         <f t="shared" si="4"/>
-        <v>69983.496555602323</v>
+        <v>77759.440617335917</v>
       </c>
       <c r="AE25" s="7"/>
       <c r="AF25" s="7"/>
@@ -40897,7 +40897,7 @@
       </c>
       <c r="G26" s="7">
         <f t="shared" si="4"/>
-        <v>69927.166529118738</v>
+        <v>77696.851699020815</v>
       </c>
       <c r="AE26" s="7"/>
       <c r="AF26" s="7"/>
@@ -40929,7 +40929,7 @@
       </c>
       <c r="G27" s="7">
         <f t="shared" si="4"/>
-        <v>69925.705144517793</v>
+        <v>77695.227938353099</v>
       </c>
       <c r="AE27" s="7"/>
       <c r="AF27" s="7"/>
@@ -40961,7 +40961,7 @@
       </c>
       <c r="G28" s="7">
         <f t="shared" si="4"/>
-        <v>69670.960332929884</v>
+        <v>77412.178147699873</v>
       </c>
       <c r="AE28" s="7"/>
       <c r="AF28" s="7"/>
@@ -40993,7 +40993,7 @@
       </c>
       <c r="G29" s="7">
         <f t="shared" si="4"/>
-        <v>69212.619531159042</v>
+        <v>76902.910590176718</v>
       </c>
       <c r="I29" s="7"/>
       <c r="AE29" s="7"/>
@@ -41026,7 +41026,7 @@
       </c>
       <c r="G30" s="7">
         <f t="shared" si="4"/>
-        <v>68553.118956179635</v>
+        <v>76170.132173532926</v>
       </c>
       <c r="AE30" s="7"/>
       <c r="AF30" s="7"/>
@@ -41058,7 +41058,7 @@
       </c>
       <c r="G31" s="7">
         <f t="shared" si="4"/>
-        <v>67791.367874503208</v>
+        <v>75323.742082781348</v>
       </c>
       <c r="AE31" s="7"/>
       <c r="AF31" s="7"/>
@@ -41090,7 +41090,7 @@
       </c>
       <c r="G32" s="7">
         <f t="shared" si="4"/>
-        <v>67185.876976210027</v>
+        <v>74650.974418011145</v>
       </c>
       <c r="AE32" s="7"/>
       <c r="AF32" s="7"/>
@@ -41122,7 +41122,7 @@
       </c>
       <c r="G33" s="7">
         <f t="shared" si="4"/>
-        <v>66202.816750685306</v>
+        <v>73558.685278539226</v>
       </c>
       <c r="AE33" s="7"/>
       <c r="AF33" s="7"/>
@@ -41154,7 +41154,7 @@
       </c>
       <c r="G34" s="7">
         <f t="shared" si="4"/>
-        <v>19190.799432485612</v>
+        <v>21323.11048053957</v>
       </c>
       <c r="AE34" s="7"/>
       <c r="AF34" s="7"/>
@@ -42302,7 +42302,7 @@
       <c r="F71" s="29"/>
       <c r="G71" s="29">
         <f>SUM(G20:G70)</f>
-        <v>982721.66500856355</v>
+        <v>1091912.9611206262</v>
       </c>
       <c r="AE71" s="2"/>
       <c r="AF71" s="2"/>
@@ -42325,7 +42325,7 @@
       <c r="F73" s="37"/>
       <c r="G73" s="29">
         <f>G17+G71</f>
-        <v>1303023.0348715773</v>
+        <v>1447803.3720795303</v>
       </c>
       <c r="AE73" s="2"/>
       <c r="AF73" s="2"/>
@@ -42400,15 +42400,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="114" t="s">
+      <c r="A1" s="117" t="s">
         <v>144</v>
       </c>
-      <c r="B1" s="114"/>
-      <c r="C1" s="114"/>
-      <c r="D1" s="114"/>
-      <c r="E1" s="114"/>
-      <c r="F1" s="114"/>
-      <c r="G1" s="114"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
       <c r="AE1" s="3"/>
       <c r="AF1" s="5"/>
       <c r="AG1" s="5"/>
@@ -42498,15 +42498,15 @@
       <c r="AF6" s="7"/>
     </row>
     <row r="7" spans="1:36" x14ac:dyDescent="0.2">
-      <c r="A7" s="121" t="s">
+      <c r="A7" s="124" t="s">
         <v>115</v>
       </c>
-      <c r="B7" s="113"/>
-      <c r="C7" s="113"/>
-      <c r="D7" s="113"/>
-      <c r="E7" s="113"/>
-      <c r="F7" s="113"/>
-      <c r="G7" s="113"/>
+      <c r="B7" s="116"/>
+      <c r="C7" s="116"/>
+      <c r="D7" s="116"/>
+      <c r="E7" s="116"/>
+      <c r="F7" s="116"/>
+      <c r="G7" s="116"/>
       <c r="AE7" s="7"/>
       <c r="AF7" s="7"/>
     </row>
@@ -42783,15 +42783,15 @@
       <c r="AF18" s="7"/>
     </row>
     <row r="19" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="A19" s="122" t="s">
+      <c r="A19" s="125" t="s">
         <v>120</v>
       </c>
-      <c r="B19" s="122"/>
-      <c r="C19" s="122"/>
-      <c r="D19" s="122"/>
-      <c r="E19" s="122"/>
-      <c r="F19" s="122"/>
-      <c r="G19" s="122"/>
+      <c r="B19" s="125"/>
+      <c r="C19" s="125"/>
+      <c r="D19" s="125"/>
+      <c r="E19" s="125"/>
+      <c r="F19" s="125"/>
+      <c r="G19" s="125"/>
       <c r="AE19" s="7"/>
       <c r="AF19" s="7"/>
     </row>
@@ -44514,15 +44514,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="114" t="s">
+      <c r="A1" s="117" t="s">
         <v>131</v>
       </c>
-      <c r="B1" s="114"/>
-      <c r="C1" s="114"/>
-      <c r="D1" s="114"/>
-      <c r="E1" s="114"/>
-      <c r="F1" s="114"/>
-      <c r="G1" s="114"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
       <c r="AE1" s="3"/>
       <c r="AF1" s="5"/>
       <c r="AG1" s="5"/>
@@ -44609,15 +44609,15 @@
       <c r="AF6" s="7"/>
     </row>
     <row r="7" spans="1:36" x14ac:dyDescent="0.2">
-      <c r="A7" s="121" t="s">
+      <c r="A7" s="124" t="s">
         <v>115</v>
       </c>
-      <c r="B7" s="113"/>
-      <c r="C7" s="113"/>
-      <c r="D7" s="113"/>
-      <c r="E7" s="113"/>
-      <c r="F7" s="113"/>
-      <c r="G7" s="113"/>
+      <c r="B7" s="116"/>
+      <c r="C7" s="116"/>
+      <c r="D7" s="116"/>
+      <c r="E7" s="116"/>
+      <c r="F7" s="116"/>
+      <c r="G7" s="116"/>
       <c r="AE7" s="7"/>
       <c r="AF7" s="7"/>
     </row>
@@ -44894,15 +44894,15 @@
       <c r="AF18" s="7"/>
     </row>
     <row r="19" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="A19" s="122" t="s">
+      <c r="A19" s="125" t="s">
         <v>118</v>
       </c>
-      <c r="B19" s="122"/>
-      <c r="C19" s="122"/>
-      <c r="D19" s="122"/>
-      <c r="E19" s="122"/>
-      <c r="F19" s="122"/>
-      <c r="G19" s="122"/>
+      <c r="B19" s="125"/>
+      <c r="C19" s="125"/>
+      <c r="D19" s="125"/>
+      <c r="E19" s="125"/>
+      <c r="F19" s="125"/>
+      <c r="G19" s="125"/>
       <c r="AE19" s="7"/>
       <c r="AF19" s="7"/>
     </row>
@@ -46625,15 +46625,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="114" t="s">
+      <c r="A1" s="117" t="s">
         <v>132</v>
       </c>
-      <c r="B1" s="114"/>
-      <c r="C1" s="114"/>
-      <c r="D1" s="114"/>
-      <c r="E1" s="114"/>
-      <c r="F1" s="114"/>
-      <c r="G1" s="114"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
       <c r="AE1" s="3"/>
       <c r="AF1" s="5"/>
       <c r="AG1" s="5"/>
@@ -46723,15 +46723,15 @@
       <c r="AF6" s="7"/>
     </row>
     <row r="7" spans="1:36" x14ac:dyDescent="0.2">
-      <c r="A7" s="121" t="s">
+      <c r="A7" s="124" t="s">
         <v>115</v>
       </c>
-      <c r="B7" s="113"/>
-      <c r="C7" s="113"/>
-      <c r="D7" s="113"/>
-      <c r="E7" s="113"/>
-      <c r="F7" s="113"/>
-      <c r="G7" s="113"/>
+      <c r="B7" s="116"/>
+      <c r="C7" s="116"/>
+      <c r="D7" s="116"/>
+      <c r="E7" s="116"/>
+      <c r="F7" s="116"/>
+      <c r="G7" s="116"/>
       <c r="AE7" s="7"/>
       <c r="AF7" s="7"/>
     </row>
@@ -47008,15 +47008,15 @@
       <c r="AF18" s="7"/>
     </row>
     <row r="19" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="A19" s="123" t="s">
+      <c r="A19" s="126" t="s">
         <v>152</v>
       </c>
-      <c r="B19" s="122"/>
-      <c r="C19" s="122"/>
-      <c r="D19" s="122"/>
-      <c r="E19" s="122"/>
-      <c r="F19" s="122"/>
-      <c r="G19" s="122"/>
+      <c r="B19" s="125"/>
+      <c r="C19" s="125"/>
+      <c r="D19" s="125"/>
+      <c r="E19" s="125"/>
+      <c r="F19" s="125"/>
+      <c r="G19" s="125"/>
       <c r="AE19" s="7"/>
       <c r="AF19" s="7"/>
     </row>
@@ -48739,15 +48739,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="114" t="s">
+      <c r="A1" s="117" t="s">
         <v>133</v>
       </c>
-      <c r="B1" s="114"/>
-      <c r="C1" s="114"/>
-      <c r="D1" s="114"/>
-      <c r="E1" s="114"/>
-      <c r="F1" s="114"/>
-      <c r="G1" s="114"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
       <c r="AE1" s="3"/>
       <c r="AF1" s="5"/>
       <c r="AG1" s="5"/>
@@ -48834,15 +48834,15 @@
       <c r="AF6" s="7"/>
     </row>
     <row r="7" spans="1:36" x14ac:dyDescent="0.2">
-      <c r="A7" s="121" t="s">
+      <c r="A7" s="124" t="s">
         <v>115</v>
       </c>
-      <c r="B7" s="113"/>
-      <c r="C7" s="113"/>
-      <c r="D7" s="113"/>
-      <c r="E7" s="113"/>
-      <c r="F7" s="113"/>
-      <c r="G7" s="113"/>
+      <c r="B7" s="116"/>
+      <c r="C7" s="116"/>
+      <c r="D7" s="116"/>
+      <c r="E7" s="116"/>
+      <c r="F7" s="116"/>
+      <c r="G7" s="116"/>
       <c r="AE7" s="7"/>
       <c r="AF7" s="7"/>
     </row>
@@ -49119,15 +49119,15 @@
       <c r="AF18" s="7"/>
     </row>
     <row r="19" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="A19" s="122" t="s">
+      <c r="A19" s="125" t="s">
         <v>118</v>
       </c>
-      <c r="B19" s="122"/>
-      <c r="C19" s="122"/>
-      <c r="D19" s="122"/>
-      <c r="E19" s="122"/>
-      <c r="F19" s="122"/>
-      <c r="G19" s="122"/>
+      <c r="B19" s="125"/>
+      <c r="C19" s="125"/>
+      <c r="D19" s="125"/>
+      <c r="E19" s="125"/>
+      <c r="F19" s="125"/>
+      <c r="G19" s="125"/>
       <c r="AE19" s="7"/>
       <c r="AF19" s="7"/>
     </row>

</xml_diff>

<commit_message>
Fully updated WC worksheet outputs
</commit_message>
<xml_diff>
--- a/EconAutomation/src/supporting_docs/sorted_econ_files/PV2 (color coded).xlsx
+++ b/EconAutomation/src/supporting_docs/sorted_econ_files/PV2 (color coded).xlsx
@@ -9,9 +9,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EricBussey\GitHub\EconAutomation-REP\EconAutomation\src\supporting_docs\sorted_econ_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FA4E890-3D2A-46A8-B39D-0AC2C2146075}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9207CE03-ADEB-4F23-BB6F-D3A754AD343F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="795" xr2:uid="{25EC3B8A-402B-47FF-80A9-5B0690A475CD}"/>
+    <workbookView xWindow="28680" yWindow="-60" windowWidth="29040" windowHeight="15720" tabRatio="795" xr2:uid="{25EC3B8A-402B-47FF-80A9-5B0690A475CD}"/>
   </bookViews>
   <sheets>
     <sheet name="REPORT_OUTPUTS" sheetId="33" r:id="rId1"/>
@@ -112,7 +112,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3643" uniqueCount="449">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3651" uniqueCount="453">
   <si>
     <t>Year</t>
   </si>
@@ -946,21 +946,6 @@
     <t>IDEALLY WILL SYNCHRONIZE WITH WORKING CALC</t>
   </si>
   <si>
-    <t>loss to trial</t>
-  </si>
-  <si>
-    <t>either pre-tax or post-tax/post-credit(actual earnings)</t>
-  </si>
-  <si>
-    <t>loss post trial</t>
-  </si>
-  <si>
-    <t>either pre-tax or post-tax/post-credit(pulled from alternate jobs earnings)</t>
-  </si>
-  <si>
-    <t>pre_injury_earning_capacity</t>
-  </si>
-  <si>
     <t>clm_age_at_DOI</t>
   </si>
   <si>
@@ -1414,9 +1399,6 @@
     <t>est_rate_of_infl</t>
   </si>
   <si>
-    <t>&lt;-- pulling from Voc report</t>
-  </si>
-  <si>
     <t>Base 1 PV Loss To Age</t>
   </si>
   <si>
@@ -1513,6 +1495,36 @@
       <t>age at trial</t>
     </r>
   </si>
+  <si>
+    <t>Table Name</t>
+  </si>
+  <si>
+    <t>Chart Name</t>
+  </si>
+  <si>
+    <t>PV_Summary_No_Rounding</t>
+  </si>
+  <si>
+    <t>GetBloombergDailyYieldCurve_cur</t>
+  </si>
+  <si>
+    <t>WC_Disc_Rate_Chart</t>
+  </si>
+  <si>
+    <t>&lt;round to 1 decimal</t>
+  </si>
+  <si>
+    <t>DR for bases are WLE years (rounded up) from Bloomberg</t>
+  </si>
+  <si>
+    <t>fraction of year multiplied by highest rate to get actual</t>
+  </si>
+  <si>
+    <t>growth rate + disc rates</t>
+  </si>
+  <si>
+    <t>will be negative for some values!!!</t>
+  </si>
 </sst>
 </file>
 
@@ -1527,7 +1539,7 @@
     <numFmt numFmtId="168" formatCode="0.0000"/>
     <numFmt numFmtId="169" formatCode="0.000"/>
   </numFmts>
-  <fonts count="37" x14ac:knownFonts="1">
+  <fonts count="38" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -1763,8 +1775,16 @@
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="12"/>
+      <color theme="1" tint="4.9989318521683403E-2"/>
+      <name val="Aptos Display"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="28">
+  <fills count="30">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1923,8 +1943,20 @@
         <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF8B20"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="18">
+  <borders count="38">
     <border>
       <left/>
       <right/>
@@ -2151,6 +2183,292 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </right>
+      <top style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color theme="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color theme="1"/>
+      </right>
+      <top style="medium">
+        <color theme="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="medium">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </left>
+      <right style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </left>
+      <right style="medium">
+        <color theme="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </left>
+      <right style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </left>
+      <right style="medium">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </top>
+      <bottom style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </left>
+      <right style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </top>
+      <bottom style="medium">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </top>
+      <bottom style="medium">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </left>
+      <right style="medium">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.14999847407452621"/>
+      </top>
+      <bottom style="medium">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -2160,7 +2478,7 @@
     <xf numFmtId="9" fontId="18" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="30" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="129">
+  <cellXfs count="150">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2429,6 +2747,61 @@
     <xf numFmtId="0" fontId="17" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="26" fillId="28" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="28" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="29" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="29" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="24" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="24" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="24" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="24" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Currency" xfId="5" builtinId="4"/>
@@ -2438,7 +2811,276 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="4" builtinId="5"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="14">
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="0" tint="-0.14999847407452621"/>
+        </left>
+        <right style="thin">
+          <color theme="0" tint="-0.14999847407452621"/>
+        </right>
+        <top style="thin">
+          <color theme="0" tint="-0.14999847407452621"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0" tint="-0.14999847407452621"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="0" tint="-0.14999847407452621"/>
+        </left>
+        <right style="thin">
+          <color theme="0" tint="-0.14999847407452621"/>
+        </right>
+        <top style="thin">
+          <color theme="0" tint="-0.14999847407452621"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0" tint="-0.14999847407452621"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color theme="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1" tint="4.9989318521683403E-2"/>
+        <name val="Aptos Display"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="1"/>
+        </left>
+        <right style="thin">
+          <color theme="1"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color theme="1"/>
+        </vertical>
+        <horizontal style="thin">
+          <color theme="1"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="0" tint="-0.14999847407452621"/>
+        </left>
+        <right style="thin">
+          <color theme="0" tint="-0.14999847407452621"/>
+        </right>
+        <top style="thin">
+          <color theme="0" tint="-0.14999847407452621"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0" tint="-0.14999847407452621"/>
+        </bottom>
+        <vertical style="thin">
+          <color theme="0" tint="-0.14999847407452621"/>
+        </vertical>
+        <horizontal style="thin">
+          <color theme="0" tint="-0.14999847407452621"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="0" tint="-0.14999847407452621"/>
+        </left>
+        <right style="thin">
+          <color theme="0" tint="-0.14999847407452621"/>
+        </right>
+        <top style="thin">
+          <color theme="0" tint="-0.14999847407452621"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0" tint="-0.14999847407452621"/>
+        </bottom>
+        <vertical style="thin">
+          <color theme="0" tint="-0.14999847407452621"/>
+        </vertical>
+        <horizontal style="thin">
+          <color theme="0" tint="-0.14999847407452621"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color theme="1" tint="4.9989318521683403E-2"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1" tint="4.9989318521683403E-2"/>
+        <name val="Aptos Display"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color auto="1"/>
+        </vertical>
+        <horizontal/>
+      </border>
+    </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
@@ -3563,12 +4205,34 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D25BA94F-F2EA-4AAE-942B-F73F6553BE39}" name="Query1" displayName="Query1" ref="A1:C31" tableType="queryTable" totalsRowShown="0" headerRowDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{87538414-6763-4762-BBF9-804546B5DEDD}" name="Table17" displayName="Table17" ref="F2:G40" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10" headerRowBorderDxfId="8" tableBorderDxfId="9">
+  <autoFilter ref="F2:G40" xr:uid="{87538414-6763-4762-BBF9-804546B5DEDD}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{1419F573-7D92-44EA-A170-A65257623B7C}" name="Worksheet Name" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{4D0D2808-2933-4647-9507-8550E222E67F}" name="Table Name" dataDxfId="6"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{D75A3BDE-F911-4A92-A4BD-22AB3C491593}" name="Table19" displayName="Table19" ref="I2:J40" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4" headerRowBorderDxfId="2" tableBorderDxfId="3">
+  <autoFilter ref="I2:J40" xr:uid="{D75A3BDE-F911-4A92-A4BD-22AB3C491593}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{76F27099-1D07-4A3E-B625-2F1D871C3A46}" name="Worksheet Name" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{C1DA07FA-4554-4D5C-B465-36F2CF159E68}" name="Chart Name" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D25BA94F-F2EA-4AAE-942B-F73F6553BE39}" name="Query1" displayName="Query1" ref="A1:C31" tableType="queryTable" totalsRowShown="0" headerRowDxfId="13">
   <autoFilter ref="A1:C31" xr:uid="{D25BA94F-F2EA-4AAE-942B-F73F6553BE39}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{C1A8695F-31C6-45EB-A63A-D4556CD17CBE}" uniqueName="1" name="Year" queryTableFieldId="1"/>
     <tableColumn id="2" xr3:uid="{0C883D22-FCA4-4161-892C-EF72796B8A2D}" uniqueName="2" name="Time To Marity" queryTableFieldId="2"/>
-    <tableColumn id="3" xr3:uid="{B219988D-00A9-4D12-9B24-7CA341ADC811}" uniqueName="3" name="Discount Rate (Nominal)" queryTableFieldId="3" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{B219988D-00A9-4D12-9B24-7CA341ADC811}" uniqueName="3" name="Discount Rate (Nominal)" queryTableFieldId="3" dataDxfId="12"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3910,25 +4574,39 @@
   <sheetPr>
     <tabColor rgb="FF00B0F0"/>
   </sheetPr>
-  <dimension ref="A1:H124"/>
+  <dimension ref="A1:J124"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="29" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.28515625" customWidth="1"/>
+    <col min="7" max="7" width="34.28515625" customWidth="1"/>
+    <col min="9" max="9" width="31.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="25.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.2">
       <c r="A1" s="111" t="s">
         <v>260</v>
       </c>
       <c r="B1" s="112"/>
       <c r="C1" s="112"/>
       <c r="D1" s="113"/>
-    </row>
-    <row r="2" spans="1:8" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="F1" s="129" t="str" cm="1">
+        <f t="array" aca="1" ref="F1" ca="1">_xlfn.TEXTAFTER(_xlfn.TEXTBEFORE(CELL("filename",A1),"]"),"[") &amp; " TABLES"</f>
+        <v>PV2 (color coded).xlsx TABLES</v>
+      </c>
+      <c r="G1" s="130"/>
+      <c r="H1" s="131"/>
+      <c r="I1" s="132" t="str" cm="1">
+        <f t="array" aca="1" ref="I1" ca="1">_xlfn.TEXTAFTER(_xlfn.TEXTBEFORE(CELL("filename",D1),"]"),"[") &amp; " CHARTS"</f>
+        <v>PV2 (color coded).xlsx CHARTS</v>
+      </c>
+      <c r="J1" s="133"/>
+    </row>
+    <row r="2" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
       <c r="A2" s="77" t="s">
         <v>256</v>
       </c>
@@ -3941,714 +4619,880 @@
       <c r="D2" s="79" t="s">
         <v>259</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="F2" s="134" t="s">
+        <v>257</v>
+      </c>
+      <c r="G2" s="135" t="s">
+        <v>443</v>
+      </c>
+      <c r="I2" s="136" t="s">
+        <v>257</v>
+      </c>
+      <c r="J2" s="137" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A3" s="80" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="B3" s="81" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="C3" s="81" t="s">
-        <v>319</v>
+        <v>314</v>
       </c>
       <c r="D3" s="82" cm="1">
         <f t="array" aca="1" ref="D3" ca="1">IF(OR(IF(OR(A3="", B3="", C3=""), "", INDIRECT("'" &amp; B3 &amp; "'!" &amp; C3))=0, IF(OR(A3="", B3="", C3=""), "", INDIRECT("'" &amp; B3 &amp; "'!" &amp; C3))=""),"",INDIRECT("'" &amp; B3 &amp; "'!" &amp; C3))</f>
         <v>46.214921286789867</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="F3" s="138" t="s">
+        <v>445</v>
+      </c>
+      <c r="G3" s="139" t="s">
+        <v>445</v>
+      </c>
+      <c r="I3" s="140" t="s">
+        <v>446</v>
+      </c>
+      <c r="J3" s="141" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A4" s="83" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="B4" s="84" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="C4" s="96" t="s">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="D4" s="85" cm="1">
         <f t="array" aca="1" ref="D4" ca="1">IF(OR(IF(OR(A4="", B4="", C4=""), "", INDIRECT("'" &amp; B4 &amp; "'!" &amp; C4))=0, IF(OR(A4="", B4="", C4=""), "", INDIRECT("'" &amp; B4 &amp; "'!" &amp; C4))=""),"",INDIRECT("'" &amp; B4 &amp; "'!" &amp; C4))</f>
         <v>50.962354551676931</v>
       </c>
-      <c r="G4" t="s">
-        <v>277</v>
-      </c>
-      <c r="H4" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="F4" s="142"/>
+      <c r="G4" s="143"/>
+      <c r="I4" s="144"/>
+      <c r="J4" s="145"/>
+    </row>
+    <row r="5" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A5" s="86" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="B5" s="87" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="C5" s="81" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
       <c r="D5" s="82" cm="1">
         <f t="array" aca="1" ref="D5" ca="1">IF(OR(IF(OR(A5="", B5="", C5=""), "", INDIRECT("'" &amp; B5 &amp; "'!" &amp; C5))=0, IF(OR(A5="", B5="", C5=""), "", INDIRECT("'" &amp; B5 &amp; "'!" &amp; C5))=""),"",INDIRECT("'" &amp; B5 &amp; "'!" &amp; C5))</f>
         <v>33.4</v>
       </c>
-      <c r="G5" t="s">
-        <v>279</v>
-      </c>
-      <c r="H5" t="s">
+      <c r="F5" s="142"/>
+      <c r="G5" s="143"/>
+      <c r="I5" s="144"/>
+      <c r="J5" s="145"/>
+    </row>
+    <row r="6" spans="1:10" ht="15" x14ac:dyDescent="0.25">
+      <c r="A6" s="83" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="A6" s="83" t="s">
-        <v>285</v>
-      </c>
       <c r="B6" s="84" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="C6" s="96" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="D6" s="85" cm="1">
         <f t="array" aca="1" ref="D6" ca="1">IF(OR(IF(OR(A6="", B6="", C6=""), "", INDIRECT("'" &amp; B6 &amp; "'!" &amp; C6))=0, IF(OR(A6="", B6="", C6=""), "", INDIRECT("'" &amp; B6 &amp; "'!" &amp; C6))=""),"",INDIRECT("'" &amp; B6 &amp; "'!" &amp; C6))</f>
         <v>28.652566735112934</v>
       </c>
-      <c r="G6" s="40" t="s">
+      <c r="F6" s="142"/>
+      <c r="G6" s="143"/>
+      <c r="I6" s="144"/>
+      <c r="J6" s="145"/>
+    </row>
+    <row r="7" spans="1:10" ht="15" x14ac:dyDescent="0.25">
+      <c r="A7" s="86" t="s">
         <v>281</v>
       </c>
-      <c r="H6" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="A7" s="86" t="s">
-        <v>286</v>
-      </c>
       <c r="B7" s="87" t="s">
+        <v>313</v>
+      </c>
+      <c r="C7" s="81" t="s">
         <v>318</v>
-      </c>
-      <c r="C7" s="81" t="s">
-        <v>323</v>
       </c>
       <c r="D7" s="82" cm="1">
         <f t="array" aca="1" ref="D7" ca="1">IF(OR(IF(OR(A7="", B7="", C7=""), "", INDIRECT("'" &amp; B7 &amp; "'!" &amp; C7))=0, IF(OR(A7="", B7="", C7=""), "", INDIRECT("'" &amp; B7 &amp; "'!" &amp; C7))=""),"",INDIRECT("'" &amp; B7 &amp; "'!" &amp; C7))</f>
         <v>19.04</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="F7" s="142"/>
+      <c r="G7" s="143"/>
+      <c r="I7" s="144"/>
+      <c r="J7" s="145"/>
+    </row>
+    <row r="8" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A8" s="83" t="s">
-        <v>348</v>
+        <v>343</v>
       </c>
       <c r="B8" s="84" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="C8" s="96" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="D8" s="85" cm="1">
         <f t="array" aca="1" ref="D8" ca="1">IF(OR(IF(OR(A8="", B8="", C8=""), "", INDIRECT("'" &amp; B8 &amp; "'!" &amp; C8))=0, IF(OR(A8="", B8="", C8=""), "", INDIRECT("'" &amp; B8 &amp; "'!" &amp; C8))=""),"",INDIRECT("'" &amp; B8 &amp; "'!" &amp; C8))</f>
         <v>14.292566735112935</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="E8" s="8" t="s">
+        <v>448</v>
+      </c>
+      <c r="F8" s="142"/>
+      <c r="G8" s="143"/>
+      <c r="I8" s="144"/>
+      <c r="J8" s="145"/>
+    </row>
+    <row r="9" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A9" s="97" t="s">
-        <v>349</v>
+        <v>344</v>
       </c>
       <c r="B9" s="98" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="C9" s="104" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
       <c r="D9" s="82" cm="1">
         <f t="array" aca="1" ref="D9" ca="1">IF(OR(IF(OR(A9="", B9="", C9=""), "", INDIRECT("'" &amp; B9 &amp; "'!" &amp; C9))=0, IF(OR(A9="", B9="", C9=""), "", INDIRECT("'" &amp; B9 &amp; "'!" &amp; C9))=""),"",INDIRECT("'" &amp; B9 &amp; "'!" &amp; C9))</f>
         <v>14</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="F9" s="142"/>
+      <c r="G9" s="143"/>
+      <c r="I9" s="144"/>
+      <c r="J9" s="145"/>
+    </row>
+    <row r="10" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A10" s="83" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="B10" s="84" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="C10" s="96" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="D10" s="85" cm="1">
         <f t="array" aca="1" ref="D10" ca="1">IF(OR(IF(OR(A10="", B10="", C10=""), "", INDIRECT("'" &amp; B10 &amp; "'!" &amp; C10))=0, IF(OR(A10="", B10="", C10=""), "", INDIRECT("'" &amp; B10 &amp; "'!" &amp; C10))=""),"",INDIRECT("'" &amp; B10 &amp; "'!" &amp; C10))</f>
         <v>0.29256673511293485</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="F10" s="142"/>
+      <c r="G10" s="143"/>
+      <c r="I10" s="144"/>
+      <c r="J10" s="145"/>
+    </row>
+    <row r="11" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A11" s="86" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="B11" s="87" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="C11" s="87" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="D11" s="82" cm="1">
         <f t="array" aca="1" ref="D11" ca="1">IF(OR(IF(OR(A11="", B11="", C11=""), "", INDIRECT("'" &amp; B11 &amp; "'!" &amp; C11))=0, IF(OR(A11="", B11="", C11=""), "", INDIRECT("'" &amp; B11 &amp; "'!" &amp; C11))=""),"",INDIRECT("'" &amp; B11 &amp; "'!" &amp; C11))</f>
         <v>70</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="F11" s="142"/>
+      <c r="G11" s="143"/>
+      <c r="I11" s="144"/>
+      <c r="J11" s="145"/>
+    </row>
+    <row r="12" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A12" s="83" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
       <c r="B12" s="84" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="C12" s="84" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="D12" s="85" cm="1">
         <f t="array" aca="1" ref="D12" ca="1">IF(OR(IF(OR(A12="", B12="", C12=""), "", INDIRECT("'" &amp; B12 &amp; "'!" &amp; C12))=0, IF(OR(A12="", B12="", C12=""), "", INDIRECT("'" &amp; B12 &amp; "'!" &amp; C12))=""),"",INDIRECT("'" &amp; B12 &amp; "'!" &amp; C12))</f>
         <v>19.037645448323069</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="E12" s="8" t="s">
+        <v>448</v>
+      </c>
+      <c r="F12" s="142"/>
+      <c r="G12" s="143"/>
+      <c r="I12" s="144"/>
+      <c r="J12" s="145"/>
+    </row>
+    <row r="13" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A13" s="97" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="B13" s="98" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="C13" s="98" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="D13" s="82" cm="1">
         <f t="array" aca="1" ref="D13" ca="1">IF(OR(IF(OR(A13="", B13="", C13=""), "", INDIRECT("'" &amp; B13 &amp; "'!" &amp; C13))=0, IF(OR(A13="", B13="", C13=""), "", INDIRECT("'" &amp; B13 &amp; "'!" &amp; C13))=""),"",INDIRECT("'" &amp; B13 &amp; "'!" &amp; C13))</f>
         <v>19</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="F13" s="142"/>
+      <c r="G13" s="143"/>
+      <c r="I13" s="144"/>
+      <c r="J13" s="145"/>
+    </row>
+    <row r="14" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A14" s="83" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
       <c r="B14" s="84" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="C14" s="84" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
       <c r="D14" s="85" cm="1">
         <f t="array" aca="1" ref="D14" ca="1">IF(OR(IF(OR(A14="", B14="", C14=""), "", INDIRECT("'" &amp; B14 &amp; "'!" &amp; C14))=0, IF(OR(A14="", B14="", C14=""), "", INDIRECT("'" &amp; B14 &amp; "'!" &amp; C14))=""),"",INDIRECT("'" &amp; B14 &amp; "'!" &amp; C14))</f>
         <v>3.764544832306882E-2</v>
       </c>
       <c r="E14" s="8"/>
-    </row>
-    <row r="15" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="F14" s="142"/>
+      <c r="G14" s="143"/>
+      <c r="I14" s="144"/>
+      <c r="J14" s="145"/>
+    </row>
+    <row r="15" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A15" s="97" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="B15" s="98" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="C15" s="98" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="D15" s="101" cm="1">
         <f t="array" aca="1" ref="D15" ca="1">IF(OR(IF(OR(A15="", B15="", C15=""), "", INDIRECT("'" &amp; B15 &amp; "'!" &amp; C15))=0, IF(OR(A15="", B15="", C15=""), "", INDIRECT("'" &amp; B15 &amp; "'!" &amp; C15))=""),"",INDIRECT("'" &amp; B15 &amp; "'!" &amp; C15))</f>
         <v>75000</v>
       </c>
       <c r="E15" s="8"/>
-    </row>
-    <row r="16" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="F15" s="142"/>
+      <c r="G15" s="143"/>
+      <c r="I15" s="144"/>
+      <c r="J15" s="145"/>
+    </row>
+    <row r="16" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A16" s="83" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
       <c r="B16" s="84" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="C16" s="84" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="D16" s="105" cm="1">
         <f t="array" aca="1" ref="D16" ca="1">IF(OR(IF(OR(A16="", B16="", C16=""), "", INDIRECT("'" &amp; B16 &amp; "'!" &amp; C16))=0, IF(OR(A16="", B16="", C16=""), "", INDIRECT("'" &amp; B16 &amp; "'!" &amp; C16))=""),"",INDIRECT("'" &amp; B16 &amp; "'!" &amp; C16))</f>
         <v>3.1E-2</v>
       </c>
       <c r="E16" s="8"/>
-    </row>
-    <row r="17" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="F16" s="142"/>
+      <c r="G16" s="143"/>
+      <c r="I16" s="144"/>
+      <c r="J16" s="145"/>
+    </row>
+    <row r="17" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A17" s="86" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="B17" s="87" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="C17" s="87" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="D17" s="101" cm="1">
         <f t="array" aca="1" ref="D17" ca="1">IF(OR(IF(OR(A17="", B17="", C17=""), "", INDIRECT("'" &amp; B17 &amp; "'!" &amp; C17))=0, IF(OR(A17="", B17="", C17=""), "", INDIRECT("'" &amp; B17 &amp; "'!" &amp; C17))=""),"",INDIRECT("'" &amp; B17 &amp; "'!" &amp; C17))</f>
         <v>355890.41095890413</v>
       </c>
       <c r="E17" s="8"/>
-    </row>
-    <row r="18" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="F17" s="142"/>
+      <c r="G17" s="143"/>
+      <c r="I17" s="144"/>
+      <c r="J17" s="145"/>
+    </row>
+    <row r="18" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A18" s="83" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
       <c r="B18" s="84" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="C18" s="84" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="D18" s="102" cm="1">
         <f t="array" aca="1" ref="D18" ca="1">IF(OR(IF(OR(A18="", B18="", C18=""), "", INDIRECT("'" &amp; B18 &amp; "'!" &amp; C18))=0, IF(OR(A18="", B18="", C18=""), "", INDIRECT("'" &amp; B18 &amp; "'!" &amp; C18))=""),"",INDIRECT("'" &amp; B18 &amp; "'!" &amp; C18))</f>
         <v>355890.41095890413</v>
       </c>
       <c r="E18" s="8"/>
-    </row>
-    <row r="19" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="F18" s="142"/>
+      <c r="G18" s="143"/>
+      <c r="I18" s="144"/>
+      <c r="J18" s="145"/>
+    </row>
+    <row r="19" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A19" s="86" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="B19" s="87" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="C19" s="87" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="D19" s="101" cm="1">
         <f t="array" aca="1" ref="D19" ca="1">IF(OR(IF(OR(A19="", B19="", C19=""), "", INDIRECT("'" &amp; B19 &amp; "'!" &amp; C19))=0, IF(OR(A19="", B19="", C19=""), "", INDIRECT("'" &amp; B19 &amp; "'!" &amp; C19))=""),"",INDIRECT("'" &amp; B19 &amp; "'!" &amp; C19))</f>
         <v>1143472.7451096461</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="F19" s="142"/>
+      <c r="G19" s="143"/>
+      <c r="I19" s="144"/>
+      <c r="J19" s="145"/>
+    </row>
+    <row r="20" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A20" s="83" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="B20" s="84" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="C20" s="84" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="D20" s="102" cm="1">
         <f t="array" aca="1" ref="D20" ca="1">IF(OR(IF(OR(A20="", B20="", C20=""), "", INDIRECT("'" &amp; B20 &amp; "'!" &amp; C20))=0, IF(OR(A20="", B20="", C20=""), "", INDIRECT("'" &amp; B20 &amp; "'!" &amp; C20))=""),"",INDIRECT("'" &amp; B20 &amp; "'!" &amp; C20))</f>
         <v>1091912.9611206262</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="F20" s="142"/>
+      <c r="G20" s="143"/>
+      <c r="I20" s="144"/>
+      <c r="J20" s="145"/>
+    </row>
+    <row r="21" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A21" s="97" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="B21" s="98" t="s">
-        <v>434</v>
+        <v>428</v>
       </c>
       <c r="C21" s="98" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="D21" s="101" cm="1">
         <f t="array" aca="1" ref="D21" ca="1">IF(OR(IF(OR(A21="", B21="", C21=""), "", INDIRECT("'" &amp; B21 &amp; "'!" &amp; C21))=0, IF(OR(A21="", B21="", C21=""), "", INDIRECT("'" &amp; B21 &amp; "'!" &amp; C21))=""),"",INDIRECT("'" &amp; B21 &amp; "'!" &amp; C21))</f>
         <v>141416</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="F21" s="142"/>
+      <c r="G21" s="143"/>
+      <c r="I21" s="144"/>
+      <c r="J21" s="145"/>
+    </row>
+    <row r="22" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A22" s="83" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="B22" s="84" t="s">
-        <v>434</v>
+        <v>428</v>
       </c>
       <c r="C22" s="84" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="D22" s="105" cm="1">
         <f t="array" aca="1" ref="D22" ca="1">IF(OR(IF(OR(A22="", B22="", C22=""), "", INDIRECT("'" &amp; B22 &amp; "'!" &amp; C22))=0, IF(OR(A22="", B22="", C22=""), "", INDIRECT("'" &amp; B22 &amp; "'!" &amp; C22))=""),"",INDIRECT("'" &amp; B22 &amp; "'!" &amp; C22))</f>
         <v>3.56E-2</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="F22" s="142"/>
+      <c r="G22" s="143"/>
+      <c r="I22" s="144"/>
+      <c r="J22" s="145"/>
+    </row>
+    <row r="23" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A23" s="86" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="B23" s="87" t="s">
-        <v>434</v>
+        <v>428</v>
       </c>
       <c r="C23" s="87" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="D23" s="101" cm="1">
         <f t="array" aca="1" ref="D23" ca="1">IF(OR(IF(OR(A23="", B23="", C23=""), "", INDIRECT("'" &amp; B23 &amp; "'!" &amp; C23))=0, IF(OR(A23="", B23="", C23=""), "", INDIRECT("'" &amp; B23 &amp; "'!" &amp; C23))=""),"",INDIRECT("'" &amp; B23 &amp; "'!" &amp; C23))</f>
         <v>671047.97808219178</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="F23" s="142"/>
+      <c r="G23" s="143"/>
+      <c r="I23" s="144"/>
+      <c r="J23" s="145"/>
+    </row>
+    <row r="24" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A24" s="83" t="s">
-        <v>375</v>
+        <v>370</v>
       </c>
       <c r="B24" s="84" t="s">
-        <v>434</v>
+        <v>428</v>
       </c>
       <c r="C24" s="84" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="D24" s="102" cm="1">
         <f t="array" aca="1" ref="D24" ca="1">IF(OR(IF(OR(A24="", B24="", C24=""), "", INDIRECT("'" &amp; B24 &amp; "'!" &amp; C24))=0, IF(OR(A24="", B24="", C24=""), "", INDIRECT("'" &amp; B24 &amp; "'!" &amp; C24))=""),"",INDIRECT("'" &amp; B24 &amp; "'!" &amp; C24))</f>
         <v>671047.97808219178</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="F24" s="142"/>
+      <c r="G24" s="143"/>
+      <c r="I24" s="144"/>
+      <c r="J24" s="145"/>
+    </row>
+    <row r="25" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A25" s="86" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="B25" s="87" t="s">
-        <v>434</v>
+        <v>428</v>
       </c>
       <c r="C25" s="87" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="D25" s="101" cm="1">
         <f t="array" aca="1" ref="D25" ca="1">IF(OR(IF(OR(A25="", B25="", C25=""), "", INDIRECT("'" &amp; B25 &amp; "'!" &amp; C25))=0, IF(OR(A25="", B25="", C25=""), "", INDIRECT("'" &amp; B25 &amp; "'!" &amp; C25))=""),"",INDIRECT("'" &amp; B25 &amp; "'!" &amp; C25))</f>
         <v>2926750.9218469802</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="F25" s="142"/>
+      <c r="G25" s="143"/>
+      <c r="I25" s="144"/>
+      <c r="J25" s="145"/>
+    </row>
+    <row r="26" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A26" s="83" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="B26" s="84" t="s">
-        <v>434</v>
+        <v>428</v>
       </c>
       <c r="C26" s="84" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="D26" s="102" cm="1">
         <f t="array" aca="1" ref="D26" ca="1">IF(OR(IF(OR(A26="", B26="", C26=""), "", INDIRECT("'" &amp; B26 &amp; "'!" &amp; C26))=0, IF(OR(A26="", B26="", C26=""), "", INDIRECT("'" &amp; B26 &amp; "'!" &amp; C26))=""),"",INDIRECT("'" &amp; B26 &amp; "'!" &amp; C26))</f>
         <v>2799954.5957609955</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="F26" s="142"/>
+      <c r="G26" s="143"/>
+      <c r="I26" s="144"/>
+      <c r="J26" s="145"/>
+    </row>
+    <row r="27" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A27" s="86" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="B27" s="87" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="C27" s="87" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="D27" s="101" cm="1">
         <f t="array" aca="1" ref="D27" ca="1">IF(OR(IF(OR(A27="", B27="", C27=""), "", INDIRECT("'" &amp; B27 &amp; "'!" &amp; C27))=0, IF(OR(A27="", B27="", C27=""), "", INDIRECT("'" &amp; B27 &amp; "'!" &amp; C27))=""),"",INDIRECT("'" &amp; B27 &amp; "'!" &amp; C27))</f>
         <v>1499363.1560685502</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="F27" s="142"/>
+      <c r="G27" s="143"/>
+      <c r="I27" s="144"/>
+      <c r="J27" s="145"/>
+    </row>
+    <row r="28" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A28" s="83" t="s">
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="B28" s="84" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="C28" s="84" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="D28" s="102" cm="1">
         <f t="array" aca="1" ref="D28" ca="1">IF(OR(IF(OR(A28="", B28="", C28=""), "", INDIRECT("'" &amp; B28 &amp; "'!" &amp; C28))=0, IF(OR(A28="", B28="", C28=""), "", INDIRECT("'" &amp; B28 &amp; "'!" &amp; C28))=""),"",INDIRECT("'" &amp; B28 &amp; "'!" &amp; C28))</f>
         <v>1447803.3720795303</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="F28" s="142"/>
+      <c r="G28" s="143"/>
+      <c r="I28" s="144"/>
+      <c r="J28" s="145"/>
+    </row>
+    <row r="29" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A29" s="86" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="B29" s="87" t="s">
-        <v>434</v>
+        <v>428</v>
       </c>
       <c r="C29" s="87" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="D29" s="101" cm="1">
         <f t="array" aca="1" ref="D29" ca="1">IF(OR(IF(OR(A29="", B29="", C29=""), "", INDIRECT("'" &amp; B29 &amp; "'!" &amp; C29))=0, IF(OR(A29="", B29="", C29=""), "", INDIRECT("'" &amp; B29 &amp; "'!" &amp; C29))=""),"",INDIRECT("'" &amp; B29 &amp; "'!" &amp; C29))</f>
         <v>3597798.8999291719</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="F29" s="142"/>
+      <c r="G29" s="143"/>
+      <c r="I29" s="144"/>
+      <c r="J29" s="145"/>
+    </row>
+    <row r="30" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A30" s="83" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
       <c r="B30" s="84" t="s">
-        <v>434</v>
+        <v>428</v>
       </c>
       <c r="C30" s="84" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="D30" s="102" cm="1">
         <f t="array" aca="1" ref="D30" ca="1">IF(OR(IF(OR(A30="", B30="", C30=""), "", INDIRECT("'" &amp; B30 &amp; "'!" &amp; C30))=0, IF(OR(A30="", B30="", C30=""), "", INDIRECT("'" &amp; B30 &amp; "'!" &amp; C30))=""),"",INDIRECT("'" &amp; B30 &amp; "'!" &amp; C30))</f>
         <v>3471002.5738431872</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="F30" s="142"/>
+      <c r="G30" s="143"/>
+      <c r="I30" s="144"/>
+      <c r="J30" s="145"/>
+    </row>
+    <row r="31" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A31" s="97" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
       <c r="B31" s="98" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="C31" s="98" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="D31" s="101" cm="1">
         <f t="array" aca="1" ref="D31" ca="1">IF(OR(IF(OR(A31="", B31="", C31=""), "", INDIRECT("'" &amp; B31 &amp; "'!" &amp; C31))=0, IF(OR(A31="", B31="", C31=""), "", INDIRECT("'" &amp; B31 &amp; "'!" &amp; C31))=""),"",INDIRECT("'" &amp; B31 &amp; "'!" &amp; C31))</f>
         <v>141416</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="F31" s="142"/>
+      <c r="G31" s="143"/>
+      <c r="I31" s="144"/>
+      <c r="J31" s="145"/>
+    </row>
+    <row r="32" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A32" s="83" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="B32" s="84" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="C32" s="84" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="D32" s="105" cm="1">
         <f t="array" aca="1" ref="D32" ca="1">IF(OR(IF(OR(A32="", B32="", C32=""), "", INDIRECT("'" &amp; B32 &amp; "'!" &amp; C32))=0, IF(OR(A32="", B32="", C32=""), "", INDIRECT("'" &amp; B32 &amp; "'!" &amp; C32))=""),"",INDIRECT("'" &amp; B32 &amp; "'!" &amp; C32))</f>
         <v>3.1E-2</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="F32" s="142"/>
+      <c r="G32" s="143"/>
+      <c r="I32" s="144"/>
+      <c r="J32" s="145"/>
+    </row>
+    <row r="33" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A33" s="86" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="B33" s="87" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="C33" s="87" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="D33" s="101" cm="1">
         <f t="array" aca="1" ref="D33" ca="1">IF(OR(IF(OR(A33="", B33="", C33=""), "", INDIRECT("'" &amp; B33 &amp; "'!" &amp; C33))=0, IF(OR(A33="", B33="", C33=""), "", INDIRECT("'" &amp; B33 &amp; "'!" &amp; C33))=""),"",INDIRECT("'" &amp; B33 &amp; "'!" &amp; C33))</f>
         <v>671047.97808219178</v>
       </c>
-    </row>
-    <row r="34" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="F33" s="142"/>
+      <c r="G33" s="143"/>
+      <c r="I33" s="144"/>
+      <c r="J33" s="145"/>
+    </row>
+    <row r="34" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A34" s="83" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
       <c r="B34" s="84" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="C34" s="84" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="D34" s="102" cm="1">
         <f t="array" aca="1" ref="D34" ca="1">IF(OR(IF(OR(A34="", B34="", C34=""), "", INDIRECT("'" &amp; B34 &amp; "'!" &amp; C34))=0, IF(OR(A34="", B34="", C34=""), "", INDIRECT("'" &amp; B34 &amp; "'!" &amp; C34))=""),"",INDIRECT("'" &amp; B34 &amp; "'!" &amp; C34))</f>
         <v>671047.97808219178</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="F34" s="142"/>
+      <c r="G34" s="143"/>
+      <c r="I34" s="144"/>
+      <c r="J34" s="145"/>
+    </row>
+    <row r="35" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A35" s="86" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="B35" s="87" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="C35" s="87" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="D35" s="101" cm="1">
         <f t="array" aca="1" ref="D35" ca="1">IF(OR(IF(OR(A35="", B35="", C35=""), "", INDIRECT("'" &amp; B35 &amp; "'!" &amp; C35))=0, IF(OR(A35="", B35="", C35=""), "", INDIRECT("'" &amp; B35 &amp; "'!" &amp; C35))=""),"",INDIRECT("'" &amp; B35 &amp; "'!" &amp; C35))</f>
         <v>2156071.2229656759</v>
       </c>
-    </row>
-    <row r="36" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="F35" s="142"/>
+      <c r="G35" s="143"/>
+      <c r="I35" s="144"/>
+      <c r="J35" s="145"/>
+    </row>
+    <row r="36" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A36" s="83" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
       <c r="B36" s="84" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="C36" s="84" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="D36" s="102" cm="1">
         <f t="array" aca="1" ref="D36" ca="1">IF(OR(IF(OR(A36="", B36="", C36=""), "", INDIRECT("'" &amp; B36 &amp; "'!" &amp; C36))=0, IF(OR(A36="", B36="", C36=""), "", INDIRECT("'" &amp; B36 &amp; "'!" &amp; C36))=""),"",INDIRECT("'" &amp; B36 &amp; "'!" &amp; C36))</f>
         <v>2058852.8441311263</v>
       </c>
-    </row>
-    <row r="37" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="F36" s="142"/>
+      <c r="G36" s="143"/>
+      <c r="I36" s="144"/>
+      <c r="J36" s="145"/>
+    </row>
+    <row r="37" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A37" s="97" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="B37" s="98" t="s">
-        <v>435</v>
+        <v>429</v>
       </c>
       <c r="C37" s="98" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="D37" s="101" cm="1">
         <f t="array" aca="1" ref="D37" ca="1">IF(OR(IF(OR(A37="", B37="", C37=""), "", INDIRECT("'" &amp; B37 &amp; "'!" &amp; C37))=0, IF(OR(A37="", B37="", C37=""), "", INDIRECT("'" &amp; B37 &amp; "'!" &amp; C37))=""),"",INDIRECT("'" &amp; B37 &amp; "'!" &amp; C37))</f>
         <v>250000</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="F37" s="142"/>
+      <c r="G37" s="143"/>
+      <c r="I37" s="144"/>
+      <c r="J37" s="145"/>
+    </row>
+    <row r="38" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A38" s="83" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="B38" s="84" t="s">
-        <v>435</v>
+        <v>429</v>
       </c>
       <c r="C38" s="84" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="D38" s="105" cm="1">
         <f t="array" aca="1" ref="D38" ca="1">IF(OR(IF(OR(A38="", B38="", C38=""), "", INDIRECT("'" &amp; B38 &amp; "'!" &amp; C38))=0, IF(OR(A38="", B38="", C38=""), "", INDIRECT("'" &amp; B38 &amp; "'!" &amp; C38))=""),"",INDIRECT("'" &amp; B38 &amp; "'!" &amp; C38))</f>
         <v>3.1E-2</v>
       </c>
-    </row>
-    <row r="39" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="F38" s="142"/>
+      <c r="G38" s="143"/>
+      <c r="I38" s="144"/>
+      <c r="J38" s="145"/>
+    </row>
+    <row r="39" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A39" s="86" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="B39" s="87" t="s">
-        <v>435</v>
+        <v>429</v>
       </c>
       <c r="C39" s="87" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="D39" s="101" cm="1">
         <f t="array" aca="1" ref="D39" ca="1">IF(OR(IF(OR(A39="", B39="", C39=""), "", INDIRECT("'" &amp; B39 &amp; "'!" &amp; C39))=0, IF(OR(A39="", B39="", C39=""), "", INDIRECT("'" &amp; B39 &amp; "'!" &amp; C39))=""),"",INDIRECT("'" &amp; B39 &amp; "'!" &amp; C39))</f>
         <v>1186301.3698630137</v>
       </c>
-    </row>
-    <row r="40" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="F39" s="142"/>
+      <c r="G39" s="143"/>
+      <c r="I39" s="144"/>
+      <c r="J39" s="145"/>
+    </row>
+    <row r="40" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="83" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="B40" s="84" t="s">
-        <v>435</v>
+        <v>429</v>
       </c>
       <c r="C40" s="84" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="D40" s="102" cm="1">
         <f t="array" aca="1" ref="D40" ca="1">IF(OR(IF(OR(A40="", B40="", C40=""), "", INDIRECT("'" &amp; B40 &amp; "'!" &amp; C40))=0, IF(OR(A40="", B40="", C40=""), "", INDIRECT("'" &amp; B40 &amp; "'!" &amp; C40))=""),"",INDIRECT("'" &amp; B40 &amp; "'!" &amp; C40))</f>
         <v>1186301.3698630137</v>
       </c>
-    </row>
-    <row r="41" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="F40" s="146"/>
+      <c r="G40" s="147"/>
+      <c r="I40" s="148"/>
+      <c r="J40" s="149"/>
+    </row>
+    <row r="41" spans="1:10" ht="15" x14ac:dyDescent="0.2">
       <c r="A41" s="86" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="B41" s="87" t="s">
-        <v>435</v>
+        <v>429</v>
       </c>
       <c r="C41" s="87" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="D41" s="101" cm="1">
         <f t="array" aca="1" ref="D41" ca="1">IF(OR(IF(OR(A41="", B41="", C41=""), "", INDIRECT("'" &amp; B41 &amp; "'!" &amp; C41))=0, IF(OR(A41="", B41="", C41=""), "", INDIRECT("'" &amp; B41 &amp; "'!" &amp; C41))=""),"",INDIRECT("'" &amp; B41 &amp; "'!" &amp; C41))</f>
         <v>4941984.4801672073</v>
       </c>
     </row>
-    <row r="42" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:10" ht="15" x14ac:dyDescent="0.2">
       <c r="A42" s="83" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
       <c r="B42" s="84" t="s">
-        <v>435</v>
+        <v>429</v>
       </c>
       <c r="C42" s="84" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="D42" s="102" cm="1">
         <f t="array" aca="1" ref="D42" ca="1">IF(OR(IF(OR(A42="", B42="", C42=""), "", INDIRECT("'" &amp; B42 &amp; "'!" &amp; C42))=0, IF(OR(A42="", B42="", C42=""), "", INDIRECT("'" &amp; B42 &amp; "'!" &amp; C42))=""),"",INDIRECT("'" &amp; B42 &amp; "'!" &amp; C42))</f>
         <v>4736924.6467422284</v>
       </c>
     </row>
-    <row r="43" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:10" ht="15" x14ac:dyDescent="0.2">
       <c r="A43" s="86" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="B43" s="87" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="C43" s="87" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="D43" s="101" cm="1">
         <f t="array" aca="1" ref="D43" ca="1">IF(OR(IF(OR(A43="", B43="", C43=""), "", INDIRECT("'" &amp; B43 &amp; "'!" &amp; C43))=0, IF(OR(A43="", B43="", C43=""), "", INDIRECT("'" &amp; B43 &amp; "'!" &amp; C43))=""),"",INDIRECT("'" &amp; B43 &amp; "'!" &amp; C43))</f>
         <v>2827119.2010478675</v>
       </c>
     </row>
-    <row r="44" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:10" ht="15" x14ac:dyDescent="0.2">
       <c r="A44" s="83" t="s">
-        <v>383</v>
+        <v>378</v>
       </c>
       <c r="B44" s="84" t="s">
+        <v>336</v>
+      </c>
+      <c r="C44" s="84" t="s">
         <v>341</v>
-      </c>
-      <c r="C44" s="84" t="s">
-        <v>346</v>
       </c>
       <c r="D44" s="102" cm="1">
         <f t="array" aca="1" ref="D44" ca="1">IF(OR(IF(OR(A44="", B44="", C44=""), "", INDIRECT("'" &amp; B44 &amp; "'!" &amp; C44))=0, IF(OR(A44="", B44="", C44=""), "", INDIRECT("'" &amp; B44 &amp; "'!" &amp; C44))=""),"",INDIRECT("'" &amp; B44 &amp; "'!" &amp; C44))</f>
         <v>2729900.8222133182</v>
       </c>
-    </row>
-    <row r="45" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="F44" s="8" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" ht="15" x14ac:dyDescent="0.2">
       <c r="A45" s="86" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="B45" s="87" t="s">
-        <v>435</v>
+        <v>429</v>
       </c>
       <c r="C45" s="87" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="D45" s="101" cm="1">
         <f t="array" aca="1" ref="D45" ca="1">IF(OR(IF(OR(A45="", B45="", C45=""), "", INDIRECT("'" &amp; B45 &amp; "'!" &amp; C45))=0, IF(OR(A45="", B45="", C45=""), "", INDIRECT("'" &amp; B45 &amp; "'!" &amp; C45))=""),"",INDIRECT("'" &amp; B45 &amp; "'!" &amp; C45))</f>
         <v>6128285.850030221</v>
       </c>
-    </row>
-    <row r="46" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="F45" s="8" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" ht="15" x14ac:dyDescent="0.2">
       <c r="A46" s="83" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
       <c r="B46" s="84" t="s">
-        <v>435</v>
+        <v>429</v>
       </c>
       <c r="C46" s="84" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="D46" s="102" cm="1">
         <f t="array" aca="1" ref="D46" ca="1">IF(OR(IF(OR(A46="", B46="", C46=""), "", INDIRECT("'" &amp; B46 &amp; "'!" &amp; C46))=0, IF(OR(A46="", B46="", C46=""), "", INDIRECT("'" &amp; B46 &amp; "'!" &amp; C46))=""),"",INDIRECT("'" &amp; B46 &amp; "'!" &amp; C46))</f>
         <v>5923226.0166052422</v>
       </c>
     </row>
-    <row r="47" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:10" ht="15" x14ac:dyDescent="0.2">
       <c r="A47" s="97" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
       <c r="B47" s="98" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="C47" s="98" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="D47" s="101" cm="1">
         <f t="array" aca="1" ref="D47" ca="1">IF(OR(IF(OR(A47="", B47="", C47=""), "", INDIRECT("'" &amp; B47 &amp; "'!" &amp; C47))=0, IF(OR(A47="", B47="", C47=""), "", INDIRECT("'" &amp; B47 &amp; "'!" &amp; C47))=""),"",INDIRECT("'" &amp; B47 &amp; "'!" &amp; C47))</f>
         <v>67888</v>
       </c>
     </row>
-    <row r="48" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:10" ht="15" x14ac:dyDescent="0.2">
       <c r="A48" s="83" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="B48" s="84" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="C48" s="84" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="D48" s="105" cm="1">
         <f t="array" aca="1" ref="D48" ca="1">IF(OR(IF(OR(A48="", B48="", C48=""), "", INDIRECT("'" &amp; B48 &amp; "'!" &amp; C48))=0, IF(OR(A48="", B48="", C48=""), "", INDIRECT("'" &amp; B48 &amp; "'!" &amp; C48))=""),"",INDIRECT("'" &amp; B48 &amp; "'!" &amp; C48))</f>
@@ -4657,13 +5501,13 @@
     </row>
     <row r="49" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A49" s="86" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="B49" s="87" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="C49" s="87" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="D49" s="101" cm="1">
         <f t="array" aca="1" ref="D49" ca="1">IF(OR(IF(OR(A49="", B49="", C49=""), "", INDIRECT("'" &amp; B49 &amp; "'!" &amp; C49))=0, IF(OR(A49="", B49="", C49=""), "", INDIRECT("'" &amp; B49 &amp; "'!" &amp; C49))=""),"",INDIRECT("'" &amp; B49 &amp; "'!" &amp; C49))</f>
@@ -4672,13 +5516,13 @@
     </row>
     <row r="50" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A50" s="83" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="B50" s="84" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="C50" s="84" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="D50" s="102" cm="1">
         <f t="array" aca="1" ref="D50" ca="1">IF(OR(IF(OR(A50="", B50="", C50=""), "", INDIRECT("'" &amp; B50 &amp; "'!" &amp; C50))=0, IF(OR(A50="", B50="", C50=""), "", INDIRECT("'" &amp; B50 &amp; "'!" &amp; C50))=""),"",INDIRECT("'" &amp; B50 &amp; "'!" &amp; C50))</f>
@@ -4687,13 +5531,13 @@
     </row>
     <row r="51" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A51" s="86" t="s">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="B51" s="87" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="C51" s="87" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="D51" s="101" cm="1">
         <f t="array" aca="1" ref="D51" ca="1">IF(OR(IF(OR(A51="", B51="", C51=""), "", INDIRECT("'" &amp; B51 &amp; "'!" &amp; C51))=0, IF(OR(A51="", B51="", C51=""), "", INDIRECT("'" &amp; B51 &amp; "'!" &amp; C51))=""),"",INDIRECT("'" &amp; B51 &amp; "'!" &amp; C51))</f>
@@ -4702,13 +5546,13 @@
     </row>
     <row r="52" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A52" s="83" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="B52" s="84" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="C52" s="84" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="D52" s="102" cm="1">
         <f t="array" aca="1" ref="D52" ca="1">IF(OR(IF(OR(A52="", B52="", C52=""), "", INDIRECT("'" &amp; B52 &amp; "'!" &amp; C52))=0, IF(OR(A52="", B52="", C52=""), "", INDIRECT("'" &amp; B52 &amp; "'!" &amp; C52))=""),"",INDIRECT("'" &amp; B52 &amp; "'!" &amp; C52))</f>
@@ -4717,13 +5561,13 @@
     </row>
     <row r="53" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A53" s="97" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
       <c r="B53" s="98" t="s">
-        <v>436</v>
+        <v>430</v>
       </c>
       <c r="C53" s="98" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="D53" s="101" cm="1">
         <f t="array" aca="1" ref="D53" ca="1">IF(OR(IF(OR(A53="", B53="", C53=""), "", INDIRECT("'" &amp; B53 &amp; "'!" &amp; C53))=0, IF(OR(A53="", B53="", C53=""), "", INDIRECT("'" &amp; B53 &amp; "'!" &amp; C53))=""),"",INDIRECT("'" &amp; B53 &amp; "'!" &amp; C53))</f>
@@ -4732,13 +5576,13 @@
     </row>
     <row r="54" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A54" s="83" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
       <c r="B54" s="84" t="s">
-        <v>436</v>
+        <v>430</v>
       </c>
       <c r="C54" s="84" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="D54" s="105" cm="1">
         <f t="array" aca="1" ref="D54" ca="1">IF(OR(IF(OR(A54="", B54="", C54=""), "", INDIRECT("'" &amp; B54 &amp; "'!" &amp; C54))=0, IF(OR(A54="", B54="", C54=""), "", INDIRECT("'" &amp; B54 &amp; "'!" &amp; C54))=""),"",INDIRECT("'" &amp; B54 &amp; "'!" &amp; C54))</f>
@@ -4747,13 +5591,13 @@
     </row>
     <row r="55" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A55" s="86" t="s">
-        <v>302</v>
+        <v>297</v>
       </c>
       <c r="B55" s="87" t="s">
-        <v>436</v>
+        <v>430</v>
       </c>
       <c r="C55" s="87" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="D55" s="101" cm="1">
         <f t="array" aca="1" ref="D55" ca="1">IF(OR(IF(OR(A55="", B55="", C55=""), "", INDIRECT("'" &amp; B55 &amp; "'!" &amp; C55))=0, IF(OR(A55="", B55="", C55=""), "", INDIRECT("'" &amp; B55 &amp; "'!" &amp; C55))=""),"",INDIRECT("'" &amp; B55 &amp; "'!" &amp; C55))</f>
@@ -4762,13 +5606,13 @@
     </row>
     <row r="56" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A56" s="83" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="B56" s="84" t="s">
-        <v>436</v>
+        <v>430</v>
       </c>
       <c r="C56" s="84" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="D56" s="102" cm="1">
         <f t="array" aca="1" ref="D56" ca="1">IF(OR(IF(OR(A56="", B56="", C56=""), "", INDIRECT("'" &amp; B56 &amp; "'!" &amp; C56))=0, IF(OR(A56="", B56="", C56=""), "", INDIRECT("'" &amp; B56 &amp; "'!" &amp; C56))=""),"",INDIRECT("'" &amp; B56 &amp; "'!" &amp; C56))</f>
@@ -4777,13 +5621,13 @@
     </row>
     <row r="57" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A57" s="86" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="B57" s="87" t="s">
-        <v>436</v>
+        <v>430</v>
       </c>
       <c r="C57" s="87" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="D57" s="101" cm="1">
         <f t="array" aca="1" ref="D57" ca="1">IF(OR(IF(OR(A57="", B57="", C57=""), "", INDIRECT("'" &amp; B57 &amp; "'!" &amp; C57))=0, IF(OR(A57="", B57="", C57=""), "", INDIRECT("'" &amp; B57 &amp; "'!" &amp; C57))=""),"",INDIRECT("'" &amp; B57 &amp; "'!" &amp; C57))</f>
@@ -4792,13 +5636,13 @@
     </row>
     <row r="58" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A58" s="83" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
       <c r="B58" s="84" t="s">
-        <v>436</v>
+        <v>430</v>
       </c>
       <c r="C58" s="84" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="D58" s="102" cm="1">
         <f t="array" aca="1" ref="D58" ca="1">IF(OR(IF(OR(A58="", B58="", C58=""), "", INDIRECT("'" &amp; B58 &amp; "'!" &amp; C58))=0, IF(OR(A58="", B58="", C58=""), "", INDIRECT("'" &amp; B58 &amp; "'!" &amp; C58))=""),"",INDIRECT("'" &amp; B58 &amp; "'!" &amp; C58))</f>
@@ -4807,13 +5651,13 @@
     </row>
     <row r="59" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A59" s="86" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="B59" s="87" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="C59" s="87" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="D59" s="101" cm="1">
         <f t="array" aca="1" ref="D59" ca="1">IF(OR(IF(OR(A59="", B59="", C59=""), "", INDIRECT("'" &amp; B59 &amp; "'!" &amp; C59))=0, IF(OR(A59="", B59="", C59=""), "", INDIRECT("'" &amp; B59 &amp; "'!" &amp; C59))=""),"",INDIRECT("'" &amp; B59 &amp; "'!" &amp; C59))</f>
@@ -4822,13 +5666,13 @@
     </row>
     <row r="60" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A60" s="83" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
       <c r="B60" s="84" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="C60" s="84" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="D60" s="102" cm="1">
         <f t="array" aca="1" ref="D60" ca="1">IF(OR(IF(OR(A60="", B60="", C60=""), "", INDIRECT("'" &amp; B60 &amp; "'!" &amp; C60))=0, IF(OR(A60="", B60="", C60=""), "", INDIRECT("'" &amp; B60 &amp; "'!" &amp; C60))=""),"",INDIRECT("'" &amp; B60 &amp; "'!" &amp; C60))</f>
@@ -4837,13 +5681,13 @@
     </row>
     <row r="61" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A61" s="86" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="B61" s="87" t="s">
-        <v>436</v>
+        <v>430</v>
       </c>
       <c r="C61" s="87" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="D61" s="101" cm="1">
         <f t="array" aca="1" ref="D61" ca="1">IF(OR(IF(OR(A61="", B61="", C61=""), "", INDIRECT("'" &amp; B61 &amp; "'!" &amp; C61))=0, IF(OR(A61="", B61="", C61=""), "", INDIRECT("'" &amp; B61 &amp; "'!" &amp; C61))=""),"",INDIRECT("'" &amp; B61 &amp; "'!" &amp; C61))</f>
@@ -4852,13 +5696,13 @@
     </row>
     <row r="62" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A62" s="83" t="s">
-        <v>390</v>
+        <v>385</v>
       </c>
       <c r="B62" s="84" t="s">
-        <v>436</v>
+        <v>430</v>
       </c>
       <c r="C62" s="84" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="D62" s="102" cm="1">
         <f t="array" aca="1" ref="D62" ca="1">IF(OR(IF(OR(A62="", B62="", C62=""), "", INDIRECT("'" &amp; B62 &amp; "'!" &amp; C62))=0, IF(OR(A62="", B62="", C62=""), "", INDIRECT("'" &amp; B62 &amp; "'!" &amp; C62))=""),"",INDIRECT("'" &amp; B62 &amp; "'!" &amp; C62))</f>
@@ -4867,13 +5711,13 @@
     </row>
     <row r="63" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A63" s="97" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="B63" s="98" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="C63" s="98" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="D63" s="101" cm="1">
         <f t="array" aca="1" ref="D63" ca="1">IF(OR(IF(OR(A63="", B63="", C63=""), "", INDIRECT("'" &amp; B63 &amp; "'!" &amp; C63))=0, IF(OR(A63="", B63="", C63=""), "", INDIRECT("'" &amp; B63 &amp; "'!" &amp; C63))=""),"",INDIRECT("'" &amp; B63 &amp; "'!" &amp; C63))</f>
@@ -4882,13 +5726,13 @@
     </row>
     <row r="64" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A64" s="83" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="B64" s="84" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="C64" s="84" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="D64" s="105" cm="1">
         <f t="array" aca="1" ref="D64" ca="1">IF(OR(IF(OR(A64="", B64="", C64=""), "", INDIRECT("'" &amp; B64 &amp; "'!" &amp; C64))=0, IF(OR(A64="", B64="", C64=""), "", INDIRECT("'" &amp; B64 &amp; "'!" &amp; C64))=""),"",INDIRECT("'" &amp; B64 &amp; "'!" &amp; C64))</f>
@@ -4897,13 +5741,13 @@
     </row>
     <row r="65" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A65" s="86" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="B65" s="87" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="C65" s="87" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="D65" s="101" cm="1">
         <f t="array" aca="1" ref="D65" ca="1">IF(OR(IF(OR(A65="", B65="", C65=""), "", INDIRECT("'" &amp; B65 &amp; "'!" &amp; C65))=0, IF(OR(A65="", B65="", C65=""), "", INDIRECT("'" &amp; B65 &amp; "'!" &amp; C65))=""),"",INDIRECT("'" &amp; B65 &amp; "'!" &amp; C65))</f>
@@ -4912,13 +5756,13 @@
     </row>
     <row r="66" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A66" s="83" t="s">
-        <v>391</v>
+        <v>386</v>
       </c>
       <c r="B66" s="84" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="C66" s="84" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="D66" s="102" cm="1">
         <f t="array" aca="1" ref="D66" ca="1">IF(OR(IF(OR(A66="", B66="", C66=""), "", INDIRECT("'" &amp; B66 &amp; "'!" &amp; C66))=0, IF(OR(A66="", B66="", C66=""), "", INDIRECT("'" &amp; B66 &amp; "'!" &amp; C66))=""),"",INDIRECT("'" &amp; B66 &amp; "'!" &amp; C66))</f>
@@ -4927,13 +5771,13 @@
     </row>
     <row r="67" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A67" s="86" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="B67" s="87" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="C67" s="87" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="D67" s="101" cm="1">
         <f t="array" aca="1" ref="D67" ca="1">IF(OR(IF(OR(A67="", B67="", C67=""), "", INDIRECT("'" &amp; B67 &amp; "'!" &amp; C67))=0, IF(OR(A67="", B67="", C67=""), "", INDIRECT("'" &amp; B67 &amp; "'!" &amp; C67))=""),"",INDIRECT("'" &amp; B67 &amp; "'!" &amp; C67))</f>
@@ -4942,13 +5786,13 @@
     </row>
     <row r="68" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A68" s="83" t="s">
-        <v>392</v>
+        <v>387</v>
       </c>
       <c r="B68" s="84" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="C68" s="84" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="D68" s="102" cm="1">
         <f t="array" aca="1" ref="D68" ca="1">IF(OR(IF(OR(A68="", B68="", C68=""), "", INDIRECT("'" &amp; B68 &amp; "'!" &amp; C68))=0, IF(OR(A68="", B68="", C68=""), "", INDIRECT("'" &amp; B68 &amp; "'!" &amp; C68))=""),"",INDIRECT("'" &amp; B68 &amp; "'!" &amp; C68))</f>
@@ -4957,13 +5801,13 @@
     </row>
     <row r="69" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A69" s="97" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="B69" s="98" t="s">
-        <v>437</v>
+        <v>431</v>
       </c>
       <c r="C69" s="98" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="D69" s="101" cm="1">
         <f t="array" aca="1" ref="D69" ca="1">IF(OR(IF(OR(A69="", B69="", C69=""), "", INDIRECT("'" &amp; B69 &amp; "'!" &amp; C69))=0, IF(OR(A69="", B69="", C69=""), "", INDIRECT("'" &amp; B69 &amp; "'!" &amp; C69))=""),"",INDIRECT("'" &amp; B69 &amp; "'!" &amp; C69))</f>
@@ -4972,13 +5816,13 @@
     </row>
     <row r="70" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A70" s="83" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
       <c r="B70" s="84" t="s">
-        <v>437</v>
+        <v>431</v>
       </c>
       <c r="C70" s="84" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="D70" s="105" cm="1">
         <f t="array" aca="1" ref="D70" ca="1">IF(OR(IF(OR(A70="", B70="", C70=""), "", INDIRECT("'" &amp; B70 &amp; "'!" &amp; C70))=0, IF(OR(A70="", B70="", C70=""), "", INDIRECT("'" &amp; B70 &amp; "'!" &amp; C70))=""),"",INDIRECT("'" &amp; B70 &amp; "'!" &amp; C70))</f>
@@ -4987,13 +5831,13 @@
     </row>
     <row r="71" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A71" s="86" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
       <c r="B71" s="87" t="s">
-        <v>437</v>
+        <v>431</v>
       </c>
       <c r="C71" s="87" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="D71" s="101" cm="1">
         <f t="array" aca="1" ref="D71" ca="1">IF(OR(IF(OR(A71="", B71="", C71=""), "", INDIRECT("'" &amp; B71 &amp; "'!" &amp; C71))=0, IF(OR(A71="", B71="", C71=""), "", INDIRECT("'" &amp; B71 &amp; "'!" &amp; C71))=""),"",INDIRECT("'" &amp; B71 &amp; "'!" &amp; C71))</f>
@@ -5002,13 +5846,13 @@
     </row>
     <row r="72" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A72" s="83" t="s">
-        <v>393</v>
+        <v>388</v>
       </c>
       <c r="B72" s="84" t="s">
-        <v>437</v>
+        <v>431</v>
       </c>
       <c r="C72" s="84" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="D72" s="102" cm="1">
         <f t="array" aca="1" ref="D72" ca="1">IF(OR(IF(OR(A72="", B72="", C72=""), "", INDIRECT("'" &amp; B72 &amp; "'!" &amp; C72))=0, IF(OR(A72="", B72="", C72=""), "", INDIRECT("'" &amp; B72 &amp; "'!" &amp; C72))=""),"",INDIRECT("'" &amp; B72 &amp; "'!" &amp; C72))</f>
@@ -5017,13 +5861,13 @@
     </row>
     <row r="73" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A73" s="86" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="B73" s="87" t="s">
-        <v>437</v>
+        <v>431</v>
       </c>
       <c r="C73" s="87" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="D73" s="101" cm="1">
         <f t="array" aca="1" ref="D73" ca="1">IF(OR(IF(OR(A73="", B73="", C73=""), "", INDIRECT("'" &amp; B73 &amp; "'!" &amp; C73))=0, IF(OR(A73="", B73="", C73=""), "", INDIRECT("'" &amp; B73 &amp; "'!" &amp; C73))=""),"",INDIRECT("'" &amp; B73 &amp; "'!" &amp; C73))</f>
@@ -5032,13 +5876,13 @@
     </row>
     <row r="74" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A74" s="83" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
       <c r="B74" s="84" t="s">
-        <v>437</v>
+        <v>431</v>
       </c>
       <c r="C74" s="84" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="D74" s="102" cm="1">
         <f t="array" aca="1" ref="D74" ca="1">IF(OR(IF(OR(A74="", B74="", C74=""), "", INDIRECT("'" &amp; B74 &amp; "'!" &amp; C74))=0, IF(OR(A74="", B74="", C74=""), "", INDIRECT("'" &amp; B74 &amp; "'!" &amp; C74))=""),"",INDIRECT("'" &amp; B74 &amp; "'!" &amp; C74))</f>
@@ -5047,13 +5891,13 @@
     </row>
     <row r="75" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A75" s="86" t="s">
-        <v>310</v>
+        <v>305</v>
       </c>
       <c r="B75" s="87" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="C75" s="87" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="D75" s="101" cm="1">
         <f t="array" aca="1" ref="D75" ca="1">IF(OR(IF(OR(A75="", B75="", C75=""), "", INDIRECT("'" &amp; B75 &amp; "'!" &amp; C75))=0, IF(OR(A75="", B75="", C75=""), "", INDIRECT("'" &amp; B75 &amp; "'!" &amp; C75))=""),"",INDIRECT("'" &amp; B75 &amp; "'!" &amp; C75))</f>
@@ -5062,13 +5906,13 @@
     </row>
     <row r="76" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A76" s="94" t="s">
-        <v>395</v>
+        <v>390</v>
       </c>
       <c r="B76" s="84" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="C76" s="88" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="D76" s="102" cm="1">
         <f t="array" aca="1" ref="D76" ca="1">IF(OR(IF(OR(A76="", B76="", C76=""), "", INDIRECT("'" &amp; B76 &amp; "'!" &amp; C76))=0, IF(OR(A76="", B76="", C76=""), "", INDIRECT("'" &amp; B76 &amp; "'!" &amp; C76))=""),"",INDIRECT("'" &amp; B76 &amp; "'!" &amp; C76))</f>
@@ -5077,13 +5921,13 @@
     </row>
     <row r="77" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A77" s="95" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="B77" s="87" t="s">
-        <v>437</v>
+        <v>431</v>
       </c>
       <c r="C77" s="89" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="D77" s="101" cm="1">
         <f t="array" aca="1" ref="D77" ca="1">IF(OR(IF(OR(A77="", B77="", C77=""), "", INDIRECT("'" &amp; B77 &amp; "'!" &amp; C77))=0, IF(OR(A77="", B77="", C77=""), "", INDIRECT("'" &amp; B77 &amp; "'!" &amp; C77))=""),"",INDIRECT("'" &amp; B77 &amp; "'!" &amp; C77))</f>
@@ -5092,13 +5936,13 @@
     </row>
     <row r="78" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A78" s="94" t="s">
-        <v>396</v>
+        <v>391</v>
       </c>
       <c r="B78" s="84" t="s">
-        <v>437</v>
+        <v>431</v>
       </c>
       <c r="C78" s="88" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="D78" s="102" cm="1">
         <f t="array" aca="1" ref="D78" ca="1">IF(OR(IF(OR(A78="", B78="", C78=""), "", INDIRECT("'" &amp; B78 &amp; "'!" &amp; C78))=0, IF(OR(A78="", B78="", C78=""), "", INDIRECT("'" &amp; B78 &amp; "'!" &amp; C78))=""),"",INDIRECT("'" &amp; B78 &amp; "'!" &amp; C78))</f>
@@ -5107,13 +5951,13 @@
     </row>
     <row r="79" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A79" s="97" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
       <c r="B79" s="98" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="C79" s="98" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="D79" s="101" cm="1">
         <f t="array" aca="1" ref="D79" ca="1">IF(OR(IF(OR(A79="", B79="", C79=""), "", INDIRECT("'" &amp; B79 &amp; "'!" &amp; C79))=0, IF(OR(A79="", B79="", C79=""), "", INDIRECT("'" &amp; B79 &amp; "'!" &amp; C79))=""),"",INDIRECT("'" &amp; B79 &amp; "'!" &amp; C79))</f>
@@ -5122,13 +5966,13 @@
     </row>
     <row r="80" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A80" s="83" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="B80" s="84" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="C80" s="84" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="D80" s="105" cm="1">
         <f t="array" aca="1" ref="D80" ca="1">IF(OR(IF(OR(A80="", B80="", C80=""), "", INDIRECT("'" &amp; B80 &amp; "'!" &amp; C80))=0, IF(OR(A80="", B80="", C80=""), "", INDIRECT("'" &amp; B80 &amp; "'!" &amp; C80))=""),"",INDIRECT("'" &amp; B80 &amp; "'!" &amp; C80))</f>
@@ -5137,13 +5981,13 @@
     </row>
     <row r="81" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A81" s="86" t="s">
-        <v>312</v>
+        <v>307</v>
       </c>
       <c r="B81" s="89" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="C81" s="89" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="D81" s="101" cm="1">
         <f t="array" aca="1" ref="D81" ca="1">IF(OR(IF(OR(A81="", B81="", C81=""), "", INDIRECT("'" &amp; B81 &amp; "'!" &amp; C81))=0, IF(OR(A81="", B81="", C81=""), "", INDIRECT("'" &amp; B81 &amp; "'!" &amp; C81))=""),"",INDIRECT("'" &amp; B81 &amp; "'!" &amp; C81))</f>
@@ -5152,13 +5996,13 @@
     </row>
     <row r="82" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A82" s="83" t="s">
-        <v>397</v>
+        <v>392</v>
       </c>
       <c r="B82" s="88" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="C82" s="88" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="D82" s="102" cm="1">
         <f t="array" aca="1" ref="D82" ca="1">IF(OR(IF(OR(A82="", B82="", C82=""), "", INDIRECT("'" &amp; B82 &amp; "'!" &amp; C82))=0, IF(OR(A82="", B82="", C82=""), "", INDIRECT("'" &amp; B82 &amp; "'!" &amp; C82))=""),"",INDIRECT("'" &amp; B82 &amp; "'!" &amp; C82))</f>
@@ -5167,13 +6011,13 @@
     </row>
     <row r="83" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A83" s="86" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="B83" s="89" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="C83" s="89" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="D83" s="101" cm="1">
         <f t="array" aca="1" ref="D83" ca="1">IF(OR(IF(OR(A83="", B83="", C83=""), "", INDIRECT("'" &amp; B83 &amp; "'!" &amp; C83))=0, IF(OR(A83="", B83="", C83=""), "", INDIRECT("'" &amp; B83 &amp; "'!" &amp; C83))=""),"",INDIRECT("'" &amp; B83 &amp; "'!" &amp; C83))</f>
@@ -5182,13 +6026,13 @@
     </row>
     <row r="84" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A84" s="83" t="s">
-        <v>398</v>
+        <v>393</v>
       </c>
       <c r="B84" s="88" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="C84" s="88" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="D84" s="102" cm="1">
         <f t="array" aca="1" ref="D84" ca="1">IF(OR(IF(OR(A84="", B84="", C84=""), "", INDIRECT("'" &amp; B84 &amp; "'!" &amp; C84))=0, IF(OR(A84="", B84="", C84=""), "", INDIRECT("'" &amp; B84 &amp; "'!" &amp; C84))=""),"",INDIRECT("'" &amp; B84 &amp; "'!" &amp; C84))</f>
@@ -5197,13 +6041,13 @@
     </row>
     <row r="85" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A85" s="97" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="B85" s="98" t="s">
-        <v>438</v>
+        <v>432</v>
       </c>
       <c r="C85" s="98" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="D85" s="101" cm="1">
         <f t="array" aca="1" ref="D85" ca="1">IF(OR(IF(OR(A85="", B85="", C85=""), "", INDIRECT("'" &amp; B85 &amp; "'!" &amp; C85))=0, IF(OR(A85="", B85="", C85=""), "", INDIRECT("'" &amp; B85 &amp; "'!" &amp; C85))=""),"",INDIRECT("'" &amp; B85 &amp; "'!" &amp; C85))</f>
@@ -5212,13 +6056,13 @@
     </row>
     <row r="86" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A86" s="83" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="B86" s="84" t="s">
-        <v>438</v>
+        <v>432</v>
       </c>
       <c r="C86" s="84" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="D86" s="105" cm="1">
         <f t="array" aca="1" ref="D86" ca="1">IF(OR(IF(OR(A86="", B86="", C86=""), "", INDIRECT("'" &amp; B86 &amp; "'!" &amp; C86))=0, IF(OR(A86="", B86="", C86=""), "", INDIRECT("'" &amp; B86 &amp; "'!" &amp; C86))=""),"",INDIRECT("'" &amp; B86 &amp; "'!" &amp; C86))</f>
@@ -5227,13 +6071,13 @@
     </row>
     <row r="87" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A87" s="86" t="s">
-        <v>314</v>
+        <v>309</v>
       </c>
       <c r="B87" s="89" t="s">
-        <v>438</v>
+        <v>432</v>
       </c>
       <c r="C87" s="89" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="D87" s="101" cm="1">
         <f t="array" aca="1" ref="D87" ca="1">IF(OR(IF(OR(A87="", B87="", C87=""), "", INDIRECT("'" &amp; B87 &amp; "'!" &amp; C87))=0, IF(OR(A87="", B87="", C87=""), "", INDIRECT("'" &amp; B87 &amp; "'!" &amp; C87))=""),"",INDIRECT("'" &amp; B87 &amp; "'!" &amp; C87))</f>
@@ -5242,13 +6086,13 @@
     </row>
     <row r="88" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A88" s="83" t="s">
-        <v>399</v>
+        <v>394</v>
       </c>
       <c r="B88" s="88" t="s">
-        <v>438</v>
+        <v>432</v>
       </c>
       <c r="C88" s="88" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="D88" s="102" cm="1">
         <f t="array" aca="1" ref="D88" ca="1">IF(OR(IF(OR(A88="", B88="", C88=""), "", INDIRECT("'" &amp; B88 &amp; "'!" &amp; C88))=0, IF(OR(A88="", B88="", C88=""), "", INDIRECT("'" &amp; B88 &amp; "'!" &amp; C88))=""),"",INDIRECT("'" &amp; B88 &amp; "'!" &amp; C88))</f>
@@ -5257,13 +6101,13 @@
     </row>
     <row r="89" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A89" s="86" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="B89" s="89" t="s">
-        <v>438</v>
+        <v>432</v>
       </c>
       <c r="C89" s="89" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="D89" s="101" cm="1">
         <f t="array" aca="1" ref="D89" ca="1">IF(OR(IF(OR(A89="", B89="", C89=""), "", INDIRECT("'" &amp; B89 &amp; "'!" &amp; C89))=0, IF(OR(A89="", B89="", C89=""), "", INDIRECT("'" &amp; B89 &amp; "'!" &amp; C89))=""),"",INDIRECT("'" &amp; B89 &amp; "'!" &amp; C89))</f>
@@ -5272,13 +6116,13 @@
     </row>
     <row r="90" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A90" s="83" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="B90" s="88" t="s">
-        <v>438</v>
+        <v>432</v>
       </c>
       <c r="C90" s="88" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="D90" s="102" cm="1">
         <f t="array" aca="1" ref="D90" ca="1">IF(OR(IF(OR(A90="", B90="", C90=""), "", INDIRECT("'" &amp; B90 &amp; "'!" &amp; C90))=0, IF(OR(A90="", B90="", C90=""), "", INDIRECT("'" &amp; B90 &amp; "'!" &amp; C90))=""),"",INDIRECT("'" &amp; B90 &amp; "'!" &amp; C90))</f>
@@ -5287,13 +6131,13 @@
     </row>
     <row r="91" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A91" s="86" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="B91" s="89" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="C91" s="89" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="D91" s="101" cm="1">
         <f t="array" aca="1" ref="D91" ca="1">IF(OR(IF(OR(A91="", B91="", C91=""), "", INDIRECT("'" &amp; B91 &amp; "'!" &amp; C91))=0, IF(OR(A91="", B91="", C91=""), "", INDIRECT("'" &amp; B91 &amp; "'!" &amp; C91))=""),"",INDIRECT("'" &amp; B91 &amp; "'!" &amp; C91))</f>
@@ -5302,13 +6146,13 @@
     </row>
     <row r="92" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A92" s="94" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="B92" s="88" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="C92" s="88" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="D92" s="102" cm="1">
         <f t="array" aca="1" ref="D92" ca="1">IF(OR(IF(OR(A92="", B92="", C92=""), "", INDIRECT("'" &amp; B92 &amp; "'!" &amp; C92))=0, IF(OR(A92="", B92="", C92=""), "", INDIRECT("'" &amp; B92 &amp; "'!" &amp; C92))=""),"",INDIRECT("'" &amp; B92 &amp; "'!" &amp; C92))</f>
@@ -5317,13 +6161,13 @@
     </row>
     <row r="93" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A93" s="95" t="s">
-        <v>317</v>
+        <v>312</v>
       </c>
       <c r="B93" s="89" t="s">
-        <v>438</v>
+        <v>432</v>
       </c>
       <c r="C93" s="89" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="D93" s="101" cm="1">
         <f t="array" aca="1" ref="D93" ca="1">IF(OR(IF(OR(A93="", B93="", C93=""), "", INDIRECT("'" &amp; B93 &amp; "'!" &amp; C93))=0, IF(OR(A93="", B93="", C93=""), "", INDIRECT("'" &amp; B93 &amp; "'!" &amp; C93))=""),"",INDIRECT("'" &amp; B93 &amp; "'!" &amp; C93))</f>
@@ -5332,13 +6176,13 @@
     </row>
     <row r="94" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A94" s="94" t="s">
-        <v>402</v>
+        <v>397</v>
       </c>
       <c r="B94" s="88" t="s">
-        <v>438</v>
+        <v>432</v>
       </c>
       <c r="C94" s="88" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="D94" s="102" cm="1">
         <f t="array" aca="1" ref="D94" ca="1">IF(OR(IF(OR(A94="", B94="", C94=""), "", INDIRECT("'" &amp; B94 &amp; "'!" &amp; C94))=0, IF(OR(A94="", B94="", C94=""), "", INDIRECT("'" &amp; B94 &amp; "'!" &amp; C94))=""),"",INDIRECT("'" &amp; B94 &amp; "'!" &amp; C94))</f>
@@ -5347,7 +6191,7 @@
     </row>
     <row r="95" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A95" s="107" t="s">
-        <v>432</v>
+        <v>427</v>
       </c>
       <c r="B95" s="89"/>
       <c r="C95" s="89"/>
@@ -5358,7 +6202,7 @@
     </row>
     <row r="96" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A96" s="107" t="s">
-        <v>440</v>
+        <v>434</v>
       </c>
       <c r="B96" s="88"/>
       <c r="C96" s="88"/>
@@ -5369,7 +6213,7 @@
     </row>
     <row r="97" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A97" s="107" t="s">
-        <v>439</v>
+        <v>433</v>
       </c>
       <c r="B97" s="89"/>
       <c r="C97" s="89"/>
@@ -5380,13 +6224,13 @@
     </row>
     <row r="98" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A98" s="94" t="s">
-        <v>441</v>
+        <v>435</v>
       </c>
       <c r="B98" s="88" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="C98" s="88" t="s">
-        <v>442</v>
+        <v>436</v>
       </c>
       <c r="D98" s="108" cm="1">
         <f t="array" aca="1" ref="D98" ca="1">IF(OR(IF(OR(A98="", B98="", C98=""), "", INDIRECT("'" &amp; B98 &amp; "'!" &amp; C98))=0, IF(OR(A98="", B98="", C98=""), "", INDIRECT("'" &amp; B98 &amp; "'!" &amp; C98))=""),"",INDIRECT("'" &amp; B98 &amp; "'!" &amp; C98))</f>
@@ -5395,7 +6239,7 @@
     </row>
     <row r="99" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A99" s="109" t="s">
-        <v>443</v>
+        <v>437</v>
       </c>
       <c r="B99" s="89"/>
       <c r="C99" s="89"/>
@@ -5406,7 +6250,7 @@
     </row>
     <row r="100" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A100" s="109" t="s">
-        <v>444</v>
+        <v>438</v>
       </c>
       <c r="B100" s="88"/>
       <c r="C100" s="88"/>
@@ -5632,12 +6476,18 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="3">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="I1:J1"/>
   </mergeCells>
   <phoneticPr fontId="31" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <tableParts count="2">
+    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -5791,7 +6641,7 @@
         <v>125</v>
       </c>
       <c r="H8" s="19" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="AE8" s="7"/>
       <c r="AF8" s="7"/>
@@ -7881,7 +8731,7 @@
         <v>125</v>
       </c>
       <c r="H8" s="19" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="AE8" s="7"/>
       <c r="AF8" s="7"/>
@@ -9790,7 +10640,7 @@
         <v>125</v>
       </c>
       <c r="H8" s="19" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="AE8" s="7"/>
       <c r="AF8" s="7"/>
@@ -11699,7 +12549,7 @@
         <v>125</v>
       </c>
       <c r="H8" s="19" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="AE8" s="7"/>
       <c r="AF8" s="7"/>
@@ -13612,7 +14462,7 @@
         <v>125</v>
       </c>
       <c r="H8" s="19" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="AE8" s="7"/>
       <c r="AF8" s="7"/>
@@ -15428,7 +16278,7 @@
         <v>6</v>
       </c>
       <c r="C2" s="33" t="s">
-        <v>403</v>
+        <v>398</v>
       </c>
       <c r="E2" s="34" t="s">
         <v>106</v>
@@ -15443,7 +16293,7 @@
         <v>8</v>
       </c>
       <c r="C3" s="33" t="s">
-        <v>404</v>
+        <v>399</v>
       </c>
       <c r="G3" s="6"/>
     </row>
@@ -15455,7 +16305,7 @@
         <v>10</v>
       </c>
       <c r="C4" s="33" t="s">
-        <v>405</v>
+        <v>400</v>
       </c>
       <c r="G4" s="6"/>
     </row>
@@ -15467,7 +16317,7 @@
         <v>12</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>406</v>
+        <v>401</v>
       </c>
       <c r="G5" s="6"/>
     </row>
@@ -15479,7 +16329,7 @@
         <v>14</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>407</v>
+        <v>402</v>
       </c>
       <c r="G6" s="6"/>
     </row>
@@ -15491,7 +16341,7 @@
         <v>16</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>408</v>
+        <v>403</v>
       </c>
       <c r="G7" s="6"/>
     </row>
@@ -15503,7 +16353,7 @@
         <v>18</v>
       </c>
       <c r="C8" s="33" t="s">
-        <v>409</v>
+        <v>404</v>
       </c>
       <c r="G8" s="6"/>
     </row>
@@ -15515,7 +16365,7 @@
         <v>20</v>
       </c>
       <c r="C9" s="33" t="s">
-        <v>410</v>
+        <v>405</v>
       </c>
       <c r="G9" s="6"/>
     </row>
@@ -15527,7 +16377,7 @@
         <v>22</v>
       </c>
       <c r="C10" s="33" t="s">
-        <v>411</v>
+        <v>406</v>
       </c>
       <c r="G10" s="6"/>
     </row>
@@ -15539,7 +16389,7 @@
         <v>24</v>
       </c>
       <c r="C11" s="33" t="s">
-        <v>412</v>
+        <v>407</v>
       </c>
       <c r="G11" s="6"/>
     </row>
@@ -15563,7 +16413,7 @@
         <v>28</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>413</v>
+        <v>408</v>
       </c>
       <c r="G13" s="6"/>
     </row>
@@ -15575,7 +16425,7 @@
         <v>30</v>
       </c>
       <c r="C14" s="33" t="s">
-        <v>414</v>
+        <v>409</v>
       </c>
       <c r="G14" s="6"/>
     </row>
@@ -15587,7 +16437,7 @@
         <v>32</v>
       </c>
       <c r="C15" s="33" t="s">
-        <v>415</v>
+        <v>410</v>
       </c>
       <c r="G15" s="6"/>
     </row>
@@ -15599,7 +16449,7 @@
         <v>34</v>
       </c>
       <c r="C16" s="33" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
       <c r="G16" s="6"/>
     </row>
@@ -15611,7 +16461,7 @@
         <v>36</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>417</v>
+        <v>412</v>
       </c>
       <c r="G17" s="6"/>
     </row>
@@ -15623,7 +16473,7 @@
         <v>38</v>
       </c>
       <c r="C18" s="33" t="s">
-        <v>418</v>
+        <v>413</v>
       </c>
       <c r="G18" s="6"/>
     </row>
@@ -15635,7 +16485,7 @@
         <v>40</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>419</v>
+        <v>414</v>
       </c>
       <c r="G19" s="6"/>
     </row>
@@ -15647,7 +16497,7 @@
         <v>42</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>420</v>
+        <v>415</v>
       </c>
       <c r="G20" s="6"/>
     </row>
@@ -15659,7 +16509,7 @@
         <v>44</v>
       </c>
       <c r="C21" s="33" t="s">
-        <v>421</v>
+        <v>416</v>
       </c>
       <c r="G21" s="6"/>
     </row>
@@ -15671,7 +16521,7 @@
         <v>46</v>
       </c>
       <c r="C22" s="33" t="s">
-        <v>422</v>
+        <v>417</v>
       </c>
       <c r="G22" s="6"/>
     </row>
@@ -15683,7 +16533,7 @@
         <v>48</v>
       </c>
       <c r="C23" s="33" t="s">
-        <v>423</v>
+        <v>418</v>
       </c>
       <c r="G23" s="6"/>
     </row>
@@ -15695,7 +16545,7 @@
         <v>50</v>
       </c>
       <c r="C24" s="33" t="s">
-        <v>424</v>
+        <v>419</v>
       </c>
       <c r="G24" s="6"/>
     </row>
@@ -15707,7 +16557,7 @@
         <v>52</v>
       </c>
       <c r="C25" s="33" t="s">
-        <v>425</v>
+        <v>420</v>
       </c>
       <c r="G25" s="6"/>
     </row>
@@ -15719,7 +16569,7 @@
         <v>54</v>
       </c>
       <c r="C26" s="33" t="s">
-        <v>426</v>
+        <v>421</v>
       </c>
       <c r="G26" s="6"/>
     </row>
@@ -15731,7 +16581,7 @@
         <v>56</v>
       </c>
       <c r="C27" s="33" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
       <c r="G27" s="6"/>
     </row>
@@ -15743,7 +16593,7 @@
         <v>58</v>
       </c>
       <c r="C28" s="33" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
       <c r="G28" s="6"/>
     </row>
@@ -15755,7 +16605,7 @@
         <v>60</v>
       </c>
       <c r="C29" s="33" t="s">
-        <v>429</v>
+        <v>424</v>
       </c>
       <c r="G29" s="6"/>
     </row>
@@ -15767,7 +16617,7 @@
         <v>62</v>
       </c>
       <c r="C30" s="33" t="s">
-        <v>430</v>
+        <v>425</v>
       </c>
       <c r="G30" s="6"/>
     </row>
@@ -15779,7 +16629,7 @@
         <v>64</v>
       </c>
       <c r="C31" s="33" t="s">
-        <v>431</v>
+        <v>426</v>
       </c>
       <c r="G31" s="6"/>
     </row>
@@ -15793,11 +16643,19 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="C37" s="103" t="s">
-        <v>347</v>
+        <v>342</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C38" s="8" t="s">
+        <v>451</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A39" s="19"/>
+      <c r="C39" s="8" t="s">
+        <v>452</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -38704,7 +39562,7 @@
         <v>170</v>
       </c>
       <c r="L19" s="110" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="99.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -38733,7 +39591,7 @@
       <c r="E21" s="116"/>
       <c r="F21" s="116"/>
       <c r="L21" s="110" t="s">
-        <v>446</v>
+        <v>440</v>
       </c>
     </row>
     <row r="22" spans="1:12" ht="15" x14ac:dyDescent="0.25">
@@ -38777,7 +39635,7 @@
         <v>3.9269999999999999E-2</v>
       </c>
       <c r="L23" s="110" t="s">
-        <v>447</v>
+        <v>441</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.2">
@@ -38804,7 +39662,7 @@
         <v>1</v>
       </c>
       <c r="L25" s="110" t="s">
-        <v>448</v>
+        <v>442</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.2">
@@ -40410,7 +41268,7 @@
         <v>125</v>
       </c>
       <c r="H8" s="19" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="AE8" s="7"/>
       <c r="AF8" s="7"/>
@@ -42293,7 +43151,7 @@
     </row>
     <row r="71" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A71" s="19" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="E71" s="29">
         <f>SUM(E20:E69)</f>
@@ -42534,7 +43392,7 @@
         <v>125</v>
       </c>
       <c r="H8" s="19" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="AE8" s="7"/>
       <c r="AF8" s="7"/>
@@ -44645,7 +45503,7 @@
         <v>125</v>
       </c>
       <c r="H8" s="19" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="AE8" s="7"/>
       <c r="AF8" s="7"/>
@@ -46759,7 +47617,7 @@
         <v>125</v>
       </c>
       <c r="H8" s="19" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="AE8" s="7"/>
       <c r="AF8" s="7"/>
@@ -48870,7 +49728,7 @@
         <v>125</v>
       </c>
       <c r="H8" s="19" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="AE8" s="7"/>
       <c r="AF8" s="7"/>

</xml_diff>